<commit_message>
Verify one-page constraint instead of just asking the model nicely
Adds a real page-count check (parsed from pdflatex's own log) after each
compile, with one automatic retry that feeds the actual overflow back to
Claude if it ran long. Caught and fixed a real bug in the same change:
pdflatex hard-wraps its log at 79 columns mid-filename with no space, so
the initial regex silently failed to match on wrapped lines and treated
that as "1 page" (i.e. never actually verified anything). Also added a
one-line-per-bullet hard rule to the tailoring prompt, since a wrapped
bullet is the most common cause of overflow in the first place.
</commit_message>
<xml_diff>
--- a/output/tailored_resumes.xlsx
+++ b/output/tailored_resumes.xlsx
@@ -1147,7 +1147,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>scored</t>
+          <t>tailored</t>
         </is>
       </c>
       <c r="M10" s="3" t="inlineStr">
@@ -1155,7 +1155,11 @@
           <t>Apply ↗</t>
         </is>
       </c>
-      <c r="N10" t="inlineStr"/>
+      <c r="N10" s="3" t="inlineStr">
+        <is>
+          <t>Fortinet_Applied_AI_Engineer_AI_Agent_bf9f59.pdf</t>
+        </is>
+      </c>
       <c r="O10" s="3" t="inlineStr">
         <is>
           <t>levels.fyi ↗</t>
@@ -1213,7 +1217,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>scored</t>
+          <t>tailored</t>
         </is>
       </c>
       <c r="M11" s="3" t="inlineStr">
@@ -1221,7 +1225,11 @@
           <t>Apply ↗</t>
         </is>
       </c>
-      <c r="N11" t="inlineStr"/>
+      <c r="N11" s="3" t="inlineStr">
+        <is>
+          <t>Symbotic_Software_Engineer_New_Grad_81ed4e.pdf</t>
+        </is>
+      </c>
       <c r="O11" s="3" t="inlineStr">
         <is>
           <t>levels.fyi ↗</t>
@@ -4869,126 +4877,128 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M9" r:id="rId20"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O9" r:id="rId21"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M10" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M11" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M12" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M13" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N13" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M14" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N14" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O14" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M15" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O15" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M16" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N16" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O16" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M17" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N17" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O17" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M18" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O18" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M19" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N19" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O19" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M20" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O20" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M21" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O21" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M22" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O22" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M23" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N23" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O23" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M24" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O24" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M25" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O25" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M26" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O26" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M27" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N27" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O27" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M28" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O28" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M29" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N29" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O29" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M30" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N30" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O30" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M31" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O31" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M32" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O32" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M33" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O33" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M34" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O34" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M35" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O35" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M36" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O36" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M37" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M38" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O38" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M39" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O39" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M40" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O40" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M41" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O41" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M42" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O42" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M43" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O43" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M44" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O44" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M45" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O45" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M46" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O46" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M47" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O47" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M48" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O48" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M49" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O49" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M50" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O50" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M51" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O51" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M52" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O52" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M53" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O53" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M54" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O54" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M55" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O55" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M56" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O56" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M57" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O57" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M58" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O58" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M59" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O59" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M60" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O60" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M61" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O61" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M62" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O62" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M63" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O63" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M64" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O64" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M65" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O65" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N10" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M11" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N11" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M12" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M13" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N13" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M14" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N14" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O14" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M15" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O15" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M16" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N16" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O16" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M17" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N17" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O17" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M18" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O18" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M19" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N19" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O19" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M20" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O20" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M21" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O21" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M22" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O22" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M23" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N23" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O23" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M24" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O24" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M25" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O25" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M26" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O26" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M27" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N27" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O27" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M28" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O28" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M29" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N29" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O29" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M30" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N30" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O30" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M31" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O31" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M32" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O32" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M33" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O33" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M34" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O34" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M35" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O35" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M36" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O36" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M37" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M38" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O38" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M39" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O39" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M40" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O40" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M41" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O41" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M42" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O42" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M43" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O43" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M44" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O44" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M45" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O45" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M46" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O46" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M47" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O47" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M48" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O48" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M49" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O49" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M50" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O50" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M51" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O51" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M52" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O52" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M53" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O53" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M54" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O54" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M55" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O55" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M56" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O56" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M57" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O57" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M58" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O58" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M59" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O59" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M60" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O60" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M61" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O61" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M62" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O62" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M63" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O63" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M64" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O64" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M65" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O65" r:id="rId144"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add scripts/add_job.py: one-shot fetch+score+tailor for a single job link
Lets a job posting found outside the SimplifyJobs feed (a link someone
sends, something found manually) go through fetch -> score -> tailor in one
command instead of waiting for the next scan. Auto-detects title/company/
location from the ATS API (Ashby/Greenhouse/Lever) when the URL matches one
of those, so a bare link is usually enough.

Verified against three real postings across all three fetch paths: Mach
Industries (Ashby API), Apple (Playwright — no ATS API, JS-rendered page),
and Uniswap (Ashby API, with title/company auto-detected from a bare URL).
</commit_message>
<xml_diff>
--- a/output/tailored_resumes.xlsx
+++ b/output/tailored_resumes.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P65"/>
+  <dimension ref="A1:P68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1175,44 +1175,44 @@
       <c r="A11" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="2" t="n">
-        <v>78</v>
+      <c r="B11" s="4" t="n">
+        <v>74</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>$100k–$135k</t>
+          <t>$140k–$175k</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Symbotic</t>
+          <t>Apple</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Software Engineer New Grad</t>
+          <t>Software Engineer - Information Systems and Technology - Early Career</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Burlington, MA</t>
+          <t>Austin, TX</t>
         </is>
       </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Burlington, MA new-grad SWE at a warehouse-automation company whose core work is large-scale distributed control/backend systems in Java/C++/Python — strong overlap with the candidate's backend and systems strengths and ideal location, docked slightly for robotics/embedded-adjacent leanings and a TC band that sits at the low end of the ~130k anchor.</t>
+          <t>Strong on-profile match — the posting explicitly lists Backend SWE and SRE tracks with Java/Python plus AWS/GCP preferred, which maps directly onto the candidate's microservices and cloud/infra strengths — but it's a generic IS&amp;T requisition weighted toward enterprise/internal systems (SAP, BI, retail tooling) rather than the low-level distributed-systems or AI-infra work the candidate is strongest in, and team assignment is out of his control; timing works since the Aug 2026 posting targets 2027 early-career starts.</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Symbotic is a public (NASDAQ: SYM) automation/robotics firm, not a top-tier tech payer; Boston-area new-grad SWE base typically ~95-115k plus modest bonus and RSU grant. Band is an estimate with moderate confidence — level and team (control systems vs. cloud platform) could shift it either way.</t>
+          <t>Apple ICT2 new-grad software engineering, adjusted down for Austin vs Bay Area and for IS&amp;T (typically at or slightly below the core-OS/silicon bands): base roughly $115–140k, first-year RSU value roughly $15–25k (4-yr vest on a ~$60–100k grant), plus ~10% target bonus and a signing bonus. Apple's leveling is fairly consistent, so the band is moderately tight; IS&amp;T-specific data is thinner than for core engineering orgs, so treat the low end as more likely for enterprise/BI/SAP teams and the high end for Infrastructure Services / SRE-type placements.</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>metadata-only</t>
+          <t>full</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -1227,7 +1227,7 @@
       </c>
       <c r="N11" s="3" t="inlineStr">
         <is>
-          <t>Symbotic_Software_Engineer_New_Grad_81ed4e.pdf</t>
+          <t>Apple_Software_Engineer_Information_Systems_and_Te_8039e5.pdf</t>
         </is>
       </c>
       <c r="O11" s="3" t="inlineStr">
@@ -1245,49 +1245,49 @@
       <c r="A12" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="4" t="n">
-        <v>73</v>
+      <c r="B12" s="2" t="n">
+        <v>78</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>$115k–$150k</t>
+          <t>$100k–$135k</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>The Walt Disney Company</t>
+          <t>Symbotic</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Product Software Engineer 1</t>
+          <t>Software Engineer New Grad</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Glendale, CA</t>
+          <t>Burlington, MA</t>
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Solid backend/data-platform new-grad role (Java/Python, pipelines, AWS, Kubernetes/Terraform) that maps well to his cloud-infra and backend strengths, docked slightly for being data-engineering-leaning rather than distributed-systems/AI-infra, fully on-site in Glendale, and a 2026 req that likely starts before his May 2027 graduation.</t>
+          <t>Burlington, MA new-grad SWE at a warehouse-automation company whose core work is large-scale distributed control/backend systems in Java/C++/Python — strong overlap with the candidate's backend and systems strengths and ideal location, docked slightly for robotics/embedded-adjacent leanings and a TC band that sits at the low end of the ~130k anchor.</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Disney Entertainment/ESPN Product Technology pays upper-mid-tier (below FAANG, above typical enterprise); CA-posted SWE I base ranges typically land ~$100–135k, plus modest bonus and small/no equity at level 1 — so ~$115–150k TC, at or slightly below his ~$130k anchor.</t>
+          <t>Symbotic is a public (NASDAQ: SYM) automation/robotics firm, not a top-tier tech payer; Boston-area new-grad SWE base typically ~95-115k plus modest bonus and RSU grant. Band is an estimate with moderate confidence — level and team (control systems vs. cloud platform) could shift it either way.</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>full</t>
+          <t>metadata-only</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>scored</t>
+          <t>tailored</t>
         </is>
       </c>
       <c r="M12" s="3" t="inlineStr">
@@ -1295,7 +1295,11 @@
           <t>Apply ↗</t>
         </is>
       </c>
-      <c r="N12" t="inlineStr"/>
+      <c r="N12" s="3" t="inlineStr">
+        <is>
+          <t>Symbotic_Software_Engineer_New_Grad_81ed4e.pdf</t>
+        </is>
+      </c>
       <c r="O12" s="3" t="inlineStr">
         <is>
           <t>levels.fyi ↗</t>
@@ -1312,38 +1316,38 @@
         <v>12</v>
       </c>
       <c r="B13" s="4" t="n">
-        <v>58</v>
+        <v>73</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>$185k–$255k</t>
+          <t>$115k–$150k</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>TikTok</t>
+          <t>The Walt Disney Company</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer Graduate - E-Commerce Recommendation Foundation</t>
+          <t>Product Software Engineer 1</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>San Jose, CA</t>
+          <t>Glendale, CA</t>
         </is>
       </c>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Excellent timing (explicit 2027 start) and compensation tier, but the role is a research-oriented ML position requiring foundation-model pre/post-training, PyTorch depth, and ideally top-conference publications — whereas the candidate's AI experience is applied/infra-side (RAG, agents, LLM plumbing) on a backend/distributed-systems base.</t>
+          <t>Solid backend/data-platform new-grad role (Java/Python, pipelines, AWS, Kubernetes/Terraform) that maps well to his cloud-infra and backend strengths, docked slightly for being data-engineering-leaning rather than distributed-systems/AI-infra, fully on-site in Glendale, and a 2026 req that likely starts before his May 2027 graduation.</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Posted base range is $128,000-$316,800; TikTok/ByteDance pays at top-tier (FAANG+) levels for new-grad ML roles, with typical new-grad MLE base ~$145-180k plus signing bonus, annual discretionary bonus, and RSUs. Estimate, not fact.</t>
+          <t>Disney Entertainment/ESPN Product Technology pays upper-mid-tier (below FAANG, above typical enterprise); CA-posted SWE I base ranges typically land ~$100–135k, plus modest bonus and small/no equity at level 1 — so ~$115–150k TC, at or slightly below his ~$130k anchor.</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -1353,7 +1357,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>tailored</t>
+          <t>scored</t>
         </is>
       </c>
       <c r="M13" s="3" t="inlineStr">
@@ -1361,11 +1365,7 @@
           <t>Apply ↗</t>
         </is>
       </c>
-      <c r="N13" s="3" t="inlineStr">
-        <is>
-          <t>TikTok_Machine_Learning_Engineer_Graduate_E_Commer_de90c7.pdf</t>
-        </is>
-      </c>
+      <c r="N13" t="inlineStr"/>
       <c r="O13" s="3" t="inlineStr">
         <is>
           <t>levels.fyi ↗</t>
@@ -1382,11 +1382,11 @@
         <v>13</v>
       </c>
       <c r="B14" s="4" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>$180k–$245k</t>
+          <t>$185k–$255k</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1401,19 +1401,19 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Seattle, WA</t>
+          <t>San Jose, CA</t>
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Timing (2027 start), US location, and Python/AI-infra exposure line up well, but this is a research-leaning ML role centered on LLM/foundation-model pre-training, multimodal tokenization, and generative recommendation — with publications preferred — which sits outside the candidate's backend/distributed-systems/applied-AI (RAG, agents) core and would make him a stretch against PhD/research-track applicants.</t>
+          <t>Excellent timing (explicit 2027 start) and compensation tier, but the role is a research-oriented ML position requiring foundation-model pre/post-training, PyTorch depth, and ideally top-conference publications — whereas the candidate's AI experience is applied/infra-side (RAG, agents, LLM plumbing) on a backend/distributed-systems base.</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Posting states base $121.6k–$243.2k for Seattle; TikTok/ByteDance new-grad ML offers typically land around $150–180k base plus RSUs and bonus, putting realistic first-year TC in the ~$180–245k range. ByteDance pays at or above top-tier US big-tech for ML/recsys new grads, so this comfortably clears the ~$130–165k anchor. Estimate only.</t>
+          <t>Posted base range is $128,000-$316,800; TikTok/ByteDance pays at top-tier (FAANG+) levels for new-grad ML roles, with typical new-grad MLE base ~$145-180k plus signing bonus, annual discretionary bonus, and RSUs. Estimate, not fact.</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -1433,7 +1433,7 @@
       </c>
       <c r="N14" s="3" t="inlineStr">
         <is>
-          <t>TikTok_Machine_Learning_Engineer_Graduate_E_Commer_b2d143.pdf</t>
+          <t>TikTok_Machine_Learning_Engineer_Graduate_E_Commer_de90c7.pdf</t>
         </is>
       </c>
       <c r="O14" s="3" t="inlineStr">
@@ -1452,42 +1452,38 @@
         <v>14</v>
       </c>
       <c r="B15" s="4" t="n">
-        <v>68</v>
+        <v>57</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>$125k–$150k</t>
+          <t>$180k–$245k</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Cohesity</t>
+          <t>TikTok</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Software Engineer New Grad</t>
+          <t>Machine Learning Engineer Graduate - E-Commerce Recommendation Foundation</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Santa Clara, CA</t>
+          <t>Seattle, WA</t>
         </is>
       </c>
       <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>start date and have the legal right to wo</t>
-        </is>
-      </c>
+      <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Near-ideal technical match — distributed systems, storage, and cloud infrastructure work in C/C++/Go/Java/Python, directly aligned with the Raft/LSM-tree/MVCC KV store and backend background — but the posting explicitly targets May/June 2026 graduates (candidate is May 2027) and requires on-site Santa Clara presence, so it's a wrong-cycle req rather than a wrong-profile role.</t>
+          <t>Timing (2027 start), US location, and Python/AI-infra exposure line up well, but this is a research-leaning ML role centered on LLM/foundation-model pre-training, multimodal tokenization, and generative recommendation — with publications preferred — which sits outside the candidate's backend/distributed-systems/applied-AI (RAG, agents) core and would make him a stretch against PhD/research-track applicants.</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Posted base range is $113.4k–$126k (stated in the JD). Cohesity is a large late-stage private infrastructure company, so add bonus plus a private-company RSU grant of roughly $15–30k/yr notional, landing total comp around $125–150k. Note the equity is illiquid/pre-IPO, so realized value is uncertain; cash portion alone sits just under the candidate's ~$130k anchor, and Santa Clara cost-of-living erodes it further.</t>
+          <t>Posting states base $121.6k–$243.2k for Seattle; TikTok/ByteDance new-grad ML offers typically land around $150–180k base plus RSUs and bonus, putting realistic first-year TC in the ~$180–245k range. ByteDance pays at or above top-tier US big-tech for ML/recsys new grads, so this comfortably clears the ~$130–165k anchor. Estimate only.</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -1497,7 +1493,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>scored</t>
+          <t>tailored</t>
         </is>
       </c>
       <c r="M15" s="3" t="inlineStr">
@@ -1505,7 +1501,11 @@
           <t>Apply ↗</t>
         </is>
       </c>
-      <c r="N15" t="inlineStr"/>
+      <c r="N15" s="3" t="inlineStr">
+        <is>
+          <t>TikTok_Machine_Learning_Engineer_Graduate_E_Commer_b2d143.pdf</t>
+        </is>
+      </c>
       <c r="O15" s="3" t="inlineStr">
         <is>
           <t>levels.fyi ↗</t>
@@ -1522,38 +1522,42 @@
         <v>15</v>
       </c>
       <c r="B16" s="4" t="n">
-        <v>52</v>
+        <v>68</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>$180k–$255k</t>
+          <t>$125k–$150k</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>TikTok</t>
+          <t>Cohesity</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer Graduate - E-Commerce Recommendation Mall</t>
+          <t>Software Engineer New Grad</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Seattle, WA</t>
+          <t>Santa Clara, CA</t>
         </is>
       </c>
       <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>start date and have the legal right to wo</t>
+        </is>
+      </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Timing (2027 start) and comp tier fit well, but this is a deep ML research role in generative recommendation/LLM/RL where the candidate's backend, distributed-systems, and AI-infra strengths only partially transfer — no recsys, modeling research, or publications.</t>
+          <t>Near-ideal technical match — distributed systems, storage, and cloud infrastructure work in C/C++/Go/Java/Python, directly aligned with the Raft/LSM-tree/MVCC KV store and backend background — but the posting explicitly targets May/June 2026 graduates (candidate is May 2027) and requires on-site Santa Clara presence, so it's a wrong-cycle req rather than a wrong-profile role.</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>Posted Seattle base band is $121.6k-$243.2k. TikTok new-grad ML/SWE typically lands base ~$145k-$180k plus ~10-15% bonus and ~$30k-$60k/yr RSU, putting total package around $180k-$255k. Given the candidate lacks the ML research/publication signal that drives the top of the band, realistic landing zone is ~$185k-$210k. Estimate, not fact.</t>
+          <t>Posted base range is $113.4k–$126k (stated in the JD). Cohesity is a large late-stage private infrastructure company, so add bonus plus a private-company RSU grant of roughly $15–30k/yr notional, landing total comp around $125–150k. Note the equity is illiquid/pre-IPO, so realized value is uncertain; cash portion alone sits just under the candidate's ~$130k anchor, and Santa Clara cost-of-living erodes it further.</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -1563,7 +1567,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>tailored</t>
+          <t>scored</t>
         </is>
       </c>
       <c r="M16" s="3" t="inlineStr">
@@ -1571,11 +1575,7 @@
           <t>Apply ↗</t>
         </is>
       </c>
-      <c r="N16" s="3" t="inlineStr">
-        <is>
-          <t>TikTok_Machine_Learning_Engineer_Graduate_E_Commer_59f20c.pdf</t>
-        </is>
-      </c>
+      <c r="N16" t="inlineStr"/>
       <c r="O16" s="3" t="inlineStr">
         <is>
           <t>levels.fyi ↗</t>
@@ -1591,12 +1591,12 @@
       <c r="A17" t="n">
         <v>16</v>
       </c>
-      <c r="B17" s="5" t="n">
-        <v>45</v>
+      <c r="B17" s="4" t="n">
+        <v>52</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>$190k–$280k</t>
+          <t>$180k–$255k</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1611,19 +1611,19 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>San Jose, CA</t>
+          <t>Seattle, WA</t>
         </is>
       </c>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2027 start date and Python/LLM-agent exposure align, but the role is a research-oriented ML/recsys position (generative retrieval, RL, LLM post-training, top-tier publications preferred) rather than the backend, distributed-systems, or AI-infrastructure work the candidate is strong in — no deep-learning modeling, PyTorch, or recommender-system background.</t>
+          <t>Timing (2027 start) and comp tier fit well, but this is a deep ML research role in generative recommendation/LLM/RL where the candidate's backend, distributed-systems, and AI-infra strengths only partially transfer — no recsys, modeling research, or publications.</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>Posting states base $128,000-$316,800 for San Jose plus RSUs and discretionary bonus. ByteDance/TikTok is a top-of-market payer for new-grad ML engineers; realistic new-grad base lands ~$150-190k with equity and bonus pushing total comp to roughly $190-280k. Estimate, not fact.</t>
+          <t>Posted Seattle base band is $121.6k-$243.2k. TikTok new-grad ML/SWE typically lands base ~$145k-$180k plus ~10-15% bonus and ~$30k-$60k/yr RSU, putting total package around $180k-$255k. Given the candidate lacks the ML research/publication signal that drives the top of the band, realistic landing zone is ~$185k-$210k. Estimate, not fact.</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -1643,7 +1643,7 @@
       </c>
       <c r="N17" s="3" t="inlineStr">
         <is>
-          <t>TikTok_Machine_Learning_Engineer_Graduate_E_Commer_40ebe3.pdf</t>
+          <t>TikTok_Machine_Learning_Engineer_Graduate_E_Commer_59f20c.pdf</t>
         </is>
       </c>
       <c r="O17" s="3" t="inlineStr">
@@ -1661,39 +1661,39 @@
       <c r="A18" t="n">
         <v>17</v>
       </c>
-      <c r="B18" s="4" t="n">
-        <v>58</v>
+      <c r="B18" s="5" t="n">
+        <v>45</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>$140k–$185k</t>
+          <t>$190k–$280k</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Handshake</t>
+          <t>TikTok</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Associate Software Engineer</t>
+          <t>Machine Learning Engineer Graduate - E-Commerce Recommendation Mall</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>SF</t>
+          <t>San Jose, CA</t>
         </is>
       </c>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Legitimate new-grad SWE role (0-2 yrs) at a hot, well-paying SF company, but it's internal operations tooling — communication-heavy, embedded/consulting work that barely touches the candidate's distributed-systems, infra, or AI-platform strengths.</t>
+          <t>2027 start date and Python/LLM-agent exposure align, but the role is a research-oriented ML/recsys position (generative retrieval, RL, LLM post-training, top-tier publications preferred) rather than the backend, distributed-systems, or AI-infrastructure work the candidate is strong in — no deep-learning modeling, PyTorch, or recommender-system background.</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Well-funded SF unicorn (~$1B run rate, Handshake AI) that competes for Bay Area new-grad talent; "Associate" title suggests the lower rung of their SWE ladder. Estimated base ~$125-150K plus meaningful equity and 401(k) match. Band is moderately wide since Handshake does not publish new-grad levels and SF startup equity valuation is uncertain.</t>
+          <t>Posting states base $128,000-$316,800 for San Jose plus RSUs and discretionary bonus. ByteDance/TikTok is a top-of-market payer for new-grad ML engineers; realistic new-grad base lands ~$150-190k with equity and bonus pushing total comp to roughly $190-280k. Estimate, not fact.</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -1703,7 +1703,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>scored</t>
+          <t>tailored</t>
         </is>
       </c>
       <c r="M18" s="3" t="inlineStr">
@@ -1711,7 +1711,11 @@
           <t>Apply ↗</t>
         </is>
       </c>
-      <c r="N18" t="inlineStr"/>
+      <c r="N18" s="3" t="inlineStr">
+        <is>
+          <t>TikTok_Machine_Learning_Engineer_Graduate_E_Commer_40ebe3.pdf</t>
+        </is>
+      </c>
       <c r="O18" s="3" t="inlineStr">
         <is>
           <t>levels.fyi ↗</t>
@@ -1727,39 +1731,39 @@
       <c r="A19" t="n">
         <v>18</v>
       </c>
-      <c r="B19" s="5" t="n">
-        <v>32</v>
+      <c r="B19" s="4" t="n">
+        <v>58</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>$230k–$400k</t>
+          <t>$140k–$185k</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>TikTok</t>
+          <t>Handshake</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>AI Infrastructure Engineer Graduate - Recommendation &amp; LLM</t>
+          <t>Associate Software Engineer</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>San Jose, CA</t>
+          <t>SF</t>
         </is>
       </c>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr">
         <is>
-          <t>The technical domain is a near-perfect match (distributed systems, LLM/AI infrastructure, C++/Python, large-scale training and serving), but the posting is explicitly a PhD-only 2027 graduate req with an onboarding deadline by end of year, which hard-filters a BS/MS May 2027 candidate regardless of skill overlap.</t>
+          <t>Legitimate new-grad SWE role (0-2 yrs) at a hot, well-paying SF company, but it's internal operations tooling — communication-heavy, embedded/consulting work that barely touches the candidate's distributed-systems, infra, or AI-platform strengths.</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>Posting states base $162k–$387.6k for San Jose plus discretionary bonus and RSUs; TikTok/ByteDance pays top-of-market for PhD AI-infra roles, so realistic PhD new-grad TC lands roughly $230k–$400k. Note this band reflects the PhD level of this req — an equivalent BS/MS new-grad AI-infra role at TikTok would be closer to $160k–$230k TC, still well above the candidate's $130k anchor.</t>
+          <t>Well-funded SF unicorn (~$1B run rate, Handshake AI) that competes for Bay Area new-grad talent; "Associate" title suggests the lower rung of their SWE ladder. Estimated base ~$125-150K plus meaningful equity and 401(k) match. Band is moderately wide since Handshake does not publish new-grad levels and SF startup equity valuation is uncertain.</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -1769,7 +1773,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>tailored</t>
+          <t>scored</t>
         </is>
       </c>
       <c r="M19" s="3" t="inlineStr">
@@ -1777,11 +1781,7 @@
           <t>Apply ↗</t>
         </is>
       </c>
-      <c r="N19" s="3" t="inlineStr">
-        <is>
-          <t>TikTok_AI_Infrastructure_Engineer_Graduate_Recomme_6aeb33.pdf</t>
-        </is>
-      </c>
+      <c r="N19" t="inlineStr"/>
       <c r="O19" s="3" t="inlineStr">
         <is>
           <t>levels.fyi ↗</t>
@@ -1797,39 +1797,39 @@
       <c r="A20" t="n">
         <v>19</v>
       </c>
-      <c r="B20" s="4" t="n">
-        <v>55</v>
+      <c r="B20" s="5" t="n">
+        <v>32</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>$100k–$128k</t>
+          <t>$230k–$400k</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>T-Mobile</t>
+          <t>TikTok</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Associate Engineer - Software</t>
+          <t>AI Infrastructure Engineer Graduate - Recommendation &amp; LLM</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Frisco, TX</t>
+          <t>San Jose, CA</t>
         </is>
       </c>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Technical scope (microservices, SDN/NFV, big data, scalable HA systems) overlaps his backend/infra profile, but it's a closely-supervised associate role at a mid-tier payer in a non-preferred location with a near-term start signal, landing below his ~130k TC anchor.</t>
+          <t>The technical domain is a near-perfect match (distributed systems, LLM/AI infrastructure, C++/Python, large-scale training and serving), but the posting is explicitly a PhD-only 2027 graduate req with an onboarding deadline by end of year, which hard-filters a BS/MS May 2027 candidate regardless of skill overlap.</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>Posting states base $66,900-$120,600 with 10% corporate bonus target; CS new grad likely ~$90-110k base, plus ~10% bonus, annual stock grant and ESPP. T-Mobile is a solid but non-top-tier engineering payer; Frisco cost-of-labor puts a new grad mid-range rather than top. Estimate, not fact.</t>
+          <t>Posting states base $162k–$387.6k for San Jose plus discretionary bonus and RSUs; TikTok/ByteDance pays top-of-market for PhD AI-infra roles, so realistic PhD new-grad TC lands roughly $230k–$400k. Note this band reflects the PhD level of this req — an equivalent BS/MS new-grad AI-infra role at TikTok would be closer to $160k–$230k TC, still well above the candidate's $130k anchor.</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -1839,7 +1839,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>scored</t>
+          <t>tailored</t>
         </is>
       </c>
       <c r="M20" s="3" t="inlineStr">
@@ -1847,7 +1847,11 @@
           <t>Apply ↗</t>
         </is>
       </c>
-      <c r="N20" t="inlineStr"/>
+      <c r="N20" s="3" t="inlineStr">
+        <is>
+          <t>TikTok_AI_Infrastructure_Engineer_Graduate_Recomme_6aeb33.pdf</t>
+        </is>
+      </c>
       <c r="O20" s="3" t="inlineStr">
         <is>
           <t>levels.fyi ↗</t>
@@ -1863,39 +1867,39 @@
       <c r="A21" t="n">
         <v>20</v>
       </c>
-      <c r="B21" s="5" t="n">
-        <v>45</v>
+      <c r="B21" s="4" t="n">
+        <v>55</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>$150k–$195k</t>
+          <t>$100k–$128k</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Adobe</t>
+          <t>T-Mobile</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Photoshop Developer - GPU/Imaging</t>
+          <t>Associate Engineer - Software</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Seattle, WA, SF, San Jose, CA, NYC</t>
+          <t>Frisco, TX</t>
         </is>
       </c>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Performance/low-level systems orientation is a partial match, but the role centers on GPU graphics programming (shaders, WGSL, Metal/Vulkan/WebGPU, color and compositing pipelines) that is entirely absent from this candidate's backend/distributed-systems/AI-infra background.</t>
+          <t>Technical scope (microservices, SDN/NFV, big data, scalable HA systems) overlaps his backend/infra profile, but it's a closely-supervised associate role at a mid-tier payer in a non-preferred location with a near-term start signal, landing below his ~130k TC anchor.</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>Adobe is upper-middle big-tech for entry-level SWE in SF/San Jose/Seattle/NYC: roughly $130-150k base + 10-15% target bonus + ~$25-40k/yr RSUs. Band is wide because the posting spans early-career through senior; a new grad would land near the low end. Estimate based on general knowledge of Adobe's comp tier, not verified data.</t>
+          <t>Posting states base $66,900-$120,600 with 10% corporate bonus target; CS new grad likely ~$90-110k base, plus ~10% bonus, annual stock grant and ESPP. T-Mobile is a solid but non-top-tier engineering payer; Frisco cost-of-labor puts a new grad mid-range rather than top. Estimate, not fact.</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -1934,34 +1938,34 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>$140k–$175k</t>
+          <t>$150k–$195k</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Cisco</t>
+          <t>Adobe</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Software Engineer 2 - Wireless Platform</t>
+          <t>Photoshop Developer - GPU/Imaging</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>SF, San Jose, CA</t>
+          <t>Seattle, WA, SF, San Jose, CA, NYC</t>
         </is>
       </c>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Embedded platform/BSP work (board bring-up, device drivers, boot-time init, UART/SPI/I2C) is squarely in the candidate's low-fit hardware/embedded bucket and the BS+2yrs / MS+0 minimum disfavors a May-2027 bachelor's new grad, though C/C++ plus a systems-security concentration and embedded-Linux debugging overlap give it partial credit.</t>
+          <t>Performance/low-level systems orientation is a partial match, but the role centers on GPU graphics programming (shaders, WGSL, Metal/Vulkan/WebGPU, color and compositing pipelines) that is entirely absent from this candidate's backend/distributed-systems/AI-infra background.</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>Posting states $125,700-$176,600 base for US/Canada new hires at this level, excluding bonus, equity, and benefits. Cisco is a solid mid-to-upper-tier payer (below FAANG/HFT, above most enterprise IT). Assuming an entry-of-band base for a near-new-grad in SF/San Jose (~$130-150k), plus ~10% target bonus and a modest RSU grant, TC lands around $140-175k. Note this is a SWE II req rather than a dedicated new-grad req, so an actual new-grad-equivalent offer could come in nearer the low end or slightly below.</t>
+          <t>Adobe is upper-middle big-tech for entry-level SWE in SF/San Jose/Seattle/NYC: roughly $130-150k base + 10-15% target bonus + ~$25-40k/yr RSUs. Band is wide because the posting spans early-career through senior; a new grad would land near the low end. Estimate based on general knowledge of Adobe's comp tier, not verified data.</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -1996,38 +2000,38 @@
         <v>22</v>
       </c>
       <c r="B23" s="5" t="n">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>$250k–$420k</t>
+          <t>$140k–$175k</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>TikTok</t>
+          <t>Cisco</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Data Knowledge System Research Scientist Graduate - Data Platform-Global Live</t>
+          <t>Software Engineer 2 - Wireless Platform</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>San Jose, CA</t>
+          <t>SF, San Jose, CA</t>
         </is>
       </c>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Technical content is an excellent match (RAG, agentic systems, vector DBs, knowledge/data platform, distributed systems, Python/Java), but the minimum qualification is a completed or near-complete PhD, which hard-gates a May 2027 bachelor's-level new grad.</t>
+          <t>Embedded platform/BSP work (board bring-up, device drivers, boot-time init, UART/SPI/I2C) is squarely in the candidate's low-fit hardware/embedded bucket and the BS+2yrs / MS+0 minimum disfavors a May-2027 bachelor's new grad, though C/C++ plus a systems-security concentration and embedded-Linux debugging overlap give it partial credit.</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>Posting states base $218,400-$480,000 for San Jose, which reflects PhD research-scientist banding rather than a BS/MS new-grad band; adding typical TikTok bonus/RSU on a mid-range base yields roughly $250k-$420k TC. This is an estimate, and it is not the band this candidate would be hired into — TikTok's comparable BS/MS new-grad SWE roles are closer to $145k-$200k TC.</t>
+          <t>Posting states $125,700-$176,600 base for US/Canada new hires at this level, excluding bonus, equity, and benefits. Cisco is a solid mid-to-upper-tier payer (below FAANG/HFT, above most enterprise IT). Assuming an entry-of-band base for a near-new-grad in SF/San Jose (~$130-150k), plus ~10% target bonus and a modest RSU grant, TC lands around $140-175k. Note this is a SWE II req rather than a dedicated new-grad req, so an actual new-grad-equivalent offer could come in nearer the low end or slightly below.</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -2037,7 +2041,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>tailored</t>
+          <t>scored</t>
         </is>
       </c>
       <c r="M23" s="3" t="inlineStr">
@@ -2045,11 +2049,7 @@
           <t>Apply ↗</t>
         </is>
       </c>
-      <c r="N23" s="3" t="inlineStr">
-        <is>
-          <t>TikTok_Data_Knowledge_System_Research_Scientist_Gr_e0c0d2.pdf</t>
-        </is>
-      </c>
+      <c r="N23" t="inlineStr"/>
       <c r="O23" s="3" t="inlineStr">
         <is>
           <t>levels.fyi ↗</t>
@@ -2066,38 +2066,38 @@
         <v>23</v>
       </c>
       <c r="B24" s="5" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>$230k–$350k</t>
+          <t>$250k–$420k</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>ByteDance</t>
+          <t>TikTok</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>AI/LLM Network Software Development Engineer Graduate - High Speed Network - PhD</t>
+          <t>Data Knowledge System Research Scientist Graduate - Data Platform-Global Live</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Seattle, WA</t>
+          <t>San Jose, CA</t>
         </is>
       </c>
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr">
         <is>
-          <t>Timing (2027 start) and the systems/infra domain fit, but the role hard-requires a completed PhD plus specialized high-speed networking research depth (RDMA, congestion control, NCCL/MPI) that a BS-level backend/distributed-systems candidate does not have.</t>
+          <t>Technical content is an excellent match (RAG, agentic systems, vector DBs, knowledge/data platform, distributed systems, Python/Java), but the minimum qualification is a completed or near-complete PhD, which hard-gates a May 2027 bachelor's-level new grad.</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>Posted base range $153.9k-$300.96k; ByteDance is a top-tier payer and PhD new-grad infra offers typically add substantial RSUs plus bonus on top of a ~$180-220k base. Estimate, not fact — and it reflects the PhD hiring level, not what this candidate would be offered.</t>
+          <t>Posting states base $218,400-$480,000 for San Jose, which reflects PhD research-scientist banding rather than a BS/MS new-grad band; adding typical TikTok bonus/RSU on a mid-range base yields roughly $250k-$420k TC. This is an estimate, and it is not the band this candidate would be hired into — TikTok's comparable BS/MS new-grad SWE roles are closer to $145k-$200k TC.</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -2107,7 +2107,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>scored</t>
+          <t>tailored</t>
         </is>
       </c>
       <c r="M24" s="3" t="inlineStr">
@@ -2115,7 +2115,11 @@
           <t>Apply ↗</t>
         </is>
       </c>
-      <c r="N24" t="inlineStr"/>
+      <c r="N24" s="3" t="inlineStr">
+        <is>
+          <t>TikTok_Data_Knowledge_System_Research_Scientist_Gr_e0c0d2.pdf</t>
+        </is>
+      </c>
       <c r="O24" s="3" t="inlineStr">
         <is>
           <t>levels.fyi ↗</t>
@@ -2132,38 +2136,38 @@
         <v>24</v>
       </c>
       <c r="B25" s="5" t="n">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>$135k–$180k</t>
+          <t>$160k–$230k</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Mach Industries</t>
+          <t>Uniswap</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Software Engineer New Grad - Software - GNC</t>
+          <t>Software Engineer - Early Career</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Huntington Beach, CA</t>
+          <t>New York</t>
         </is>
       </c>
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr">
         <is>
-          <t>Hard eligibility mismatch — the posting requires graduation by end of 2026 or January 2027 and Nate graduates May 2027 — and the role centers on GNC/embedded/real-time firmware rather than his backend/distributed-systems/AI-infra profile, though his Rust, C/C++, Linux, concurrency, and CI/CD background would otherwise be a reasonable partial match.</t>
+          <t>Comp, tier, and NYC location are excellent fits, but the posting hard-gates on a degree completed between December 2024 and September 2026 while the candidate graduates May 2027, making him ineligible for this cohort; the role is also full-stack/web-leaning rather than backend/distributed-systems focused.</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>Mach Industries is a well-funded (Sequoia/Bridgewater-backed) defense-tech startup in the Anduril/Applied Intuition orbit; those firms typically pay new-grad SWEs ~$120-150k base in high-COL SoCal plus meaningful early-stage equity, which the posting explicitly says is part of TC. Band is wide because private-startup equity value is speculative and Mach does not publish new-grad levels — this is an estimate, not fact.</t>
+          <t>Posted NYC base range is $138,400-$198,000; a new grad would land near the low end (~$138-155k base). Uniswap Labs is a well-funded crypto/DeFi employer paying at or above top-tier tech, and the posting explicitly lists token compensation plus benefits on top of base. The band is intentionally wide on the upper end because token grant sizing and valuation are undisclosed and volatile. Estimate, not fact.</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -2173,7 +2177,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>scored</t>
+          <t>tailored</t>
         </is>
       </c>
       <c r="M25" s="3" t="inlineStr">
@@ -2181,7 +2185,11 @@
           <t>Apply ↗</t>
         </is>
       </c>
-      <c r="N25" t="inlineStr"/>
+      <c r="N25" s="3" t="inlineStr">
+        <is>
+          <t>Uniswap_Software_Engineer_Early_Career_5a340c.pdf</t>
+        </is>
+      </c>
       <c r="O25" s="3" t="inlineStr">
         <is>
           <t>levels.fyi ↗</t>
@@ -2198,43 +2206,43 @@
         <v>25</v>
       </c>
       <c r="B26" s="5" t="n">
-        <v>45</v>
+        <v>20</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>$85k–$110k</t>
+          <t>$230k–$350k</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Abbott</t>
+          <t>ByteDance</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Associate Software Engineer - Multiple Teams</t>
+          <t>AI/LLM Network Software Development Engineer Graduate - High Speed Network - PhD</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Irving, TX</t>
+          <t>Seattle, WA</t>
         </is>
       </c>
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr">
         <is>
-          <t>Entry-level SWE title is right, but Abbott's software work is medtech/embedded and regulated rather than backend distributed systems or AI infra, and the comp tier falls short of the candidate's ~130k anchor.</t>
+          <t>Timing (2027 start) and the systems/infra domain fit, but the role hard-requires a completed PhD plus specialized high-speed networking research depth (RDMA, congestion control, NCCL/MPI) that a BS-level backend/distributed-systems candidate does not have.</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>Abbott is a large non-tech medical-device employer; new-grad associate engineer base in Irving, TX typically ~$75-95k plus a small bonus and negligible equity. Posting gave no level or comp detail, so the band is widened; estimate only.</t>
+          <t>Posted base range $153.9k-$300.96k; ByteDance is a top-tier payer and PhD new-grad infra offers typically add substantial RSUs plus bonus on top of a ~$180-220k base. Estimate, not fact — and it reflects the PhD hiring level, not what this candidate would be offered.</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>metadata-only</t>
+          <t>full</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
@@ -2264,38 +2272,38 @@
         <v>26</v>
       </c>
       <c r="B27" s="5" t="n">
-        <v>15</v>
+        <v>37</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>$280k–$450k</t>
+          <t>$135k–$180k</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>TikTok</t>
+          <t>Mach Industries</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer Graduate - E-Commerce Recommendation Mall - PhD</t>
+          <t>Software Engineer New Grad - Software - GNC</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Seattle, WA</t>
+          <t>Huntington Beach, CA</t>
         </is>
       </c>
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr">
         <is>
-          <t>Role hard-requires a completing/completed PhD with ML research depth in generative recommenders, LLM/RL post-training, and top-tier publications — off-profile for a May 2027 BS-level backend/distributed-systems new grad, despite some adjacent AI/agentic and infra exposure.</t>
+          <t>Hard eligibility mismatch — the posting requires graduation by end of 2026 or January 2027 and Nate graduates May 2027 — and the role centers on GNC/embedded/real-time firmware rather than his backend/distributed-systems/AI-infra profile, though his Rust, C/C++, Linux, concurrency, and CI/CD background would otherwise be a reasonable partial match.</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>Posting states base $153,900-$300,960 for Seattle; TikTok/ByteDance PhD MLE offers typically add sizable RSU grants plus discretionary bonus, putting total package well above base. Band is wide because PhD research-track comp varies heavily with publication record and competing offers. Estimate reflects the posted PhD role, not a level this candidate would be hired into.</t>
+          <t>Mach Industries is a well-funded (Sequoia/Bridgewater-backed) defense-tech startup in the Anduril/Applied Intuition orbit; those firms typically pay new-grad SWEs ~$120-150k base in high-COL SoCal plus meaningful early-stage equity, which the posting explicitly says is part of TC. Band is wide because private-startup equity value is speculative and Mach does not publish new-grad levels — this is an estimate, not fact.</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -2305,7 +2313,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>tailored</t>
+          <t>scored</t>
         </is>
       </c>
       <c r="M27" s="3" t="inlineStr">
@@ -2313,11 +2321,7 @@
           <t>Apply ↗</t>
         </is>
       </c>
-      <c r="N27" s="3" t="inlineStr">
-        <is>
-          <t>TikTok_Machine_Learning_Engineer_Graduate_E_Commer_1700a5.pdf</t>
-        </is>
-      </c>
+      <c r="N27" t="inlineStr"/>
       <c r="O27" s="3" t="inlineStr">
         <is>
           <t>levels.fyi ↗</t>
@@ -2334,43 +2338,43 @@
         <v>27</v>
       </c>
       <c r="B28" s="5" t="n">
-        <v>15</v>
+        <v>45</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>$300k–$550k</t>
+          <t>$85k–$110k</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>ByteDance</t>
+          <t>Abbott</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Research Engineer Graduate - Seed Infra - PhD</t>
+          <t>Associate Software Engineer - Multiple Teams</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>San Jose, CA</t>
+          <t>Irving, TX</t>
         </is>
       </c>
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr">
         <is>
-          <t>The AI-training-infrastructure domain (distributed systems, fault-tolerant infra, GPU cluster scaling) maps well to Nate's Raft/KV-store and ML-infra interests, but the posting is a hard PhD-only requirement with a 2026 onboarding deadline and expects deep LLM/RL training-systems research experience — disqualifying for a May 2027 bachelor's/master's new grad.</t>
+          <t>Entry-level SWE title is right, but Abbott's software work is medtech/embedded and regulated rather than backend distributed systems or AI infra, and the comp tier falls short of the candidate's ~130k anchor.</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>Posted base range is $254.4k–$480k for this San Jose Seed Infra PhD role; adding RSUs and bonus puts realistic first-year TC around $300k–$550k. Note this is PhD-research-engineer compensation at ByteDance's top AI-lab band, not a standard new-grad SWE band (ByteDance new-grad SWE is more like $200–250k TC) — the figures above are not attainable at Nate's level.</t>
+          <t>Abbott is a large non-tech medical-device employer; new-grad associate engineer base in Irving, TX typically ~$75-95k plus a small bonus and negligible equity. Posting gave no level or comp detail, so the band is widened; estimate only.</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>full</t>
+          <t>metadata-only</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
@@ -2400,11 +2404,11 @@
         <v>28</v>
       </c>
       <c r="B29" s="5" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>$250k–$400k</t>
+          <t>$280k–$450k</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -2414,24 +2418,24 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer Graduate - E-Commerce Recommendation Foundation - PhD</t>
+          <t>Machine Learning Engineer Graduate - E-Commerce Recommendation Mall - PhD</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>San Jose, CA</t>
+          <t>Seattle, WA</t>
         </is>
       </c>
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr">
         <is>
-          <t>Hard PhD requirement plus deep ML-research expectations (LLM pre/post-training, generative recommendation, top-tier publications) that a BS-level backend/distributed-systems new grad cannot meet, despite some adjacent applied-AI/RAG experience.</t>
+          <t>Role hard-requires a completing/completed PhD with ML research depth in generative recommenders, LLM/RL post-training, and top-tier publications — off-profile for a May 2027 BS-level backend/distributed-systems new grad, despite some adjacent AI/agentic and infra exposure.</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>Posting states base $162k–$387.6k for this PhD ML role; TikTok pays top-of-market for PhD ML/recsys, with RSUs and bonus on top of base — typical PhD new-grad offers land ~$250k–$400k TC (higher for exceptional research profiles). Not applicable to this candidate's BS-level band (~$130–165k).</t>
+          <t>Posting states base $153,900-$300,960 for Seattle; TikTok/ByteDance PhD MLE offers typically add sizable RSU grants plus discretionary bonus, putting total package well above base. Band is wide because PhD research-track comp varies heavily with publication record and competing offers. Estimate reflects the posted PhD role, not a level this candidate would be hired into.</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -2451,7 +2455,7 @@
       </c>
       <c r="N29" s="3" t="inlineStr">
         <is>
-          <t>TikTok_Machine_Learning_Engineer_Graduate_E_Commer_bfd35d.pdf</t>
+          <t>TikTok_Machine_Learning_Engineer_Graduate_E_Commer_1700a5.pdf</t>
         </is>
       </c>
       <c r="O29" s="3" t="inlineStr">
@@ -2470,38 +2474,38 @@
         <v>29</v>
       </c>
       <c r="B30" s="5" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>$250k–$350k</t>
+          <t>$300k–$550k</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>TikTok</t>
+          <t>ByteDance</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer Graduate - E-Commerce Recommendation Foundation - PhD</t>
+          <t>Research Engineer Graduate - Seed Infra - PhD</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Seattle, WA</t>
+          <t>San Jose, CA</t>
         </is>
       </c>
       <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Hard PhD requirement plus a research profile (LLM pre/post-training, generative recommendation, NeurIPS/ICML-tier publications) that a BS-level backend/distributed-systems candidate cannot satisfy — the AI/RAG experience is applied infra, not foundation-model research.</t>
+          <t>The AI-training-infrastructure domain (distributed systems, fault-tolerant infra, GPU cluster scaling) maps well to Nate's Raft/KV-store and ML-infra interests, but the posting is a hard PhD-only requirement with a 2026 onboarding deadline and expects deep LLM/RL training-systems research experience — disqualifying for a May 2027 bachelor's/master's new grad.</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Posting states base $153,900–$300,960 for Seattle; TikTok PhD MLE new-grad offers typically land in the low-to-mid $200k base range plus RSUs (~$40–100k/yr) and bonus, putting realistic total comp for a fresh PhD around $250k–$350k. Band is wide because TikTok's ML research bands are unusually broad and heavily calibrated to publication record.</t>
+          <t>Posted base range is $254.4k–$480k for this San Jose Seed Infra PhD role; adding RSUs and bonus puts realistic first-year TC around $300k–$550k. Note this is PhD-research-engineer compensation at ByteDance's top AI-lab band, not a standard new-grad SWE band (ByteDance new-grad SWE is more like $200–250k TC) — the figures above are not attainable at Nate's level.</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -2511,7 +2515,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>tailored</t>
+          <t>scored</t>
         </is>
       </c>
       <c r="M30" s="3" t="inlineStr">
@@ -2519,11 +2523,7 @@
           <t>Apply ↗</t>
         </is>
       </c>
-      <c r="N30" s="3" t="inlineStr">
-        <is>
-          <t>TikTok_Machine_Learning_Engineer_Graduate_E_Commer_499a7c.pdf</t>
-        </is>
-      </c>
+      <c r="N30" t="inlineStr"/>
       <c r="O30" s="3" t="inlineStr">
         <is>
           <t>levels.fyi ↗</t>
@@ -2540,38 +2540,38 @@
         <v>30</v>
       </c>
       <c r="B31" s="5" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>$200k–$300k</t>
+          <t>$250k–$400k</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>ByteDance</t>
+          <t>TikTok</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Video/Image AI/ML Software Engineer Graduate - Multimedia</t>
+          <t>Machine Learning Engineer Graduate - E-Commerce Recommendation Foundation - PhD</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>San Diego, CA</t>
+          <t>San Jose, CA</t>
         </is>
       </c>
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr">
         <is>
-          <t>Hard PhD requirement (candidate is a 2027 bachelor's-level new grad) combined with a deeply specialized video codec / image-quality-algorithm domain (VMAF, PSNR, SSIM, AVC/HEVC/AV1, FPGA/ASIC C-models, RTOS/embedded) that has almost no overlap with his distributed-systems, backend, and AI-infra background.</t>
+          <t>Hard PhD requirement plus deep ML-research expectations (LLM pre/post-training, generative recommendation, top-tier publications) that a BS-level backend/distributed-systems new grad cannot meet, despite some adjacent applied-AI/RAG experience.</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>ByteDance is a top-of-market payer; the posting itself lists $122.6k–$301k base for this PhD-level San Diego role, plus RSUs and bonus. PhD new-grad hires typically land in the upper-middle of that band, so ~$200–300k TC is realistic here. Note this is a PhD-track number — a bachelor's new-grad SWE at ByteDance would be closer to $180–230k TC, and this specific req would not be open to him.</t>
+          <t>Posting states base $162k–$387.6k for this PhD ML role; TikTok pays top-of-market for PhD ML/recsys, with RSUs and bonus on top of base — typical PhD new-grad offers land ~$250k–$400k TC (higher for exceptional research profiles). Not applicable to this candidate's BS-level band (~$130–165k).</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -2581,7 +2581,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>scored</t>
+          <t>tailored</t>
         </is>
       </c>
       <c r="M31" s="3" t="inlineStr">
@@ -2589,7 +2589,11 @@
           <t>Apply ↗</t>
         </is>
       </c>
-      <c r="N31" t="inlineStr"/>
+      <c r="N31" s="3" t="inlineStr">
+        <is>
+          <t>TikTok_Machine_Learning_Engineer_Graduate_E_Commer_bfd35d.pdf</t>
+        </is>
+      </c>
       <c r="O31" s="3" t="inlineStr">
         <is>
           <t>levels.fyi ↗</t>
@@ -2606,38 +2610,34 @@
         <v>31</v>
       </c>
       <c r="B32" s="5" t="n">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>$80k–$105k</t>
+          <t>$130k–$190k</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>RTX</t>
+          <t>Mach Industries</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Software Engineer 1</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>Cedar Rapids, IA</t>
-        </is>
-      </c>
+          <t>Software Engineer New Grad - Software - GNC</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr"/>
       <c r="I32" t="inlineStr">
         <is>
-          <t>Generic entry-level SWE title is nominally on-profile, but RTX/Collins avionics work in Cedar Rapids skews embedded/safety-critical C rather than distributed systems or AI infra, almost certainly requires clearance eligibility (candidate has none), and the TC ceiling sits well under the ~130k anchor.</t>
+          <t>Hard timing blocker — the posting requires graduation by end of 2026 or January 2027 and Nate graduates May 2027 — and the role centers on GNC/embedded/real-time firmware rather than his backend and distributed-systems core, though his Rust/C++ depth and the "Linux, concurrency, distributed systems" preferred bullet keep it from scoring lower.</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>Description body failed to scrape (cookie banner only), so this is based on general knowledge: RTX/Collins Aerospace in Cedar Rapids, IA is defense-primes tier — new-grad SWE 1 base typically ~$75-95k with a small bonus, and low-COL Iowa pulls it further down. Defense primes also commonly gate these roles on US citizenship plus clearance eligibility. Band is wide given the missing posting text.</t>
+          <t>Mach Industries is a well-funded defense-tech startup (Sequoia/Bedrock-backed, ~350 employees) competing with Anduril/SpaceX for talent; new-grad SWE base likely ~$120-160k with meaningful equity on top. Estimate is uncertain — no public leveling data for Mach specifically, so band is wide.</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -2647,7 +2647,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>scored</t>
+          <t>tailored</t>
         </is>
       </c>
       <c r="M32" s="3" t="inlineStr">
@@ -2655,7 +2655,11 @@
           <t>Apply ↗</t>
         </is>
       </c>
-      <c r="N32" t="inlineStr"/>
+      <c r="N32" s="3" t="inlineStr">
+        <is>
+          <t>Mach_Industries_Software_Engineer_New_Grad_Softwar_82c258.pdf</t>
+        </is>
+      </c>
       <c r="O32" s="3" t="inlineStr">
         <is>
           <t>levels.fyi ↗</t>
@@ -2672,38 +2676,38 @@
         <v>32</v>
       </c>
       <c r="B33" s="5" t="n">
-        <v>30</v>
+        <v>12</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>$95k–$130k</t>
+          <t>$250k–$350k</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Vector Atomic</t>
+          <t>TikTok</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Associate Firmware Engineer - Firmware</t>
+          <t>Machine Learning Engineer Graduate - E-Commerce Recommendation Foundation - PhD</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Pleasanton, CA</t>
+          <t>Seattle, WA</t>
         </is>
       </c>
       <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr">
         <is>
-          <t>This is an embedded/firmware role at a quantum-hardware company — squarely in the candidate's stated low-fit bucket (hardware/embedded-only, EE-centric), with no backend, distributed-systems, cloud, or AI-infra surface; only the C/C++/Rust overlap and systems concentration keep it from scoring lower, and the on-site Pleasanton requirement plus likely sub-$120k associate-tier comp further weaken the match.</t>
+          <t>Hard PhD requirement plus a research profile (LLM pre/post-training, generative recommendation, NeurIPS/ICML-tier publications) that a BS-level backend/distributed-systems candidate cannot satisfy — the AI/RAG experience is applied infra, not foundation-model research.</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>Vector Atomic is a small deep-tech quantum-sensing startup (atomic clocks/inertial sensors, DoD-adjacent funding), not a big-tech or high-comp software firm. New-grad "Associate" firmware roles there typically land around $95-125k base with modest early-stage equity and limited bonus; the scraped "29.2" in the posting may even hint at an hourly/associate-tier rate, which would push the low end down. Band is wide because private startup comp data for this company is sparse — this is an estimate, not fact.</t>
+          <t>Posting states base $153,900–$300,960 for Seattle; TikTok PhD MLE new-grad offers typically land in the low-to-mid $200k base range plus RSUs (~$40–100k/yr) and bonus, putting realistic total comp for a fresh PhD around $250k–$350k. Band is wide because TikTok's ML research bands are unusually broad and heavily calibrated to publication record.</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -2713,7 +2717,7 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>scored</t>
+          <t>tailored</t>
         </is>
       </c>
       <c r="M33" s="3" t="inlineStr">
@@ -2721,7 +2725,11 @@
           <t>Apply ↗</t>
         </is>
       </c>
-      <c r="N33" t="inlineStr"/>
+      <c r="N33" s="3" t="inlineStr">
+        <is>
+          <t>TikTok_Machine_Learning_Engineer_Graduate_E_Commer_499a7c.pdf</t>
+        </is>
+      </c>
       <c r="O33" s="3" t="inlineStr">
         <is>
           <t>levels.fyi ↗</t>
@@ -2738,38 +2746,38 @@
         <v>33</v>
       </c>
       <c r="B34" s="5" t="n">
-        <v>33</v>
+        <v>12</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>$78k–$108k</t>
+          <t>$200k–$300k</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t xml:space="preserve">Seagate Technology </t>
+          <t>ByteDance</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Firmware Engineer</t>
+          <t>Video/Image AI/ML Software Engineer Graduate - Multimedia</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Longmont, CO</t>
+          <t>San Diego, CA</t>
         </is>
       </c>
       <c r="G34" t="inlineStr"/>
       <c r="H34" t="inlineStr"/>
       <c r="I34" t="inlineStr">
         <is>
-          <t>Embedded C/C++ firmware for HDDs is squarely in the candidate's low-fit bucket (hardware-adjacent, EE-centric) despite tangential overlap with his storage-engine/LSM-tree work and C/C++ fluency, and the posted base of $72.6-103.8k sits well below his ~130k anchor.</t>
+          <t>Hard PhD requirement (candidate is a 2027 bachelor's-level new grad) combined with a deeply specialized video codec / image-quality-algorithm domain (VMAF, PSNR, SSIM, AVC/HEVC/AV1, FPGA/ASIC C-models, RTOS/embedded) that has almost no overlap with his distributed-systems, backend, and AI-infra background.</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>Posting states base $72,571-$103,784 for Longmont, CO; adding Seagate's discretionary bonus (~5-8%) and ESPP but no meaningful RSU grant at NCG level puts realistic TC in the high-70s to ~108k — hardware-tier compensation, roughly 20-40% under the candidate's target.</t>
+          <t>ByteDance is a top-of-market payer; the posting itself lists $122.6k–$301k base for this PhD-level San Diego role, plus RSUs and bonus. PhD new-grad hires typically land in the upper-middle of that band, so ~$200–300k TC is realistic here. Note this is a PhD-track number — a bachelor's new-grad SWE at ByteDance would be closer to $180–230k TC, and this specific req would not be open to him.</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -2804,38 +2812,38 @@
         <v>34</v>
       </c>
       <c r="B35" s="5" t="n">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>$75k–$95k</t>
+          <t>$80k–$105k</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Securian Financial Group</t>
+          <t>RTX</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Engineering Analyst</t>
+          <t>Software Engineer 1</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>St Paul, MN</t>
+          <t>Cedar Rapids, IA</t>
         </is>
       </c>
       <c r="G35" t="inlineStr"/>
       <c r="H35" t="inlineStr"/>
       <c r="I35" t="inlineStr">
         <is>
-          <t>Generic entry-level enterprise application/IT engineering role at an insurance carrier — technically adjacent but with no distributed-systems, infra, or AI depth, hybrid-onsite in a non-target metro, and a posted base band whose midpoint sits far below the candidate's ~130k TC anchor.</t>
+          <t>Generic entry-level SWE title is nominally on-profile, but RTX/Collins avionics work in Cedar Rapids skews embedded/safety-critical C rather than distributed systems or AI infra, almost certainly requires clearance eligibility (candidate has none), and the TC ceiling sits well under the ~130k anchor.</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>Posting states base range $55,700–$103,400; a new grad would land in the lower-middle (~$72–85k). Add performance-tied 401k contribution (target 5%, up to 10%) and a company-funded pension; no equity. Midwest insurance-carrier tier — well below FAANG/Wayfair-level new-grad comp.</t>
+          <t>Description body failed to scrape (cookie banner only), so this is based on general knowledge: RTX/Collins Aerospace in Cedar Rapids, IA is defense-primes tier — new-grad SWE 1 base typically ~$75-95k with a small bonus, and low-COL Iowa pulls it further down. Defense primes also commonly gate these roles on US citizenship plus clearance eligibility. Band is wide given the missing posting text.</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
@@ -2874,34 +2882,34 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>$72k–$95k</t>
+          <t>$95k–$130k</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>AbbVie</t>
+          <t>Vector Atomic</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Associate Software Engineer 1</t>
+          <t>Associate Firmware Engineer - Firmware</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>North Chicago, IL</t>
+          <t>Pleasanton, CA</t>
         </is>
       </c>
       <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr"/>
       <c r="I36" t="inlineStr">
         <is>
-          <t>Generic pharma-IT associate SWE role centered on GxP documentation, vendor estimates, and supervised routine tasks rather than backend/distributed-systems or AI-infra engineering, and the posted comp band sits well below Nate's ~120k floor — the one bright spot is the "agentic workflows and LLMs" preferred qualification, which he over-satisfies.</t>
+          <t>This is an embedded/firmware role at a quantum-hardware company — squarely in the candidate's stated low-fit bucket (hardware/embedded-only, EE-centric), with no backend, distributed-systems, cloud, or AI-infra surface; only the C/C++/Rust overlap and systems concentration keep it from scoring lower, and the on-site Pleasanton requirement plus likely sub-$120k associate-tier comp further weaken the match.</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>Posting discloses base 58,656–103,500 (Workday grade 12); a zero-experience new grad in North Chicago realistically lands in the lower-middle of that band (~70–88k base), plus a modest short-term incentive (~5–8%) and 401k match. AbbVie is a large-pharma non-tech employer, so software comp tracks internal IT grades rather than tech-industry scales — no equity component typical at this level.</t>
+          <t>Vector Atomic is a small deep-tech quantum-sensing startup (atomic clocks/inertial sensors, DoD-adjacent funding), not a big-tech or high-comp software firm. New-grad "Associate" firmware roles there typically land around $95-125k base with modest early-stage equity and limited bonus; the scraped "29.2" in the posting may even hint at an hourly/associate-tier rate, which would push the low end down. Band is wide because private startup comp data for this company is sparse — this is an estimate, not fact.</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
@@ -2936,38 +2944,38 @@
         <v>36</v>
       </c>
       <c r="B37" s="5" t="n">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>$78k–$105k</t>
+          <t>$78k–$108k</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Abbott</t>
+          <t xml:space="preserve">Seagate Technology </t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Associate Software Engineer - Multiple Teams</t>
+          <t>Firmware Engineer</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Irving, TX</t>
+          <t>Longmont, CO</t>
         </is>
       </c>
       <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr"/>
       <c r="I37" t="inlineStr">
         <is>
-          <t>Regulated medical-device C++ work across embedded/desktop/IoT connectivity in a mandatory on-site Irving TX role is well off Nate's backend/distributed-systems/AI-infra profile, and the posted base range tops out below his ~130k TC anchor.</t>
+          <t>Embedded C/C++ firmware for HDDs is squarely in the candidate's low-fit bucket (hardware-adjacent, EE-centric) despite tangential overlap with his storage-engine/LSM-tree work and C/C++ fluency, and the posted base of $72.6-103.8k sits well below his ~130k anchor.</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>Posting states base $50.7k–$101.3k; a new grad realistically lands in the low-to-mid part of that band (~$75–95k base) plus a modest ~5% bonus and strong retirement match typical of Abbott's non-tech-tier medtech comp — TX cost of living keeps offers lower than coastal tech.</t>
+          <t>Posting states base $72,571-$103,784 for Longmont, CO; adding Seagate's discretionary bonus (~5-8%) and ESPP but no meaningful RSU grant at NCG level puts realistic TC in the high-70s to ~108k — hardware-tier compensation, roughly 20-40% under the candidate's target.</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -3002,38 +3010,38 @@
         <v>37</v>
       </c>
       <c r="B38" s="5" t="n">
-        <v>22</v>
+        <v>32</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>$70k–$115k</t>
+          <t>$75k–$95k</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>AmNet Services</t>
+          <t>Securian Financial Group</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Software Systems Engineer 3</t>
+          <t>Engineering Analyst</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Warren, NJ</t>
+          <t>St Paul, MN</t>
         </is>
       </c>
       <c r="G38" t="inlineStr"/>
       <c r="H38" t="inlineStr"/>
       <c r="I38" t="inlineStr">
         <is>
-          <t>Contract role at a small IoT/sensor networking firm requiring 7-10 years of experience (new grads only via fresh CS Master's), on an Erlang backend with no distributed-systems, cloud, or AI-infra overlap — off-profile on seniority, employment type, and stack despite being nominally "backend."</t>
+          <t>Generic entry-level enterprise application/IT engineering role at an insurance carrier — technically adjacent but with no distributed-systems, infra, or AI depth, hybrid-onsite in a non-target metro, and a posted base band whose midpoint sits far below the candidate's ~130k TC anchor.</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>AmNet Services (America Networks) is a small private sensor/networking and staffing-style firm with no public comp tier, so this is a wide, low-confidence band. Posting is explicitly a Contract engagement, which typically means hourly pay (~$40-55/hr for a junior contractor in NJ), no equity, and limited or no benefits. Annualized that lands roughly $85-115k gross at the top end and well below at the bottom — under the candidate's ~$130k anchor and below the ~$120k low-match threshold.</t>
+          <t>Posting states base range $55,700–$103,400; a new grad would land in the lower-middle (~$72–85k). Add performance-tied 401k contribution (target 5%, up to 10%) and a company-funded pension; no equity. Midwest insurance-carrier tier — well below FAANG/Wayfair-level new-grad comp.</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -3068,7 +3076,7 @@
         <v>38</v>
       </c>
       <c r="B39" s="5" t="n">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -3077,29 +3085,29 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Barrios</t>
+          <t>AbbVie</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Software Developer</t>
+          <t>Associate Software Engineer 1</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Houston, TX</t>
+          <t>North Chicago, IL</t>
         </is>
       </c>
       <c r="G39" t="inlineStr"/>
       <c r="H39" t="inlineStr"/>
       <c r="I39" t="inlineStr">
         <is>
-          <t>Off-profile: C#/.NET web-app maintenance at a NASA support contractor in Houston, with clearance-eligibility requirements and gov-contractor pay well under the candidate's ~130k anchor — little overlap with his Rust/Java distributed-systems and AI-infra strengths beyond incidental Docker/K8s/CI-CD exposure.</t>
+          <t>Generic pharma-IT associate SWE role centered on GxP documentation, vendor estimates, and supervised routine tasks rather than backend/distributed-systems or AI-infra engineering, and the posted comp band sits well below Nate's ~120k floor — the one bright spot is the "agentic workflows and LLMs" preferred qualification, which he over-satisfies.</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>Estimate only. Barrios Technology is a mid-size NASA/JSC engineering services contractor; government cost-plus contract labor rates put entry-level SWE base around 70-88k in Houston, with minimal bonus/equity (typically none), so TC ≈ base. Band is wide because the posting spans 0-5 YOE and comp data for this employer is sparse.</t>
+          <t>Posting discloses base 58,656–103,500 (Workday grade 12); a zero-experience new grad in North Chicago realistically lands in the lower-middle of that band (~70–88k base), plus a modest short-term incentive (~5–8%) and 401k match. AbbVie is a large-pharma non-tech employer, so software comp tracks internal IT grades rather than tech-industry scales — no equity component typical at this level.</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
@@ -3134,38 +3142,38 @@
         <v>39</v>
       </c>
       <c r="B40" s="5" t="n">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>$70k–$90k</t>
+          <t>$78k–$105k</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>D.R. Horton</t>
+          <t>Abbott</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Application Developer 1</t>
+          <t>Associate Software Engineer - Multiple Teams</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Arlington, TX</t>
+          <t>Irving, TX</t>
         </is>
       </c>
       <c r="G40" t="inlineStr"/>
       <c r="H40" t="inlineStr"/>
       <c r="I40" t="inlineStr">
         <is>
-          <t>Internal .NET/C#/React business-application and legacy-app maintenance work at a homebuilder's corporate IT group, which has essentially no overlap with the candidate's backend/distributed-systems, cloud-infra, or AI-platform focus and sits at a much lower comp and technical tier.</t>
+          <t>Regulated medical-device C++ work across embedded/desktop/IoT connectivity in a mandatory on-site Irving TX role is well off Nate's backend/distributed-systems/AI-infra profile, and the posted base range tops out below his ~130k TC anchor.</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>Non-tech Fortune 500 homebuilder; corporate IT cost-center role in the Dallas-Fort Worth market, posting accepts a HS diploma with 0-1 years experience. Estimate assumes ~$70-85k base plus modest bonus/ESPP; band is approximate since D.R. Horton IT comp is not widely reported on levels.fyi.</t>
+          <t>Posting states base $50.7k–$101.3k; a new grad realistically lands in the low-to-mid part of that band (~$75–95k base) plus a modest ~5% bonus and strong retirement match typical of Abbott's non-tech-tier medtech comp — TX cost of living keeps offers lower than coastal tech.</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -3200,38 +3208,38 @@
         <v>40</v>
       </c>
       <c r="B41" s="5" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>$85k–$115k</t>
+          <t>$70k–$115k</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>RTX</t>
+          <t>AmNet Services</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Software Engineer 1</t>
+          <t>Software Systems Engineer 3</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Anaheim, CA</t>
+          <t>Warren, NJ</t>
         </is>
       </c>
       <c r="G41" t="inlineStr"/>
       <c r="H41" t="inlineStr"/>
       <c r="I41" t="inlineStr">
         <is>
-          <t>Hard-blocked: the req demands an active TS/SCI with polygraph on day 1 and is earmarked for an RTX intern converting to full-time, and the C++/Qt/Angular defense-systems work plus sub-$120k band misses both the candidate's clearance-free constraint and TC anchor.</t>
+          <t>Contract role at a small IoT/sensor networking firm requiring 7-10 years of experience (new grads only via fresh CS Master's), on an Erlang backend with no distributed-systems, cloud, or AI-infra overlap — off-profile on seniority, employment type, and stack despite being nominally "backend."</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>Posting states salary range 62,900–119,700 USD; RTX new-grad SWE offers typically land near the lower-middle of that band (~$85–100k base) plus modest 401k match and small/no annual incentive at level 1. Defense-primes pay well below the candidate's ~$130–165k anchor; cleared work in Anaheim may add a slight premium, hence the top of the band.</t>
+          <t>AmNet Services (America Networks) is a small private sensor/networking and staffing-style firm with no public comp tier, so this is a wide, low-confidence band. Posting is explicitly a Contract engagement, which typically means hourly pay (~$40-55/hr for a junior contractor in NJ), no equity, and limited or no benefits. Annualized that lands roughly $85-115k gross at the top end and well below at the bottom — under the candidate's ~$130k anchor and below the ~$120k low-match threshold.</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
@@ -3266,42 +3274,38 @@
         <v>41</v>
       </c>
       <c r="B42" s="5" t="n">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>$85k–$115k</t>
+          <t>$72k–$95k</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>General Motors</t>
+          <t>Barrios</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Software Engineer</t>
+          <t>Software Developer</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Warren, MI</t>
+          <t>Houston, TX</t>
         </is>
       </c>
       <c r="G42" t="inlineStr"/>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>graduating between december 2025</t>
-        </is>
-      </c>
+      <c r="H42" t="inlineStr"/>
       <c r="I42" t="inlineStr">
         <is>
-          <t>Hard-disqualifying graduation window (Dec 2025–Aug 2026 vs. candidate's May 2027) combined with an Android/Kotlin infotainment HMI focus that sits far from his backend/distributed-systems/AI-infra profile, in a hybrid Warren, MI role paying below his TC floor.</t>
+          <t>Off-profile: C#/.NET web-app maintenance at a NASA support contractor in Houston, with clearance-eligibility requirements and gov-contractor pay well under the candidate's ~130k anchor — little overlap with his Rust/Java distributed-systems and AI-infra strengths beyond incidental Docker/K8s/CI-CD exposure.</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>GM is a non-tech-tier automotive employer; entry-level SWE base in Warren, MI typically ~$80–100k plus modest performance bonus (~5-10%) and relocation, putting TC roughly $85–115k — well below the candidate's ~$130k anchor. Estimate from general knowledge of GM/Big Three new-grad pay in low-cost Midwest markets, not from the posting (no range disclosed).</t>
+          <t>Estimate only. Barrios Technology is a mid-size NASA/JSC engineering services contractor; government cost-plus contract labor rates put entry-level SWE base around 70-88k in Houston, with minimal bonus/equity (typically none), so TC ≈ base. Band is wide because the posting spans 0-5 YOE and comp data for this employer is sparse.</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
@@ -3336,38 +3340,38 @@
         <v>42</v>
       </c>
       <c r="B43" s="5" t="n">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>$72k–$92k</t>
+          <t>$70k–$90k</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Integration Innovation (i3)</t>
+          <t>D.R. Horton</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Associate Software Developer - COMPASS</t>
+          <t>Application Developer 1</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Huntsville, AL</t>
+          <t>Arlington, TX</t>
         </is>
       </c>
       <c r="G43" t="inlineStr"/>
       <c r="H43" t="inlineStr"/>
       <c r="I43" t="inlineStr">
         <is>
-          <t>Requires an active/obtainable DoD Secret clearance and on-site residency near Redstone Arsenal with a C#/HTML/CSS stack, all of which conflict with the candidate's stated constraints and backend/distributed-systems strengths, despite some Azure/AWS microservices and event-queue overlap.</t>
+          <t>Internal .NET/C#/React business-application and legacy-app maintenance work at a homebuilder's corporate IT group, which has essentially no overlap with the candidate's backend/distributed-systems, cloud-infra, or AI-platform focus and sits at a much lower comp and technical tier.</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>Mid-size employee-owned defense/government services contractor (i3) in Huntsville, AL — low cost-of-living market with cost-plus contract rate structures. Typical 0-3 yr associate developer base ~$70-85k plus 401(k) match and ESOP; no equity grant or notable signing bonus. Band is a general-knowledge estimate for the defense-services tier, not verified company data, and falls well below the candidate's ~$130k anchor.</t>
+          <t>Non-tech Fortune 500 homebuilder; corporate IT cost-center role in the Dallas-Fort Worth market, posting accepts a HS diploma with 0-1 years experience. Estimate assumes ~$70-85k base plus modest bonus/ESPP; band is approximate since D.R. Horton IT comp is not widely reported on levels.fyi.</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
@@ -3402,38 +3406,38 @@
         <v>43</v>
       </c>
       <c r="B44" s="5" t="n">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>$45k–$62k</t>
+          <t>$85k–$115k</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Trustpilot</t>
+          <t>RTX</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Software Engineer 1 - Trust Tech</t>
+          <t>Software Engineer 1</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Edinburgh, UK</t>
+          <t>Anaheim, CA</t>
         </is>
       </c>
       <c r="G44" t="inlineStr"/>
       <c r="H44" t="inlineStr"/>
       <c r="I44" t="inlineStr">
         <is>
-          <t>Backend-adjacent work the candidate could handle, but it is a UK/EU-located role (Edinburgh/London/Copenhagen) he lacks work authorization for, and the Node/TypeScript/React full-stack stack is off his Rust/Java distributed-systems and AI-infra profile.</t>
+          <t>Hard-blocked: the req demands an active TS/SCI with polygraph on day 1 and is earmarked for an RTX intern converting to full-time, and the C++/Qt/Angular defense-systems work plus sub-$120k band misses both the candidate's clearance-free constraint and TC anchor.</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>Trustpilot is a profitable FTSE-250 tech company, not a top-tier payer. Edinburgh/UK graduate-to-SWE I base bands typically run ~£35-48k with a modest bonus, converting to roughly $45-62k USD — well below the candidate's ~$130k anchor. Wide-ish band; UK pay data for this specific level is inferred from general UK market rates rather than verified comp reports.</t>
+          <t>Posting states salary range 62,900–119,700 USD; RTX new-grad SWE offers typically land near the lower-middle of that band (~$85–100k base) plus modest 401k match and small/no annual incentive at level 1. Defense-primes pay well below the candidate's ~$130–165k anchor; cleared work in Anaheim may add a slight premium, hence the top of the band.</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
@@ -3468,38 +3472,42 @@
         <v>44</v>
       </c>
       <c r="B45" s="5" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>$48k–$65k</t>
+          <t>$85k–$115k</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Trustpilot</t>
+          <t>General Motors</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Software Engineer 1 - Trust Tech</t>
+          <t>Software Engineer</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>London, UK</t>
+          <t>Warren, MI</t>
         </is>
       </c>
       <c r="G45" t="inlineStr"/>
-      <c r="H45" t="inlineStr"/>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>graduating between december 2025</t>
+        </is>
+      </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>UK/Denmark-only role (no US location or stated sponsorship) with a Node.js/TypeScript full-stack + React internal-tooling focus, which misses the candidate's Java/Rust/Go backend and distributed-systems profile despite some AWS/Postgres and applied-AI overlap.</t>
+          <t>Hard-disqualifying graduation window (Dec 2025–Aug 2026 vs. candidate's May 2027) combined with an Android/Kotlin infotainment HMI focus that sits far from his backend/distributed-systems/AI-infra profile, in a hybrid Warren, MI role paying below his TC floor.</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>Estimate, not fact: Trustpilot is a profitable FTSE-250 mid-tier tech company; London/Edinburgh graduate SWE I base typically ~£38-50k plus a modest bonus, converting to roughly $48-65k USD. UK/EU pay scales sit far below the candidate's ~$130-165k US anchor, so the shortfall is structural rather than negotiable.</t>
+          <t>GM is a non-tech-tier automotive employer; entry-level SWE base in Warren, MI typically ~$80–100k plus modest performance bonus (~5-10%) and relocation, putting TC roughly $85–115k — well below the candidate's ~$130k anchor. Estimate from general knowledge of GM/Big Three new-grad pay in low-cost Midwest markets, not from the posting (no range disclosed).</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
@@ -3534,38 +3542,38 @@
         <v>45</v>
       </c>
       <c r="B46" s="5" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>$65k–$90k</t>
+          <t>$72k–$92k</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>9to9 Software Solutions</t>
+          <t>Integration Innovation (i3)</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Entry Level .NET Developer</t>
+          <t>Associate Software Developer - COMPASS</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Louisville, CO</t>
+          <t>Huntsville, AL</t>
         </is>
       </c>
       <c r="G46" t="inlineStr"/>
       <c r="H46" t="inlineStr"/>
       <c r="I46" t="inlineStr">
         <is>
-          <t>Hard-blocked by the SECRET clearance and Security+ certification requirements, and the work is legacy Java/.NET web-app consulting with no backend-distributed-systems, infra, or AI-platform overlap.</t>
+          <t>Requires an active/obtainable DoD Secret clearance and on-site residency near Redstone Arsenal with a C#/HTML/CSS stack, all of which conflict with the candidate's stated constraints and backend/distributed-systems strengths, despite some Azure/AWS microservices and event-queue overlap.</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>Small IT staffing/consulting firm (Connecticut-based body shop) with no public comp data; estimate based on typical entry-level government-contract staffing pay in a mid-cost Colorado market. Wide band due to unknown company; likely far below the candidate's ~130k anchor.</t>
+          <t>Mid-size employee-owned defense/government services contractor (i3) in Huntsville, AL — low cost-of-living market with cost-plus contract rate structures. Typical 0-3 yr associate developer base ~$70-85k plus 401(k) match and ESOP; no equity grant or notable signing bonus. Band is a general-knowledge estimate for the defense-services tier, not verified company data, and falls well below the candidate's ~$130k anchor.</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
@@ -3600,38 +3608,38 @@
         <v>46</v>
       </c>
       <c r="B47" s="5" t="n">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>$65k–$90k</t>
+          <t>$45k–$62k</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>9to9 Software Solutions</t>
+          <t>Trustpilot</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Java Developer</t>
+          <t>Software Engineer 1 - Trust Tech</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Portland, OR</t>
+          <t>Edinburgh, UK</t>
         </is>
       </c>
       <c r="G47" t="inlineStr"/>
       <c r="H47" t="inlineStr"/>
       <c r="I47" t="inlineStr">
         <is>
-          <t>Hard disqualifier: the posting requires an interim SECRET clearance to begin work plus existing CompTIA Security+ certification, which the candidate explicitly lacks — and the role itself is legacy full-stack JSP/Hibernate/WebLogic consulting work with graphic-designer/site-design duties, far from backend distributed systems or AI infra, at a comp tier well under the 120k floor.</t>
+          <t>Backend-adjacent work the candidate could handle, but it is a UK/EU-located role (Edinburgh/London/Copenhagen) he lacks work authorization for, and the Node/TypeScript/React full-stack stack is off his Rust/Java distributed-systems and AI-infra profile.</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>9to9 Software Solutions is a small Connecticut-based IT services/staffing consultancy, not a product company — entry-level Java/consulting roles at this tier typically pay near-flat base with minimal bonus or equity. Wide band due to low visibility into this specific firm's pay; Portland, OR cost-of-living offers slight upward pressure but government-contract billing rates cap entry-level comp. Well below the candidate's ~130-165k anchor.</t>
+          <t>Trustpilot is a profitable FTSE-250 tech company, not a top-tier payer. Edinburgh/UK graduate-to-SWE I base bands typically run ~£35-48k with a modest bonus, converting to roughly $45-62k USD — well below the candidate's ~$130k anchor. Wide-ish band; UK pay data for this specific level is inferred from general UK market rates rather than verified comp reports.</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
@@ -3666,38 +3674,38 @@
         <v>47</v>
       </c>
       <c r="B48" s="5" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>$60k–$85k</t>
+          <t>$48k–$65k</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>9to9 Software Solutions</t>
+          <t>Trustpilot</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Entry Level Java Developer</t>
+          <t>Software Engineer 1 - Trust Tech</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Silver Creek, NY</t>
+          <t>London, UK</t>
         </is>
       </c>
       <c r="G48" t="inlineStr"/>
       <c r="H48" t="inlineStr"/>
       <c r="I48" t="inlineStr">
         <is>
-          <t>IT staffing/consulting shop posting a legacy Java web-app contract role that hard-requires an interim SECRET clearance plus Security+ certification — an explicit disqualifier for this candidate — and the work (JSP/WebLogic/Subversion, "site-design instincts") is far below his distributed-systems/AI-infra profile and TC anchor.</t>
+          <t>UK/Denmark-only role (no US location or stated sponsorship) with a Node.js/TypeScript full-stack + React internal-tooling focus, which misses the candidate's Java/Rust/Go backend and distributed-systems profile despite some AWS/Postgres and applied-AI overlap.</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>9to9 Software Solutions is a small Connecticut-based IT services/staffing firm with no public compensation data, so this is a wide, low-confidence band inferred from typical entry-level government-contract Java staffing rates (largely base salary, minimal equity or bonus). Well below the candidate's ~130-165k anchor.</t>
+          <t>Estimate, not fact: Trustpilot is a profitable FTSE-250 mid-tier tech company; London/Edinburgh graduate SWE I base typically ~£38-50k plus a modest bonus, converting to roughly $48-65k USD. UK/EU pay scales sit far below the candidate's ~$130-165k US anchor, so the shortfall is structural rather than negotiable.</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
@@ -3736,7 +3744,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>$60k–$85k</t>
+          <t>$65k–$90k</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -3746,24 +3754,24 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Entry Level Java Developer</t>
+          <t>Entry Level .NET Developer</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Elk Grove, CA</t>
+          <t>Louisville, CO</t>
         </is>
       </c>
       <c r="G49" t="inlineStr"/>
       <c r="H49" t="inlineStr"/>
       <c r="I49" t="inlineStr">
         <is>
-          <t>Contract staffing role that hard-requires an interim/full SECRET clearance and Security+ certification (both explicit candidate disqualifiers), on legacy JSP/Hibernate/WebLogic web-app work with design responsibilities — off-profile for a backend/distributed-systems new grad and almost certainly below the ~120k TC floor.</t>
+          <t>Hard-blocked by the SECRET clearance and Security+ certification requirements, and the work is legacy Java/.NET web-app consulting with no backend-distributed-systems, infra, or AI-platform overlap.</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>No public comp data for 9to9 Software Solutions — a small CT-based IT staffing/consulting firm. Band inferred from typical entry-level contract Java roles at government-contract body shops (roughly $30–40/hr, little to no bonus or equity). Wide band reflects low confidence and the contract (non-FTE) structure.</t>
+          <t>Small IT staffing/consulting firm (Connecticut-based body shop) with no public comp data; estimate based on typical entry-level government-contract staffing pay in a mid-cost Colorado market. Wide band due to unknown company; likely far below the candidate's ~130k anchor.</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
@@ -3798,38 +3806,38 @@
         <v>49</v>
       </c>
       <c r="B50" s="5" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>$85k–$110k</t>
+          <t>$65k–$90k</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Cisco</t>
+          <t>9to9 Software Solutions</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Failure Analysis Engineer</t>
+          <t>Java Developer</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Acton, MA</t>
+          <t>Portland, OR</t>
         </is>
       </c>
       <c r="G50" t="inlineStr"/>
       <c r="H50" t="inlineStr"/>
       <c r="I50" t="inlineStr">
         <is>
-          <t>EE/photonics lab failure-analysis role (coherent optical transceivers, oscilloscopes, RF/optical spectrum analyzers) with zero software content, requiring prior hands-on FA experience — squarely in the candidate's hardware/embedded-only low-fit bucket, and the immediate onsite start conflicts with a mid-2027 new-grad timeline.</t>
+          <t>Hard disqualifier: the posting requires an interim SECRET clearance to begin work plus existing CompTIA Security+ certification, which the candidate explicitly lacks — and the role itself is legacy full-stack JSP/Hibernate/WebLogic consulting work with graphic-designer/site-design duties, far from backend distributed systems or AI infra, at a comp tier well under the 120k floor.</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>Posting explicitly states a new-hire base range of $79,200-$100,400; adding a ~5-8% Cisco bonus and a small RSU grant yields roughly $85-110k TC. Cisco's Supply Chain and Manufacturing Ops org pays materially below its SWE ladder, and a new grad would land in the lower half of the posted band, so the realistic center is ~$90k — below the candidate's ~120k low-match floor.</t>
+          <t>9to9 Software Solutions is a small Connecticut-based IT services/staffing consultancy, not a product company — entry-level Java/consulting roles at this tier typically pay near-flat base with minimal bonus or equity. Wide band due to low visibility into this specific firm's pay; Portland, OR cost-of-living offers slight upward pressure but government-contract billing rates cap entry-level comp. Well below the candidate's ~130-165k anchor.</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
@@ -3864,38 +3872,38 @@
         <v>50</v>
       </c>
       <c r="B51" s="5" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>$90k–$110k</t>
+          <t>$60k–$85k</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Microchip Technology</t>
+          <t>9to9 Software Solutions</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Reliability Engineer 2</t>
+          <t>Entry Level Java Developer</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Chandler, AZ</t>
+          <t>Silver Creek, NY</t>
         </is>
       </c>
       <c r="G51" t="inlineStr"/>
       <c r="H51" t="inlineStr"/>
       <c r="I51" t="inlineStr">
         <is>
-          <t>This is an EE-centric hardware reliability role (device physics, transistor-level ICs, HTOL burn-in, lab bench equipment, JMP/LabVIEW) with essentially no backend, distributed-systems, or AI-infra content — squarely in the candidate's stated low-fit bucket, and it's an immediate-start req rather than a May 2027 new-grad pipeline.</t>
+          <t>IT staffing/consulting shop posting a legacy Java web-app contract role that hard-requires an interim SECRET clearance plus Security+ certification — an explicit disqualifier for this candidate — and the work (JSP/WebLogic/Subversion, "site-design instincts") is far below his distributed-systems/AI-infra profile and TC anchor.</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>Microchip is a mid-tier semiconductor employer in a low-cost metro (Chandler, AZ); new-grad/Engineer II reliability roles there typically pay ~$80-95k base plus modest bonus/ESPP/small RSU, landing around $90-110k TC. Estimate based on general semiconductor-industry knowledge, not a verified data point.</t>
+          <t>9to9 Software Solutions is a small Connecticut-based IT services/staffing firm with no public compensation data, so this is a wide, low-confidence band inferred from typical entry-level government-contract Java staffing rates (largely base salary, minimal equity or bonus). Well below the candidate's ~130-165k anchor.</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
@@ -3930,38 +3938,38 @@
         <v>51</v>
       </c>
       <c r="B52" s="5" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>$75k–$95k</t>
+          <t>$60k–$85k</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>RTX</t>
+          <t>9to9 Software Solutions</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Software Engineer 1</t>
+          <t>Entry Level Java Developer</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Fort Wayne, IN</t>
+          <t>Elk Grove, CA</t>
         </is>
       </c>
       <c r="G52" t="inlineStr"/>
       <c r="H52" t="inlineStr"/>
       <c r="I52" t="inlineStr">
         <is>
-          <t>Hard-blocked: the req demands an active DoD Secret clearance from day 1 and is explicitly reserved for an RTX intern converting to full-time, and the Ada/Java C2 work in onsite Fort Wayne at 57–109k misses the candidate's distributed-systems/AI-infra profile and ~130k TC anchor.</t>
+          <t>Contract staffing role that hard-requires an interim/full SECRET clearance and Security+ certification (both explicit candidate disqualifiers), on legacy JSP/Hibernate/WebLogic web-app work with design responsibilities — off-profile for a backend/distributed-systems new grad and almost certainly below the ~120k TC floor.</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>Posted range 57.2k–108.8k; RTX defense new-grad SWE typically lands ~75–90k base with small (0–5%) bonus and no equity, and Fort Wayne IN is a low cost-of-living site so offers skew to the lower-middle of the band. Well below the candidate's ~130k anchor.</t>
+          <t>No public comp data for 9to9 Software Solutions — a small CT-based IT staffing/consulting firm. Band inferred from typical entry-level contract Java roles at government-contract body shops (roughly $30–40/hr, little to no bonus or equity). Wide band reflects low confidence and the contract (non-FTE) structure.</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
@@ -3996,38 +4004,38 @@
         <v>52</v>
       </c>
       <c r="B53" s="5" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>$68k–$80k</t>
+          <t>$85k–$110k</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Axos Bank</t>
+          <t>Cisco</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Data Engineer</t>
+          <t>Failure Analysis Engineer</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>San Diego, CA</t>
+          <t>Acton, MA</t>
         </is>
       </c>
       <c r="G53" t="inlineStr"/>
       <c r="H53" t="inlineStr"/>
       <c r="I53" t="inlineStr">
         <is>
-          <t>SQL Server/SSIS/Salesforce-Apex BI rotational program at ~$75k TC — off-profile for a backend/distributed-systems candidate and far below the ~$130k anchor.</t>
+          <t>EE/photonics lab failure-analysis role (coherent optical transceivers, oscilloscopes, RF/optical spectrum analyzers) with zero software content, requiring prior hands-on FA experience — squarely in the candidate's hardware/embedded-only low-fit bucket, and the immediate onsite start conflicts with a mid-2027 new-grad timeline.</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>Posting states an explicit flat rate of $30.00/hr (~$62.4k base at 2,080 hrs) plus a 10% discretionary cash bonus target and a 10% discretionary RSU target; band spans low-to-full attainment of both. Consistent with Axos as a mid-size digital bank running a below-market entry-level rotational pipeline rather than a comp-competitive tech employer.</t>
+          <t>Posting explicitly states a new-hire base range of $79,200-$100,400; adding a ~5-8% Cisco bonus and a small RSU grant yields roughly $85-110k TC. Cisco's Supply Chain and Manufacturing Ops org pays materially below its SWE ladder, and a new grad would land in the lower half of the posted band, so the realistic center is ~$90k — below the candidate's ~120k low-match floor.</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
@@ -4062,38 +4070,38 @@
         <v>53</v>
       </c>
       <c r="B54" s="5" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>$60k–$85k</t>
+          <t>$90k–$110k</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>9to9 Software Solutions</t>
+          <t>Microchip Technology</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Entry Level Software Developer</t>
+          <t>Reliability Engineer 2</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Randolph AFB, TX</t>
+          <t>Chandler, AZ</t>
         </is>
       </c>
       <c r="G54" t="inlineStr"/>
       <c r="H54" t="inlineStr"/>
       <c r="I54" t="inlineStr">
         <is>
-          <t>Requires an interim SECRET clearance to start plus Security+ certification (candidate has no clearance — an explicit disqualifier), and the work is legacy Java/JSP/WebLogic/Subversion web development at an IT staffing firm on an Air Force base, with no overlap with the candidate's distributed-systems, cloud-infra, or AI-platform strengths.</t>
+          <t>This is an EE-centric hardware reliability role (device physics, transistor-level ICs, HTOL burn-in, lab bench equipment, JMP/LabVIEW) with essentially no backend, distributed-systems, or AI-infra content — squarely in the candidate's stated low-fit bucket, and it's an immediate-start req rather than a May 2027 new-grad pipeline.</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>9to9 Software Solutions is a small Connecticut-based IT services/staffing firm placing contractors on government contracts. This tier typically pays far below product-company new-grad bands, and clearance-gated entry-level contract roles rarely carry equity or meaningful bonus. No public comp data for this company, so the band is wide and low-confidence; it falls well under the candidate's ~$120k floor.</t>
+          <t>Microchip is a mid-tier semiconductor employer in a low-cost metro (Chandler, AZ); new-grad/Engineer II reliability roles there typically pay ~$80-95k base plus modest bonus/ESPP/small RSU, landing around $90-110k TC. Estimate based on general semiconductor-industry knowledge, not a verified data point.</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
@@ -4128,38 +4136,38 @@
         <v>54</v>
       </c>
       <c r="B55" s="5" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>$60k–$90k</t>
+          <t>$75k–$95k</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>9to9 Software Solutions</t>
+          <t>RTX</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Software Developer</t>
+          <t>Software Engineer 1</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Pittsburgh, PA</t>
+          <t>Fort Wayne, IN</t>
         </is>
       </c>
       <c r="G55" t="inlineStr"/>
       <c r="H55" t="inlineStr"/>
       <c r="I55" t="inlineStr">
         <is>
-          <t>Hard-blocked by an explicit interim SECRET clearance + Security+ certification requirement (both listed as minimum quals) that the candidate cannot meet, and the work itself is legacy contract JSP/Hibernate/WebLogic web development at a staffing firm — no overlap with distributed systems, infra, or AI platform work, at contractor-tier pay far below the $130k anchor.</t>
+          <t>Hard-blocked: the req demands an active DoD Secret clearance from day 1 and is explicitly reserved for an RTX intern converting to full-time, and the Ada/Java C2 work in onsite Fort Wayne at 57–109k misses the candidate's distributed-systems/AI-infra profile and ~130k TC anchor.</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>9to9 Software Solutions is a small IT staffing/consulting body shop, and this is an explicitly Contract (not FTE) government-adjacent role — no equity, likely hourly with little or no bonus. Comparable entry-level contract Java dev rates through such firms run roughly $30-45/hr, i.e. ~$60-90k annualized. Low confidence, wide band; well below the candidate's ~$130k anchor.</t>
+          <t>Posted range 57.2k–108.8k; RTX defense new-grad SWE typically lands ~75–90k base with small (0–5%) bonus and no equity, and Fort Wayne IN is a low cost-of-living site so offers skew to the lower-middle of the band. Well below the candidate's ~130k anchor.</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
@@ -4194,38 +4202,38 @@
         <v>55</v>
       </c>
       <c r="B56" s="5" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>$60k–$85k</t>
+          <t>$68k–$80k</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>9to9 Software Solutions</t>
+          <t>Axos Bank</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Entry Level Software Developer</t>
+          <t>Data Engineer</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Copperhill, TN</t>
+          <t>San Diego, CA</t>
         </is>
       </c>
       <c r="G56" t="inlineStr"/>
       <c r="H56" t="inlineStr"/>
       <c r="I56" t="inlineStr">
         <is>
-          <t>Requires an existing interim SECRET clearance and Security+ certification to start (candidate has neither and lists clearance roles as a hard mismatch), and it is a contract legacy Java/JSP/WebLogic web-dev role at a staffing consultancy in rural Copperhill, TN with no distributed-systems, infra, or AI-platform content.</t>
+          <t>SQL Server/SSIS/Salesforce-Apex BI rotational program at ~$75k TC — off-profile for a backend/distributed-systems candidate and far below the ~$130k anchor.</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>Company is not well known publicly — wide, low-confidence band. 9to9 Software Solutions is a small Connecticut-based IT staffing/services consultancy rather than a product company, and this is explicitly a Contract position, implying an hourly rate with minimal-to-no equity or bonus. Cleared entry-level government-contract Java work in a low-cost rural TN market typically pays in the $60-85k equivalent range, well below the candidate's ~$130-165k anchor and under the ~$120k low-match floor.</t>
+          <t>Posting states an explicit flat rate of $30.00/hr (~$62.4k base at 2,080 hrs) plus a 10% discretionary cash bonus target and a 10% discretionary RSU target; band spans low-to-full attainment of both. Consistent with Axos as a mid-size digital bank running a below-market entry-level rotational pipeline rather than a comp-competitive tech employer.</t>
         </is>
       </c>
       <c r="K56" t="inlineStr">
@@ -4260,38 +4268,38 @@
         <v>56</v>
       </c>
       <c r="B57" s="5" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>$65k–$85k</t>
+          <t>$60k–$85k</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>SOSi</t>
+          <t>9to9 Software Solutions</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>PeopleSoft Software Developer</t>
+          <t>Entry Level Software Developer</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Charleston, SC</t>
+          <t>Randolph AFB, TX</t>
         </is>
       </c>
       <c r="G57" t="inlineStr"/>
       <c r="H57" t="inlineStr"/>
       <c r="I57" t="inlineStr">
         <is>
-          <t>Hard-blocked by the Secret clearance requirement (an explicit candidate constraint) and the work is PeopleSoft/PeopleCode ERP maintenance — no overlap with backend distributed systems, Rust/systems, or AI infra — plus onsite 5 days in Charleston at roughly half the target TC.</t>
+          <t>Requires an interim SECRET clearance to start plus Security+ certification (candidate has no clearance — an explicit disqualifier), and the work is legacy Java/JSP/WebLogic/Subversion web development at an IT staffing firm on an Air Force base, with no overlap with the candidate's distributed-systems, cloud-infra, or AI-platform strengths.</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>Defense/government services integrator (SOSi) entry-level ERP developer in Charleston, SC — cleared-work government contracting pay bands are well below product-tech; base likely $65-80k with minimal bonus/equity. Wide band due to no public comp data for SOSi.</t>
+          <t>9to9 Software Solutions is a small Connecticut-based IT services/staffing firm placing contractors on government contracts. This tier typically pays far below product-company new-grad bands, and clearance-gated entry-level contract roles rarely carry equity or meaningful bonus. No public comp data for this company, so the band is wide and low-confidence; it falls well under the candidate's ~$120k floor.</t>
         </is>
       </c>
       <c r="K57" t="inlineStr">
@@ -4330,12 +4338,12 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>$45k–$70k</t>
+          <t>$60k–$90k</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>ERPA</t>
+          <t>9to9 Software Solutions</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -4345,19 +4353,19 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Franklin County, OH</t>
+          <t>Pittsburgh, PA</t>
         </is>
       </c>
       <c r="G58" t="inlineStr"/>
       <c r="H58" t="inlineStr"/>
       <c r="I58" t="inlineStr">
         <is>
-          <t>Contract "training and placement" body-shop posting at an Oracle/PeopleSoft consulting partner targeting candidates with "basic technical skills" — no backend, distributed-systems, or AI-infra content, and the contract/staffing model is far off-profile for this candidate.</t>
+          <t>Hard-blocked by an explicit interim SECRET clearance + Security+ certification requirement (both listed as minimum quals) that the candidate cannot meet, and the work itself is legacy contract JSP/Hibernate/WebLogic web development at a staffing firm — no overlap with distributed systems, infra, or AI platform work, at contractor-tier pay far below the $130k anchor.</t>
         </is>
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>ERP Analysts is a small Oracle Platinum Partner consulting/staffing firm; "training and placement" contract roles are typically hourly W2/C2C with no equity and minimal bonus. Band is wide because comp is unpublished and contract terms vary — estimate based on general IT-staffing/consulting entry-level market rates, not company data. Well below the candidate's ~$130k anchor.</t>
+          <t>9to9 Software Solutions is a small IT staffing/consulting body shop, and this is an explicitly Contract (not FTE) government-adjacent role — no equity, likely hourly with little or no bonus. Comparable entry-level contract Java dev rates through such firms run roughly $30-45/hr, i.e. ~$60-90k annualized. Low confidence, wide band; well below the candidate's ~$130k anchor.</t>
         </is>
       </c>
       <c r="K58" t="inlineStr">
@@ -4396,34 +4404,34 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>$35k–$50k</t>
+          <t>$60k–$85k</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Valeo Foods</t>
+          <t>9to9 Software Solutions</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Enterprise Applications Developer - Enterprise Applications</t>
+          <t>Entry Level Software Developer</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Leeds, UK</t>
+          <t>Copperhill, TN</t>
         </is>
       </c>
       <c r="G59" t="inlineStr"/>
       <c r="H59" t="inlineStr"/>
       <c r="I59" t="inlineStr">
         <is>
-          <t>UK-based (Leeds) ERP/Power Apps/SSRS enterprise-applications role in a Microsoft low-code stack at a food manufacturer — no backend/distributed-systems or AI-infra content, wrong geography for a US-authorized candidate, immediate start rather than mid-2027, and comp far below the ~$130k anchor.</t>
+          <t>Requires an existing interim SECRET clearance and Security+ certification to start (candidate has neither and lists clearance roles as a hard mismatch), and it is a contract legacy Java/JSP/WebLogic web-dev role at a staffing consultancy in rural Copperhill, TN with no distributed-systems, infra, or AI-platform content.</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>UK non-tech-sector (food manufacturing) enterprise applications developer in a regional, non-London market; junior/grad-level Microsoft ERP dev bands in Leeds run roughly £28-38k base, converting to ~$35-50k USD. Benefits listed are largely non-cash (25 days + bank holidays, matched pension, cycle-to-work, staff discount), so total cash comp is close to base. Wide-ish band because no salary was posted and the company is not a known tech-comp benchmark; this is an estimate, not fact.</t>
+          <t>Company is not well known publicly — wide, low-confidence band. 9to9 Software Solutions is a small Connecticut-based IT staffing/services consultancy rather than a product company, and this is explicitly a Contract position, implying an hourly rate with minimal-to-no equity or bonus. Cleared entry-level government-contract Java work in a low-cost rural TN market typically pays in the $60-85k equivalent range, well below the candidate's ~$130-165k anchor and under the ~$120k low-match floor.</t>
         </is>
       </c>
       <c r="K59" t="inlineStr">
@@ -4458,38 +4466,38 @@
         <v>59</v>
       </c>
       <c r="B60" s="5" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>$34k–$48k</t>
+          <t>$65k–$85k</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Valeo Foods</t>
+          <t>SOSi</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Enterprise Applications Developer - Enterprise Applications</t>
+          <t>PeopleSoft Software Developer</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Norwich, UK</t>
+          <t>Charleston, SC</t>
         </is>
       </c>
       <c r="G60" t="inlineStr"/>
       <c r="H60" t="inlineStr"/>
       <c r="I60" t="inlineStr">
         <is>
-          <t>UK-only (Norwich) internal-IT ERP/low-code role built on C#, SSRS/Power BI, Logic Apps and Power Apps — no overlap with the candidate's backend/distributed-systems/AI-infra profile, and the location is impractical for a US-authorized new grad.</t>
+          <t>Hard-blocked by the Secret clearance requirement (an explicit candidate constraint) and the work is PeopleSoft/PeopleCode ERP maintenance — no overlap with backend distributed systems, Rust/systems, or AI infra — plus onsite 5 days in Charleston at roughly half the target TC.</t>
         </is>
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>Valeo Foods is a UK food manufacturer, not a tech company; this is an internal enterprise-applications/IT position in Norwich, a low-cost regional UK market. No salary posted, so the band is inferred from typical UK junior enterprise/ERP developer pay outside London (~£27-38k) converted to USD. Wide band, low confidence; well below the candidate's ~$130k anchor.</t>
+          <t>Defense/government services integrator (SOSi) entry-level ERP developer in Charleston, SC — cleared-work government contracting pay bands are well below product-tech; base likely $65-80k with minimal bonus/equity. Wide band due to no public comp data for SOSi.</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
@@ -4528,34 +4536,34 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>$33k–$45k</t>
+          <t>$45k–$70k</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Radius Limited</t>
+          <t>ERPA</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Graduate Mobile Developer - Vehicle Telematics</t>
+          <t>Software Developer</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Crewe, UK</t>
+          <t>Franklin County, OH</t>
         </is>
       </c>
       <c r="G61" t="inlineStr"/>
       <c r="H61" t="inlineStr"/>
       <c r="I61" t="inlineStr">
         <is>
-          <t>UK-only role in Crewe with explicit no-visa-sponsorship and UK right-to-work requirement, focused on cross-platform mobile app development (Flutter/React Native/Kotlin/Swift) — off-profile on both geography/authorization and technical domain for a US-based backend/distributed-systems candidate.</t>
+          <t>Contract "training and placement" body-shop posting at an Oracle/PeopleSoft consulting partner targeting candidates with "basic technical skills" — no backend, distributed-systems, or AI-infra content, and the contract/staffing model is far off-profile for this candidate.</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>Estimate, not fact. Radius Limited is a mid-market UK fleet services/telematics company (fuel cards, leasing, telecoms), not a tech-tier compensator. Regional graduate developer salaries in Cheshire/North West England typically run roughly £26–35k GBP base with a benefits package (pension, life assurance, fuel card, EV scheme) and little to no equity; converted at ~1.27 USD/GBP that is ~$33–45k USD. Band is wide because the posting states only "competitive salary" with no figure. Note this is GBP-denominated UK comp and not directly comparable to US new-grad TC benchmarks — it sits far below the candidate's ~$130k anchor.</t>
+          <t>ERP Analysts is a small Oracle Platinum Partner consulting/staffing firm; "training and placement" contract roles are typically hourly W2/C2C with no equity and minimal bonus. Band is wide because comp is unpublished and contract terms vary — estimate based on general IT-staffing/consulting entry-level market rates, not company data. Well below the candidate's ~$130k anchor.</t>
         </is>
       </c>
       <c r="K61" t="inlineStr">
@@ -4590,38 +4598,38 @@
         <v>61</v>
       </c>
       <c r="B62" s="5" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>$44k–$56k</t>
+          <t>$35k–$50k</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>TOMRA</t>
+          <t>Valeo Foods</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Field Service Engineer - London/South East</t>
+          <t>Enterprise Applications Developer - Enterprise Applications</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>London, UK</t>
+          <t>Leeds, UK</t>
         </is>
       </c>
       <c r="G62" t="inlineStr"/>
       <c r="H62" t="inlineStr"/>
       <c r="I62" t="inlineStr">
         <is>
-          <t>Hands-on electro-mechanical field service role repairing reverse vending machines across London/South East, requiring a full UK driving licence and on-site/rota shift work — zero software engineering overlap with the candidate's backend/distributed-systems/AI-infra profile, and wrong country.</t>
+          <t>UK-based (Leeds) ERP/Power Apps/SSRS enterprise-applications role in a Microsoft low-code stack at a food manufacturer — no backend/distributed-systems or AI-infra content, wrong geography for a US-authorized candidate, immediate start rather than mid-2027, and comp far below the ~$130k anchor.</t>
         </is>
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>Posting explicitly lists GBP 35,000-41,000/year base; adding 10% non-contributory pension, company bonus, and paid overtime and converting at ~1.27 USD/GBP gives roughly $44k-$56k USD equivalent. UK field-service comp bands are not comparable to US new-grad SWE, and this sits far below the candidate's ~$130k target.</t>
+          <t>UK non-tech-sector (food manufacturing) enterprise applications developer in a regional, non-London market; junior/grad-level Microsoft ERP dev bands in Leeds run roughly £28-38k base, converting to ~$35-50k USD. Benefits listed are largely non-cash (25 days + bank holidays, matched pension, cycle-to-work, staff discount), so total cash comp is close to base. Wide-ish band because no salary was posted and the company is not a known tech-comp benchmark; this is an estimate, not fact.</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
@@ -4656,38 +4664,38 @@
         <v>62</v>
       </c>
       <c r="B63" s="5" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>$36k–$40k</t>
+          <t>$34k–$48k</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>PaperCut</t>
+          <t>Valeo Foods</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Associate Support Engineer</t>
+          <t>Enterprise Applications Developer - Enterprise Applications</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Bracknell, UK</t>
+          <t>Norwich, UK</t>
         </is>
       </c>
       <c r="G63" t="inlineStr"/>
       <c r="H63" t="inlineStr"/>
       <c r="I63" t="inlineStr">
         <is>
-          <t>Frontline customer-support role in Bracknell, UK — not a backend/distributed-systems SWE position, outside the candidate's US work authorization, and capped at ~$38k TC versus a ~$130k anchor.</t>
+          <t>UK-only (Norwich) internal-IT ERP/low-code role built on C#, SSRS/Power BI, Logic Apps and Power Apps — no overlap with the candidate's backend/distributed-systems/AI-infra profile, and the location is impractical for a US-authorized new grad.</t>
         </is>
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>Posting states "up to GBP 30,000 - yearly"; converted at ~1.27 USD/GBP. PaperCut is a mid-size private print-management vendor, and associate support roles in the UK typically have no meaningful equity component, so base is effectively total comp. Estimate, not fact.</t>
+          <t>Valeo Foods is a UK food manufacturer, not a tech company; this is an internal enterprise-applications/IT position in Norwich, a low-cost regional UK market. No salary posted, so the band is inferred from typical UK junior enterprise/ERP developer pay outside London (~£27-38k) converted to USD. Wide band, low confidence; well below the candidate's ~$130k anchor.</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
@@ -4722,42 +4730,38 @@
         <v>63</v>
       </c>
       <c r="B64" s="5" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>$20k–$45k</t>
+          <t>$33k–$45k</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Hawk-Eye Innovations</t>
+          <t>Radius Limited</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Football Tracking Systems Operator - Remote Operations Centre</t>
+          <t>Graduate Mobile Developer - Vehicle Telematics</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>Basingstoke, UK, Southampton, UK, Reading, UK</t>
+          <t>Crewe, UK</t>
         </is>
       </c>
       <c r="G64" t="inlineStr"/>
-      <c r="H64" t="inlineStr">
-        <is>
-          <t>start date: july</t>
-        </is>
-      </c>
+      <c r="H64" t="inlineStr"/>
       <c r="I64" t="inlineStr">
         <is>
-          <t>A UK-based, in-office casual hourly shift role operating live Goal Line Technology broadcast systems — not a software engineering position, wrong country, wrong start date (July/August 2026 vs. May 2027 graduation), and pay far below the candidate's floor.</t>
+          <t>UK-only role in Crewe with explicit no-visa-sponsorship and UK right-to-work requirement, focused on cross-platform mobile app development (Flutter/React Native/Kotlin/Swift) — off-profile on both geography/authorization and technical domain for a US-based backend/distributed-systems candidate.</t>
         </is>
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>Posting states £13.00–£18.20/hr on a casual contract with 10–12 hour match-day shifts. At ~$1.27/£, full-time-equivalent hours (~2,080) would be roughly $34k–48k; because hours are casual and clustered around the football calendar, realized annual earnings are likely lower, hence the wide $20k–45k band. This is not a salaried new-grad SWE offer and Hawk-Eye (Sony-owned sports tech) does not run this as a graduate engineering pipeline, so no standard new-grad TC benchmark applies. Estimate only, low confidence on total realized comp.</t>
+          <t>Estimate, not fact. Radius Limited is a mid-market UK fleet services/telematics company (fuel cards, leasing, telecoms), not a tech-tier compensator. Regional graduate developer salaries in Cheshire/North West England typically run roughly £26–35k GBP base with a benefits package (pension, life assurance, fuel card, EV scheme) and little to no equity; converted at ~1.27 USD/GBP that is ~$33–45k USD. Band is wide because the posting states only "competitive salary" with no figure. Note this is GBP-denominated UK comp and not directly comparable to US new-grad TC benchmarks — it sits far below the candidate's ~$130k anchor.</t>
         </is>
       </c>
       <c r="K64" t="inlineStr">
@@ -4796,34 +4800,34 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>$15k–$45k</t>
+          <t>$44k–$56k</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Lilt</t>
+          <t>TOMRA</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>AI Training Contributor - French</t>
+          <t>Field Service Engineer - London/South East</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Remote in Canada, Québec City, QC, Canada</t>
+          <t>London, UK</t>
         </is>
       </c>
       <c r="G65" t="inlineStr"/>
       <c r="H65" t="inlineStr"/>
       <c r="I65" t="inlineStr">
         <is>
-          <t>This is a part-time 1099 data-annotation/linguist gig in Canada requiring native French fluency — no software engineering content, no US full-time new-grad path, and nothing touching the candidate's backend/distributed-systems/AI-infra profile.</t>
+          <t>Hands-on electro-mechanical field service role repairing reverse vending machines across London/South East, requiring a full UK driving licence and on-site/rota shift work — zero software engineering overlap with the candidate's backend/distributed-systems/AI-infra profile, and wrong country.</t>
         </is>
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>Not a salaried role — Lilt pays AI-training contractors hourly/per-task (typically ~$15-30/hr USD equivalent) with no benefits and no guaranteed hours; the posting explicitly says it is unsuitable as primary income. Band shown is a rough annualized figure assuming the stated 10+ hrs/week minimum up to near-full-time utilization, and is highly uncertain. Far below the ~$130k anchor.</t>
+          <t>Posting explicitly lists GBP 35,000-41,000/year base; adding 10% non-contributory pension, company bonus, and paid overtime and converting at ~1.27 USD/GBP gives roughly $44k-$56k USD equivalent. UK field-service comp bands are not comparable to US new-grad SWE, and this sits far below the candidate's ~$130k target.</t>
         </is>
       </c>
       <c r="K65" t="inlineStr">
@@ -4848,6 +4852,208 @@
         </is>
       </c>
       <c r="P65" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="n">
+        <v>65</v>
+      </c>
+      <c r="B66" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>$36k–$40k</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>PaperCut</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Associate Support Engineer</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>Bracknell, UK</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr"/>
+      <c r="H66" t="inlineStr"/>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>Frontline customer-support role in Bracknell, UK — not a backend/distributed-systems SWE position, outside the candidate's US work authorization, and capped at ~$38k TC versus a ~$130k anchor.</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>Posting states "up to GBP 30,000 - yearly"; converted at ~1.27 USD/GBP. PaperCut is a mid-size private print-management vendor, and associate support roles in the UK typically have no meaningful equity component, so base is effectively total comp. Estimate, not fact.</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>scored</t>
+        </is>
+      </c>
+      <c r="M66" s="3" t="inlineStr">
+        <is>
+          <t>Apply ↗</t>
+        </is>
+      </c>
+      <c r="N66" t="inlineStr"/>
+      <c r="O66" s="3" t="inlineStr">
+        <is>
+          <t>levels.fyi ↗</t>
+        </is>
+      </c>
+      <c r="P66" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="n">
+        <v>66</v>
+      </c>
+      <c r="B67" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>$20k–$45k</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Hawk-Eye Innovations</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Football Tracking Systems Operator - Remote Operations Centre</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>Basingstoke, UK, Southampton, UK, Reading, UK</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr"/>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>start date: july</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>A UK-based, in-office casual hourly shift role operating live Goal Line Technology broadcast systems — not a software engineering position, wrong country, wrong start date (July/August 2026 vs. May 2027 graduation), and pay far below the candidate's floor.</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>Posting states £13.00–£18.20/hr on a casual contract with 10–12 hour match-day shifts. At ~$1.27/£, full-time-equivalent hours (~2,080) would be roughly $34k–48k; because hours are casual and clustered around the football calendar, realized annual earnings are likely lower, hence the wide $20k–45k band. This is not a salaried new-grad SWE offer and Hawk-Eye (Sony-owned sports tech) does not run this as a graduate engineering pipeline, so no standard new-grad TC benchmark applies. Estimate only, low confidence on total realized comp.</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>scored</t>
+        </is>
+      </c>
+      <c r="M67" s="3" t="inlineStr">
+        <is>
+          <t>Apply ↗</t>
+        </is>
+      </c>
+      <c r="N67" t="inlineStr"/>
+      <c r="O67" s="3" t="inlineStr">
+        <is>
+          <t>levels.fyi ↗</t>
+        </is>
+      </c>
+      <c r="P67" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="n">
+        <v>67</v>
+      </c>
+      <c r="B68" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>$15k–$45k</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Lilt</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>AI Training Contributor - French</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>Remote in Canada, Québec City, QC, Canada</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr"/>
+      <c r="H68" t="inlineStr"/>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>This is a part-time 1099 data-annotation/linguist gig in Canada requiring native French fluency — no software engineering content, no US full-time new-grad path, and nothing touching the candidate's backend/distributed-systems/AI-infra profile.</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>Not a salaried role — Lilt pays AI-training contractors hourly/per-task (typically ~$15-30/hr USD equivalent) with no benefits and no guaranteed hours; the posting explicitly says it is unsuitable as primary income. Band shown is a rough annualized figure assuming the stated 10+ hrs/week minimum up to near-full-time utilization, and is highly uncertain. Far below the ~$130k anchor.</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>scored</t>
+        </is>
+      </c>
+      <c r="M68" s="3" t="inlineStr">
+        <is>
+          <t>Apply ↗</t>
+        </is>
+      </c>
+      <c r="N68" t="inlineStr"/>
+      <c r="O68" s="3" t="inlineStr">
+        <is>
+          <t>levels.fyi ↗</t>
+        </is>
+      </c>
+      <c r="P68" t="inlineStr">
         <is>
           <t>2026-08-12</t>
         </is>
@@ -4883,122 +5089,131 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N11" r:id="rId26"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId27"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M12" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M13" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N13" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N12" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M13" r:id="rId31"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId32"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M14" r:id="rId33"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N14" r:id="rId34"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O14" r:id="rId35"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M15" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O15" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M16" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N16" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N15" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O15" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M16" r:id="rId39"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O16" r:id="rId40"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M17" r:id="rId41"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N17" r:id="rId42"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O17" r:id="rId43"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M18" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O18" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M19" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N19" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N18" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O18" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M19" r:id="rId47"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O19" r:id="rId48"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M20" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O20" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M21" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O21" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M22" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O22" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M23" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N23" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N20" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O20" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M21" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O21" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M22" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O22" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M23" r:id="rId56"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O23" r:id="rId57"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M24" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O24" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M25" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O25" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M26" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O26" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M27" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N27" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O27" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M28" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O28" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M29" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N29" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O29" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M30" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N30" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N24" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O24" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M25" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N25" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O25" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M26" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O26" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M27" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O27" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M28" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O28" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M29" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N29" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O29" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M30" r:id="rId73"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O30" r:id="rId74"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M31" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O31" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M32" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O32" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M33" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O33" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M34" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O34" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M35" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O35" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M36" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O36" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M37" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M38" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O38" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M39" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O39" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M40" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O40" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M41" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O41" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M42" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O42" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M43" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O43" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M44" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O44" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M45" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O45" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M46" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O46" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M47" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O47" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M48" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O48" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M49" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O49" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M50" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O50" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M51" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O51" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M52" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O52" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M53" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O53" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M54" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O54" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M55" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O55" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M56" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O56" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M57" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O57" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M58" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O58" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M59" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O59" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M60" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O60" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M61" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O61" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M62" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O62" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M63" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O63" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M64" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O64" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M65" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O65" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N31" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O31" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M32" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N32" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O32" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M33" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N33" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O33" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M34" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O34" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M35" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O35" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M36" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O36" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M37" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M38" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O38" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M39" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O39" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M40" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O40" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M41" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O41" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M42" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O42" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M43" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O43" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M44" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O44" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M45" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O45" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M46" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O46" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M47" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O47" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M48" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O48" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M49" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O49" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M50" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O50" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M51" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O51" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M52" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O52" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M53" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O53" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M54" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O54" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M55" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O55" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M56" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O56" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M57" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O57" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M58" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O58" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M59" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O59" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M60" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O60" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M61" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O61" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M62" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O62" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M63" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O63" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M64" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O64" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M65" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O65" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M66" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O66" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M67" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O67" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M68" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O68" r:id="rId153"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Ad-hoc: tailored 3 job(s) via tailor_selected.py
</commit_message>
<xml_diff>
--- a/output/tailored_resumes.xlsx
+++ b/output/tailored_resumes.xlsx
@@ -2721,7 +2721,7 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>scored</t>
+          <t>tailored</t>
         </is>
       </c>
       <c r="M33" s="3" t="inlineStr">
@@ -2729,7 +2729,11 @@
           <t>Apply ↗</t>
         </is>
       </c>
-      <c r="N33" t="inlineStr"/>
+      <c r="N33" s="3" t="inlineStr">
+        <is>
+          <t>Composio_Forward_Deployed_Engineer_New_Grad_55c35f.pdf</t>
+        </is>
+      </c>
       <c r="O33" s="3" t="inlineStr">
         <is>
           <t>levels.fyi ↗</t>
@@ -4497,7 +4501,7 @@
       </c>
       <c r="L59" t="inlineStr">
         <is>
-          <t>scored</t>
+          <t>tailored</t>
         </is>
       </c>
       <c r="M59" s="3" t="inlineStr">
@@ -4505,7 +4509,11 @@
           <t>Apply ↗</t>
         </is>
       </c>
-      <c r="N59" t="inlineStr"/>
+      <c r="N59" s="3" t="inlineStr">
+        <is>
+          <t>LiteLLM_Forward_Deployed_Engineer_New_Grad_609cc8.pdf</t>
+        </is>
+      </c>
       <c r="O59" s="3" t="inlineStr">
         <is>
           <t>levels.fyi ↗</t>
@@ -5573,7 +5581,7 @@
       </c>
       <c r="L75" t="inlineStr">
         <is>
-          <t>scored</t>
+          <t>tailored</t>
         </is>
       </c>
       <c r="M75" s="3" t="inlineStr">
@@ -5581,7 +5589,11 @@
           <t>Apply ↗</t>
         </is>
       </c>
-      <c r="N75" t="inlineStr"/>
+      <c r="N75" s="3" t="inlineStr">
+        <is>
+          <t>Applied_Intuition_Software_Integration_Engineer_Ne_72fe15.pdf</t>
+        </is>
+      </c>
       <c r="O75" s="3" t="inlineStr">
         <is>
           <t>levels.fyi ↗</t>
@@ -23075,631 +23087,634 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M32" r:id="rId72"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O32" r:id="rId73"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M33" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O33" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M34" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O34" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M35" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O35" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M36" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N36" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O36" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M37" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N37" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M38" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O38" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M39" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O39" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M40" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N40" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O40" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M41" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N41" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O41" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M42" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N42" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O42" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M43" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O43" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M44" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O44" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M45" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O45" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M46" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N46" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O46" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M47" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O47" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M48" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O48" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M49" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N49" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O49" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M50" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O50" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M51" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O51" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M52" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O52" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M53" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O53" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M54" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N54" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O54" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M55" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O55" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M56" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N56" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O56" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M57" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N57" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O57" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M58" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O58" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M59" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O59" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M60" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O60" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M61" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O61" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M62" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O62" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M63" r:id="rId144"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O63" r:id="rId145"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M64" r:id="rId146"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O64" r:id="rId147"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M65" r:id="rId148"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O65" r:id="rId149"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M66" r:id="rId150"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O66" r:id="rId151"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M67" r:id="rId152"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N67" r:id="rId153"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O67" r:id="rId154"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M68" r:id="rId155"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O68" r:id="rId156"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M69" r:id="rId157"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O69" r:id="rId158"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M70" r:id="rId159"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O70" r:id="rId160"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M71" r:id="rId161"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O71" r:id="rId162"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M72" r:id="rId163"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O72" r:id="rId164"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M73" r:id="rId165"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O73" r:id="rId166"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M74" r:id="rId167"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O74" r:id="rId168"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M75" r:id="rId169"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O75" r:id="rId170"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M76" r:id="rId171"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="rId172"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M77" r:id="rId173"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O77" r:id="rId174"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M78" r:id="rId175"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O78" r:id="rId176"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M79" r:id="rId177"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N79" r:id="rId178"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O79" r:id="rId179"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M80" r:id="rId180"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O80" r:id="rId181"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M81" r:id="rId182"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O81" r:id="rId183"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M82" r:id="rId184"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O82" r:id="rId185"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M83" r:id="rId186"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N83" r:id="rId187"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O83" r:id="rId188"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M84" r:id="rId189"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O84" r:id="rId190"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M85" r:id="rId191"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O85" r:id="rId192"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M86" r:id="rId193"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O86" r:id="rId194"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M87" r:id="rId195"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O87" r:id="rId196"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M88" r:id="rId197"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O88" r:id="rId198"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M89" r:id="rId199"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O89" r:id="rId200"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M90" r:id="rId201"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O90" r:id="rId202"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M91" r:id="rId203"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O91" r:id="rId204"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M92" r:id="rId205"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O92" r:id="rId206"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M93" r:id="rId207"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O93" r:id="rId208"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M94" r:id="rId209"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O94" r:id="rId210"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M95" r:id="rId211"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O95" r:id="rId212"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M96" r:id="rId213"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O96" r:id="rId214"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M97" r:id="rId215"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O97" r:id="rId216"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M98" r:id="rId217"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O98" r:id="rId218"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M99" r:id="rId219"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O99" r:id="rId220"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M100" r:id="rId221"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N100" r:id="rId222"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O100" r:id="rId223"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M101" r:id="rId224"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O101" r:id="rId225"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M102" r:id="rId226"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O102" r:id="rId227"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M103" r:id="rId228"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O103" r:id="rId229"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M104" r:id="rId230"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O104" r:id="rId231"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M105" r:id="rId232"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O105" r:id="rId233"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M106" r:id="rId234"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N106" r:id="rId235"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O106" r:id="rId236"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M107" r:id="rId237"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O107" r:id="rId238"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M108" r:id="rId239"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O108" r:id="rId240"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M109" r:id="rId241"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N109" r:id="rId242"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O109" r:id="rId243"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M110" r:id="rId244"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N110" r:id="rId245"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O110" r:id="rId246"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M111" r:id="rId247"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O111" r:id="rId248"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M112" r:id="rId249"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O112" r:id="rId250"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M113" r:id="rId251"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O113" r:id="rId252"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M114" r:id="rId253"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O114" r:id="rId254"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M115" r:id="rId255"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O115" r:id="rId256"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M116" r:id="rId257"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O116" r:id="rId258"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M117" r:id="rId259"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O117" r:id="rId260"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M118" r:id="rId261"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O118" r:id="rId262"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M119" r:id="rId263"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O119" r:id="rId264"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M120" r:id="rId265"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O120" r:id="rId266"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M121" r:id="rId267"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O121" r:id="rId268"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M122" r:id="rId269"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O122" r:id="rId270"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M123" r:id="rId271"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O123" r:id="rId272"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M124" r:id="rId273"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O124" r:id="rId274"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M125" r:id="rId275"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O125" r:id="rId276"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M126" r:id="rId277"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O126" r:id="rId278"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M127" r:id="rId279"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O127" r:id="rId280"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M128" r:id="rId281"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O128" r:id="rId282"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M129" r:id="rId283"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O129" r:id="rId284"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M130" r:id="rId285"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O130" r:id="rId286"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M131" r:id="rId287"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O131" r:id="rId288"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M132" r:id="rId289"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O132" r:id="rId290"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M133" r:id="rId291"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O133" r:id="rId292"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M134" r:id="rId293"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O134" r:id="rId294"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M135" r:id="rId295"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O135" r:id="rId296"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M136" r:id="rId297"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O136" r:id="rId298"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M137" r:id="rId299"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O137" r:id="rId300"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M138" r:id="rId301"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O138" r:id="rId302"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M139" r:id="rId303"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O139" r:id="rId304"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M140" r:id="rId305"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O140" r:id="rId306"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M141" r:id="rId307"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O141" r:id="rId308"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M142" r:id="rId309"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O142" r:id="rId310"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M143" r:id="rId311"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O143" r:id="rId312"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M144" r:id="rId313"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O144" r:id="rId314"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M145" r:id="rId315"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O145" r:id="rId316"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M146" r:id="rId317"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O146" r:id="rId318"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M147" r:id="rId319"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O147" r:id="rId320"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M148" r:id="rId321"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O148" r:id="rId322"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M149" r:id="rId323"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O149" r:id="rId324"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M150" r:id="rId325"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O150" r:id="rId326"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M151" r:id="rId327"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O151" r:id="rId328"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M152" r:id="rId329"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O152" r:id="rId330"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M153" r:id="rId331"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O153" r:id="rId332"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M154" r:id="rId333"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O154" r:id="rId334"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M155" r:id="rId335"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O155" r:id="rId336"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M156" r:id="rId337"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O156" r:id="rId338"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M157" r:id="rId339"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O157" r:id="rId340"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M158" r:id="rId341"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O158" r:id="rId342"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M159" r:id="rId343"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O159" r:id="rId344"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M160" r:id="rId345"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O160" r:id="rId346"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M161" r:id="rId347"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N161" r:id="rId348"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O161" r:id="rId349"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M162" r:id="rId350"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O162" r:id="rId351"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M163" r:id="rId352"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O163" r:id="rId353"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M164" r:id="rId354"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O164" r:id="rId355"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M165" r:id="rId356"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O165" r:id="rId357"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M166" r:id="rId358"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O166" r:id="rId359"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M167" r:id="rId360"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O167" r:id="rId361"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M168" r:id="rId362"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O168" r:id="rId363"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M169" r:id="rId364"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O169" r:id="rId365"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M170" r:id="rId366"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O170" r:id="rId367"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M171" r:id="rId368"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O171" r:id="rId369"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M172" r:id="rId370"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O172" r:id="rId371"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M173" r:id="rId372"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O173" r:id="rId373"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M174" r:id="rId374"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O174" r:id="rId375"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M175" r:id="rId376"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O175" r:id="rId377"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M176" r:id="rId378"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O176" r:id="rId379"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M177" r:id="rId380"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O177" r:id="rId381"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M178" r:id="rId382"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O178" r:id="rId383"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M179" r:id="rId384"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O179" r:id="rId385"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M180" r:id="rId386"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O180" r:id="rId387"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M181" r:id="rId388"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O181" r:id="rId389"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M182" r:id="rId390"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O182" r:id="rId391"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M183" r:id="rId392"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O183" r:id="rId393"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M184" r:id="rId394"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O184" r:id="rId395"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M185" r:id="rId396"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O185" r:id="rId397"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M186" r:id="rId398"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O186" r:id="rId399"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M187" r:id="rId400"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O187" r:id="rId401"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M188" r:id="rId402"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O188" r:id="rId403"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M189" r:id="rId404"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O189" r:id="rId405"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M190" r:id="rId406"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O190" r:id="rId407"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M191" r:id="rId408"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O191" r:id="rId409"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M192" r:id="rId410"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O192" r:id="rId411"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M193" r:id="rId412"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O193" r:id="rId413"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M194" r:id="rId414"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O194" r:id="rId415"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M195" r:id="rId416"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O195" r:id="rId417"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M196" r:id="rId418"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O196" r:id="rId419"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M197" r:id="rId420"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O197" r:id="rId421"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M198" r:id="rId422"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O198" r:id="rId423"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M199" r:id="rId424"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O199" r:id="rId425"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M200" r:id="rId426"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O200" r:id="rId427"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M201" r:id="rId428"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O201" r:id="rId429"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M202" r:id="rId430"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O202" r:id="rId431"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M203" r:id="rId432"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O203" r:id="rId433"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M204" r:id="rId434"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O204" r:id="rId435"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M205" r:id="rId436"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O205" r:id="rId437"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M206" r:id="rId438"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O206" r:id="rId439"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M207" r:id="rId440"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O207" r:id="rId441"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M208" r:id="rId442"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O208" r:id="rId443"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M209" r:id="rId444"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O209" r:id="rId445"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M210" r:id="rId446"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O210" r:id="rId447"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M211" r:id="rId448"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O211" r:id="rId449"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M212" r:id="rId450"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O212" r:id="rId451"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M213" r:id="rId452"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O213" r:id="rId453"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M214" r:id="rId454"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O214" r:id="rId455"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M215" r:id="rId456"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O215" r:id="rId457"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M216" r:id="rId458"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O216" r:id="rId459"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M217" r:id="rId460"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O217" r:id="rId461"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M218" r:id="rId462"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O218" r:id="rId463"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M219" r:id="rId464"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O219" r:id="rId465"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M220" r:id="rId466"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O220" r:id="rId467"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M221" r:id="rId468"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O221" r:id="rId469"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M222" r:id="rId470"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O222" r:id="rId471"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M223" r:id="rId472"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O223" r:id="rId473"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M224" r:id="rId474"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O224" r:id="rId475"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M225" r:id="rId476"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O225" r:id="rId477"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M226" r:id="rId478"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O226" r:id="rId479"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M227" r:id="rId480"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O227" r:id="rId481"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M228" r:id="rId482"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O228" r:id="rId483"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M229" r:id="rId484"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O229" r:id="rId485"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M230" r:id="rId486"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O230" r:id="rId487"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M231" r:id="rId488"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O231" r:id="rId489"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M232" r:id="rId490"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O232" r:id="rId491"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M233" r:id="rId492"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O233" r:id="rId493"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M234" r:id="rId494"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O234" r:id="rId495"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M235" r:id="rId496"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O235" r:id="rId497"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M236" r:id="rId498"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O236" r:id="rId499"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M237" r:id="rId500"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O237" r:id="rId501"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M238" r:id="rId502"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O238" r:id="rId503"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M239" r:id="rId504"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O239" r:id="rId505"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M240" r:id="rId506"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O240" r:id="rId507"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M241" r:id="rId508"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O241" r:id="rId509"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M242" r:id="rId510"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O242" r:id="rId511"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M243" r:id="rId512"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O243" r:id="rId513"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M244" r:id="rId514"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O244" r:id="rId515"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M245" r:id="rId516"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O245" r:id="rId517"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M246" r:id="rId518"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O246" r:id="rId519"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M247" r:id="rId520"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O247" r:id="rId521"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M248" r:id="rId522"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O248" r:id="rId523"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M249" r:id="rId524"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O249" r:id="rId525"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M250" r:id="rId526"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O250" r:id="rId527"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M251" r:id="rId528"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O251" r:id="rId529"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M252" r:id="rId530"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O252" r:id="rId531"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M253" r:id="rId532"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O253" r:id="rId533"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M254" r:id="rId534"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O254" r:id="rId535"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M255" r:id="rId536"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O255" r:id="rId537"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M256" r:id="rId538"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O256" r:id="rId539"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M257" r:id="rId540"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O257" r:id="rId541"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M258" r:id="rId542"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O258" r:id="rId543"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M259" r:id="rId544"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O259" r:id="rId545"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M260" r:id="rId546"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O260" r:id="rId547"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M261" r:id="rId548"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O261" r:id="rId549"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M262" r:id="rId550"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O262" r:id="rId551"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M263" r:id="rId552"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O263" r:id="rId553"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M264" r:id="rId554"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O264" r:id="rId555"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M265" r:id="rId556"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O265" r:id="rId557"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M266" r:id="rId558"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O266" r:id="rId559"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M267" r:id="rId560"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O267" r:id="rId561"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M268" r:id="rId562"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O268" r:id="rId563"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M269" r:id="rId564"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O269" r:id="rId565"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M270" r:id="rId566"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O270" r:id="rId567"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M271" r:id="rId568"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O271" r:id="rId569"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M272" r:id="rId570"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O272" r:id="rId571"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M273" r:id="rId572"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O273" r:id="rId573"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M274" r:id="rId574"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O274" r:id="rId575"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M275" r:id="rId576"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O275" r:id="rId577"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M276" r:id="rId578"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O276" r:id="rId579"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M277" r:id="rId580"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O277" r:id="rId581"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M278" r:id="rId582"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O278" r:id="rId583"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M279" r:id="rId584"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O279" r:id="rId585"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M280" r:id="rId586"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O280" r:id="rId587"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M281" r:id="rId588"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O281" r:id="rId589"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M282" r:id="rId590"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O282" r:id="rId591"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M283" r:id="rId592"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O283" r:id="rId593"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M284" r:id="rId594"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O284" r:id="rId595"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M285" r:id="rId596"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O285" r:id="rId597"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M286" r:id="rId598"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O286" r:id="rId599"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M287" r:id="rId600"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O287" r:id="rId601"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M288" r:id="rId602"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O288" r:id="rId603"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M289" r:id="rId604"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O289" r:id="rId605"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M290" r:id="rId606"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O290" r:id="rId607"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M291" r:id="rId608"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O291" r:id="rId609"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M292" r:id="rId610"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O292" r:id="rId611"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M293" r:id="rId612"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O293" r:id="rId613"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M294" r:id="rId614"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O294" r:id="rId615"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M295" r:id="rId616"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O295" r:id="rId617"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M296" r:id="rId618"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O296" r:id="rId619"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M297" r:id="rId620"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O297" r:id="rId621"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M298" r:id="rId622"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O298" r:id="rId623"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M299" r:id="rId624"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O299" r:id="rId625"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M300" r:id="rId626"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O300" r:id="rId627"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M301" r:id="rId628"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O301" r:id="rId629"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M302" r:id="rId630"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O302" r:id="rId631"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M303" r:id="rId632"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O303" r:id="rId633"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M304" r:id="rId634"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O304" r:id="rId635"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M305" r:id="rId636"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O305" r:id="rId637"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M306" r:id="rId638"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O306" r:id="rId639"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M307" r:id="rId640"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O307" r:id="rId641"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M308" r:id="rId642"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O308" r:id="rId643"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M309" r:id="rId644"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O309" r:id="rId645"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M310" r:id="rId646"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O310" r:id="rId647"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M311" r:id="rId648"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O311" r:id="rId649"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M312" r:id="rId650"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O312" r:id="rId651"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M313" r:id="rId652"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O313" r:id="rId653"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M314" r:id="rId654"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O314" r:id="rId655"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M315" r:id="rId656"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O315" r:id="rId657"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M316" r:id="rId658"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O316" r:id="rId659"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M317" r:id="rId660"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O317" r:id="rId661"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M318" r:id="rId662"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O318" r:id="rId663"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M319" r:id="rId664"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O319" r:id="rId665"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M320" r:id="rId666"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O320" r:id="rId667"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M321" r:id="rId668"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O321" r:id="rId669"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M322" r:id="rId670"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O322" r:id="rId671"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M323" r:id="rId672"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O323" r:id="rId673"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M324" r:id="rId674"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O324" r:id="rId675"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M325" r:id="rId676"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O325" r:id="rId677"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M326" r:id="rId678"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O326" r:id="rId679"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M327" r:id="rId680"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O327" r:id="rId681"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M328" r:id="rId682"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O328" r:id="rId683"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M329" r:id="rId684"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O329" r:id="rId685"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M330" r:id="rId686"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O330" r:id="rId687"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M331" r:id="rId688"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O331" r:id="rId689"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M332" r:id="rId690"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O332" r:id="rId691"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M333" r:id="rId692"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O333" r:id="rId693"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M334" r:id="rId694"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O334" r:id="rId695"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M335" r:id="rId696"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O335" r:id="rId697"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M336" r:id="rId698"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O336" r:id="rId699"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N33" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O33" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M34" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O34" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M35" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O35" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M36" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N36" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O36" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M37" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N37" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M38" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O38" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M39" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O39" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M40" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N40" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O40" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M41" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N41" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O41" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M42" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N42" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O42" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M43" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O43" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M44" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O44" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M45" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O45" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M46" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N46" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O46" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M47" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O47" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M48" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O48" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M49" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N49" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O49" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M50" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O50" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M51" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O51" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M52" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O52" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M53" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O53" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M54" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N54" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O54" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M55" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O55" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M56" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N56" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O56" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M57" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N57" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O57" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M58" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O58" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M59" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N59" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O59" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M60" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O60" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M61" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O61" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M62" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O62" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M63" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O63" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M64" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O64" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M65" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O65" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M66" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O66" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M67" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N67" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O67" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M68" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O68" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M69" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O69" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M70" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O70" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M71" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O71" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M72" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O72" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M73" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O73" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M74" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O74" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M75" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N75" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O75" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M76" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M77" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O77" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M78" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O78" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M79" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N79" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O79" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M80" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O80" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M81" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O81" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M82" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O82" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M83" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N83" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O83" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M84" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O84" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M85" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O85" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M86" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O86" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M87" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O87" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M88" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O88" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M89" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O89" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M90" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O90" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M91" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O91" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M92" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O92" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M93" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O93" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M94" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O94" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M95" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O95" r:id="rId215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M96" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O96" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M97" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O97" r:id="rId219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M98" r:id="rId220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O98" r:id="rId221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M99" r:id="rId222"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O99" r:id="rId223"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M100" r:id="rId224"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N100" r:id="rId225"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O100" r:id="rId226"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M101" r:id="rId227"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O101" r:id="rId228"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M102" r:id="rId229"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O102" r:id="rId230"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M103" r:id="rId231"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O103" r:id="rId232"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M104" r:id="rId233"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O104" r:id="rId234"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M105" r:id="rId235"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O105" r:id="rId236"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M106" r:id="rId237"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N106" r:id="rId238"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O106" r:id="rId239"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M107" r:id="rId240"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O107" r:id="rId241"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M108" r:id="rId242"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O108" r:id="rId243"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M109" r:id="rId244"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N109" r:id="rId245"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O109" r:id="rId246"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M110" r:id="rId247"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N110" r:id="rId248"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O110" r:id="rId249"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M111" r:id="rId250"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O111" r:id="rId251"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M112" r:id="rId252"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O112" r:id="rId253"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M113" r:id="rId254"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O113" r:id="rId255"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M114" r:id="rId256"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O114" r:id="rId257"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M115" r:id="rId258"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O115" r:id="rId259"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M116" r:id="rId260"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O116" r:id="rId261"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M117" r:id="rId262"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O117" r:id="rId263"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M118" r:id="rId264"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O118" r:id="rId265"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M119" r:id="rId266"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O119" r:id="rId267"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M120" r:id="rId268"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O120" r:id="rId269"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M121" r:id="rId270"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O121" r:id="rId271"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M122" r:id="rId272"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O122" r:id="rId273"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M123" r:id="rId274"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O123" r:id="rId275"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M124" r:id="rId276"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O124" r:id="rId277"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M125" r:id="rId278"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O125" r:id="rId279"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M126" r:id="rId280"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O126" r:id="rId281"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M127" r:id="rId282"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O127" r:id="rId283"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M128" r:id="rId284"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O128" r:id="rId285"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M129" r:id="rId286"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O129" r:id="rId287"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M130" r:id="rId288"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O130" r:id="rId289"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M131" r:id="rId290"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O131" r:id="rId291"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M132" r:id="rId292"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O132" r:id="rId293"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M133" r:id="rId294"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O133" r:id="rId295"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M134" r:id="rId296"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O134" r:id="rId297"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M135" r:id="rId298"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O135" r:id="rId299"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M136" r:id="rId300"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O136" r:id="rId301"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M137" r:id="rId302"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O137" r:id="rId303"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M138" r:id="rId304"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O138" r:id="rId305"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M139" r:id="rId306"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O139" r:id="rId307"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M140" r:id="rId308"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O140" r:id="rId309"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M141" r:id="rId310"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O141" r:id="rId311"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M142" r:id="rId312"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O142" r:id="rId313"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M143" r:id="rId314"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O143" r:id="rId315"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M144" r:id="rId316"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O144" r:id="rId317"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M145" r:id="rId318"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O145" r:id="rId319"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M146" r:id="rId320"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O146" r:id="rId321"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M147" r:id="rId322"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O147" r:id="rId323"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M148" r:id="rId324"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O148" r:id="rId325"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M149" r:id="rId326"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O149" r:id="rId327"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M150" r:id="rId328"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O150" r:id="rId329"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M151" r:id="rId330"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O151" r:id="rId331"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M152" r:id="rId332"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O152" r:id="rId333"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M153" r:id="rId334"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O153" r:id="rId335"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M154" r:id="rId336"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O154" r:id="rId337"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M155" r:id="rId338"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O155" r:id="rId339"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M156" r:id="rId340"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O156" r:id="rId341"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M157" r:id="rId342"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O157" r:id="rId343"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M158" r:id="rId344"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O158" r:id="rId345"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M159" r:id="rId346"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O159" r:id="rId347"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M160" r:id="rId348"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O160" r:id="rId349"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M161" r:id="rId350"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N161" r:id="rId351"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O161" r:id="rId352"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M162" r:id="rId353"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O162" r:id="rId354"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M163" r:id="rId355"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O163" r:id="rId356"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M164" r:id="rId357"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O164" r:id="rId358"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M165" r:id="rId359"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O165" r:id="rId360"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M166" r:id="rId361"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O166" r:id="rId362"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M167" r:id="rId363"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O167" r:id="rId364"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M168" r:id="rId365"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O168" r:id="rId366"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M169" r:id="rId367"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O169" r:id="rId368"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M170" r:id="rId369"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O170" r:id="rId370"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M171" r:id="rId371"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O171" r:id="rId372"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M172" r:id="rId373"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O172" r:id="rId374"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M173" r:id="rId375"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O173" r:id="rId376"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M174" r:id="rId377"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O174" r:id="rId378"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M175" r:id="rId379"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O175" r:id="rId380"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M176" r:id="rId381"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O176" r:id="rId382"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M177" r:id="rId383"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O177" r:id="rId384"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M178" r:id="rId385"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O178" r:id="rId386"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M179" r:id="rId387"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O179" r:id="rId388"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M180" r:id="rId389"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O180" r:id="rId390"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M181" r:id="rId391"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O181" r:id="rId392"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M182" r:id="rId393"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O182" r:id="rId394"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M183" r:id="rId395"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O183" r:id="rId396"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M184" r:id="rId397"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O184" r:id="rId398"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M185" r:id="rId399"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O185" r:id="rId400"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M186" r:id="rId401"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O186" r:id="rId402"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M187" r:id="rId403"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O187" r:id="rId404"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M188" r:id="rId405"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O188" r:id="rId406"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M189" r:id="rId407"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O189" r:id="rId408"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M190" r:id="rId409"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O190" r:id="rId410"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M191" r:id="rId411"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O191" r:id="rId412"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M192" r:id="rId413"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O192" r:id="rId414"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M193" r:id="rId415"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O193" r:id="rId416"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M194" r:id="rId417"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O194" r:id="rId418"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M195" r:id="rId419"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O195" r:id="rId420"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M196" r:id="rId421"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O196" r:id="rId422"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M197" r:id="rId423"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O197" r:id="rId424"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M198" r:id="rId425"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O198" r:id="rId426"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M199" r:id="rId427"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O199" r:id="rId428"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M200" r:id="rId429"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O200" r:id="rId430"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M201" r:id="rId431"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O201" r:id="rId432"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M202" r:id="rId433"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O202" r:id="rId434"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M203" r:id="rId435"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O203" r:id="rId436"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M204" r:id="rId437"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O204" r:id="rId438"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M205" r:id="rId439"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O205" r:id="rId440"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M206" r:id="rId441"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O206" r:id="rId442"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M207" r:id="rId443"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O207" r:id="rId444"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M208" r:id="rId445"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O208" r:id="rId446"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M209" r:id="rId447"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O209" r:id="rId448"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M210" r:id="rId449"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O210" r:id="rId450"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M211" r:id="rId451"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O211" r:id="rId452"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M212" r:id="rId453"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O212" r:id="rId454"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M213" r:id="rId455"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O213" r:id="rId456"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M214" r:id="rId457"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O214" r:id="rId458"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M215" r:id="rId459"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O215" r:id="rId460"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M216" r:id="rId461"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O216" r:id="rId462"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M217" r:id="rId463"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O217" r:id="rId464"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M218" r:id="rId465"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O218" r:id="rId466"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M219" r:id="rId467"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O219" r:id="rId468"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M220" r:id="rId469"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O220" r:id="rId470"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M221" r:id="rId471"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O221" r:id="rId472"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M222" r:id="rId473"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O222" r:id="rId474"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M223" r:id="rId475"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O223" r:id="rId476"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M224" r:id="rId477"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O224" r:id="rId478"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M225" r:id="rId479"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O225" r:id="rId480"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M226" r:id="rId481"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O226" r:id="rId482"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M227" r:id="rId483"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O227" r:id="rId484"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M228" r:id="rId485"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O228" r:id="rId486"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M229" r:id="rId487"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O229" r:id="rId488"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M230" r:id="rId489"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O230" r:id="rId490"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M231" r:id="rId491"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O231" r:id="rId492"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M232" r:id="rId493"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O232" r:id="rId494"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M233" r:id="rId495"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O233" r:id="rId496"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M234" r:id="rId497"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O234" r:id="rId498"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M235" r:id="rId499"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O235" r:id="rId500"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M236" r:id="rId501"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O236" r:id="rId502"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M237" r:id="rId503"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O237" r:id="rId504"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M238" r:id="rId505"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O238" r:id="rId506"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M239" r:id="rId507"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O239" r:id="rId508"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M240" r:id="rId509"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O240" r:id="rId510"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M241" r:id="rId511"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O241" r:id="rId512"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M242" r:id="rId513"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O242" r:id="rId514"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M243" r:id="rId515"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O243" r:id="rId516"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M244" r:id="rId517"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O244" r:id="rId518"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M245" r:id="rId519"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O245" r:id="rId520"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M246" r:id="rId521"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O246" r:id="rId522"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M247" r:id="rId523"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O247" r:id="rId524"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M248" r:id="rId525"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O248" r:id="rId526"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M249" r:id="rId527"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O249" r:id="rId528"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M250" r:id="rId529"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O250" r:id="rId530"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M251" r:id="rId531"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O251" r:id="rId532"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M252" r:id="rId533"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O252" r:id="rId534"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M253" r:id="rId535"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O253" r:id="rId536"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M254" r:id="rId537"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O254" r:id="rId538"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M255" r:id="rId539"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O255" r:id="rId540"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M256" r:id="rId541"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O256" r:id="rId542"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M257" r:id="rId543"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O257" r:id="rId544"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M258" r:id="rId545"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O258" r:id="rId546"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M259" r:id="rId547"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O259" r:id="rId548"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M260" r:id="rId549"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O260" r:id="rId550"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M261" r:id="rId551"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O261" r:id="rId552"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M262" r:id="rId553"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O262" r:id="rId554"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M263" r:id="rId555"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O263" r:id="rId556"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M264" r:id="rId557"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O264" r:id="rId558"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M265" r:id="rId559"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O265" r:id="rId560"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M266" r:id="rId561"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O266" r:id="rId562"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M267" r:id="rId563"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O267" r:id="rId564"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M268" r:id="rId565"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O268" r:id="rId566"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M269" r:id="rId567"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O269" r:id="rId568"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M270" r:id="rId569"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O270" r:id="rId570"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M271" r:id="rId571"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O271" r:id="rId572"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M272" r:id="rId573"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O272" r:id="rId574"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M273" r:id="rId575"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O273" r:id="rId576"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M274" r:id="rId577"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O274" r:id="rId578"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M275" r:id="rId579"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O275" r:id="rId580"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M276" r:id="rId581"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O276" r:id="rId582"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M277" r:id="rId583"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O277" r:id="rId584"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M278" r:id="rId585"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O278" r:id="rId586"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M279" r:id="rId587"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O279" r:id="rId588"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M280" r:id="rId589"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O280" r:id="rId590"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M281" r:id="rId591"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O281" r:id="rId592"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M282" r:id="rId593"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O282" r:id="rId594"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M283" r:id="rId595"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O283" r:id="rId596"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M284" r:id="rId597"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O284" r:id="rId598"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M285" r:id="rId599"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O285" r:id="rId600"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M286" r:id="rId601"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O286" r:id="rId602"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M287" r:id="rId603"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O287" r:id="rId604"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M288" r:id="rId605"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O288" r:id="rId606"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M289" r:id="rId607"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O289" r:id="rId608"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M290" r:id="rId609"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O290" r:id="rId610"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M291" r:id="rId611"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O291" r:id="rId612"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M292" r:id="rId613"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O292" r:id="rId614"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M293" r:id="rId615"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O293" r:id="rId616"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M294" r:id="rId617"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O294" r:id="rId618"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M295" r:id="rId619"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O295" r:id="rId620"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M296" r:id="rId621"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O296" r:id="rId622"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M297" r:id="rId623"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O297" r:id="rId624"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M298" r:id="rId625"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O298" r:id="rId626"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M299" r:id="rId627"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O299" r:id="rId628"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M300" r:id="rId629"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O300" r:id="rId630"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M301" r:id="rId631"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O301" r:id="rId632"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M302" r:id="rId633"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O302" r:id="rId634"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M303" r:id="rId635"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O303" r:id="rId636"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M304" r:id="rId637"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O304" r:id="rId638"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M305" r:id="rId639"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O305" r:id="rId640"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M306" r:id="rId641"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O306" r:id="rId642"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M307" r:id="rId643"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O307" r:id="rId644"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M308" r:id="rId645"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O308" r:id="rId646"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M309" r:id="rId647"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O309" r:id="rId648"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M310" r:id="rId649"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O310" r:id="rId650"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M311" r:id="rId651"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O311" r:id="rId652"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M312" r:id="rId653"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O312" r:id="rId654"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M313" r:id="rId655"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O313" r:id="rId656"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M314" r:id="rId657"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O314" r:id="rId658"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M315" r:id="rId659"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O315" r:id="rId660"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M316" r:id="rId661"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O316" r:id="rId662"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M317" r:id="rId663"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O317" r:id="rId664"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M318" r:id="rId665"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O318" r:id="rId666"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M319" r:id="rId667"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O319" r:id="rId668"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M320" r:id="rId669"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O320" r:id="rId670"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M321" r:id="rId671"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O321" r:id="rId672"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M322" r:id="rId673"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O322" r:id="rId674"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M323" r:id="rId675"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O323" r:id="rId676"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M324" r:id="rId677"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O324" r:id="rId678"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M325" r:id="rId679"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O325" r:id="rId680"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M326" r:id="rId681"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O326" r:id="rId682"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M327" r:id="rId683"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O327" r:id="rId684"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M328" r:id="rId685"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O328" r:id="rId686"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M329" r:id="rId687"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O329" r:id="rId688"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M330" r:id="rId689"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O330" r:id="rId690"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M331" r:id="rId691"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O331" r:id="rId692"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M332" r:id="rId693"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O332" r:id="rId694"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M333" r:id="rId695"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O333" r:id="rId696"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M334" r:id="rId697"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O334" r:id="rId698"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M335" r:id="rId699"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O335" r:id="rId700"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M336" r:id="rId701"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O336" r:id="rId702"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Ad-hoc: added NVIDIA — 2027 Internships - Software Engineering
</commit_message>
<xml_diff>
--- a/output/tailored_resumes.xlsx
+++ b/output/tailored_resumes.xlsx
@@ -8192,39 +8192,43 @@
         <v>114</v>
       </c>
       <c r="B115" s="5" t="n">
-        <v>38</v>
+        <v>25</v>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>$150k–$210k</t>
+          <t>$250k–$420k</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>NVIDIA</t>
+          <t>TikTok</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>2027 Internships - Software Engineering</t>
-        </is>
-      </c>
-      <c r="F115" t="inlineStr"/>
+          <t>Data Knowledge System Research Scientist Graduate - Data Platform-Global Live</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>San Jose, CA</t>
+        </is>
+      </c>
       <c r="G115" t="inlineStr"/>
       <c r="H115" t="inlineStr"/>
       <c r="I115" t="inlineStr">
         <is>
-          <t>Excellent technical and company-tier alignment (systems, CUDA/GPU, AI infrastructure), but this is a 2027 internship requisition rather than a full-time new-grad role, and a Summer 2027 internship falls after the candidate's May 2027 graduation and target full-time start.</t>
+          <t>Technical content is an excellent match (RAG, agentic systems, vector DBs, knowledge/data platform, distributed systems, Python/Java), but the minimum qualification is a completed or near-complete PhD, which hard-gates a May 2027 bachelor's-level new grad.</t>
         </is>
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>Band reflects NVIDIA full-time new-grad SWE TC (roughly $130-150k base + ~$25-50k/yr RSU + 10-15% bonus), which has run high given stock appreciation; the actual posting is an internship (~$45-60/hr plus housing/relocation, i.e. ~$25-35k for a summer), so the full-time figure is the comparable-role estimate rather than what this req pays. Estimate only.</t>
+          <t>Posting states base $218,400-$480,000 for San Jose, which reflects PhD research-scientist banding rather than a BS/MS new-grad band; adding typical TikTok bonus/RSU on a mid-range base yields roughly $250k-$420k TC. This is an estimate, and it is not the band this candidate would be hired into — TikTok's comparable BS/MS new-grad SWE roles are closer to $145k-$200k TC.</t>
         </is>
       </c>
       <c r="K115" t="inlineStr">
         <is>
-          <t>metadata-only</t>
+          <t>full</t>
         </is>
       </c>
       <c r="L115" t="inlineStr">
@@ -8239,7 +8243,7 @@
       </c>
       <c r="N115" s="3" t="inlineStr">
         <is>
-          <t>NVIDIA_2027_Internships_Software_Engineering_4d8ba5.pdf</t>
+          <t>TikTok_Data_Knowledge_System_Research_Scientist_Gr_e0c0d2.pdf</t>
         </is>
       </c>
       <c r="O115" s="3" t="inlineStr">
@@ -8249,7 +8253,7 @@
       </c>
       <c r="P115" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
@@ -8262,17 +8266,17 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>$250k–$420k</t>
+          <t>$300k–$550k</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>TikTok</t>
+          <t>ByteDance</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>Data Knowledge System Research Scientist Graduate - Data Platform-Global Live</t>
+          <t>Research Scientist Graduate - Seed AI Foundation Model Infrastructure - PhD</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
@@ -8284,12 +8288,12 @@
       <c r="H116" t="inlineStr"/>
       <c r="I116" t="inlineStr">
         <is>
-          <t>Technical content is an excellent match (RAG, agentic systems, vector DBs, knowledge/data platform, distributed systems, Python/Java), but the minimum qualification is a completed or near-complete PhD, which hard-gates a May 2027 bachelor's-level new grad.</t>
+          <t>Domain is an excellent match (distributed training infra, ML systems, C++/Python, large-scale reliability), but the posting hard-requires a completed/near-complete PhD for a Research Scientist track, which disqualifies a May 2027 non-PhD new grad — the parallel ByteDance SWE Graduate (Infrastructure/AML) 2027 req is the correct target.</t>
         </is>
       </c>
       <c r="J116" t="inlineStr">
         <is>
-          <t>Posting states base $218,400-$480,000 for San Jose, which reflects PhD research-scientist banding rather than a BS/MS new-grad band; adding typical TikTok bonus/RSU on a mid-range base yields roughly $250k-$420k TC. This is an estimate, and it is not the band this candidate would be hired into — TikTok's comparable BS/MS new-grad SWE roles are closer to $145k-$200k TC.</t>
+          <t>Posted base range for this PhD Research Scientist role is $254,400-$480,000 plus RSUs and discretionary bonus, implying roughly $300k-$550k TC at that level. This is not the band Nate would see: ByteDance BS/MS new-grad SWE TC is approximately $180k-$240k (base ~$145-175k plus RSUs and sign-on), which still clears the ~$130k anchor.</t>
         </is>
       </c>
       <c r="K116" t="inlineStr">
@@ -8299,7 +8303,7 @@
       </c>
       <c r="L116" t="inlineStr">
         <is>
-          <t>tailored</t>
+          <t>scored</t>
         </is>
       </c>
       <c r="M116" s="3" t="inlineStr">
@@ -8307,11 +8311,7 @@
           <t>Apply ↗</t>
         </is>
       </c>
-      <c r="N116" s="3" t="inlineStr">
-        <is>
-          <t>TikTok_Data_Knowledge_System_Research_Scientist_Gr_e0c0d2.pdf</t>
-        </is>
-      </c>
+      <c r="N116" t="inlineStr"/>
       <c r="O116" s="3" t="inlineStr">
         <is>
           <t>levels.fyi ↗</t>
@@ -8319,7 +8319,7 @@
       </c>
       <c r="P116" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
@@ -8328,38 +8328,38 @@
         <v>116</v>
       </c>
       <c r="B117" s="5" t="n">
-        <v>25</v>
+        <v>42</v>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>$300k–$550k</t>
+          <t>$110k–$170k</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>ByteDance</t>
+          <t>Normal Computing</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Research Scientist Graduate - Seed AI Foundation Model Infrastructure - PhD</t>
+          <t>AI Research Resident</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>San Jose, CA</t>
+          <t>Palo Alto, CA, London, UK, NYC</t>
         </is>
       </c>
       <c r="G117" t="inlineStr"/>
       <c r="H117" t="inlineStr"/>
       <c r="I117" t="inlineStr">
         <is>
-          <t>Domain is an excellent match (distributed training infra, ML systems, C++/Python, large-scale reliability), but the posting hard-requires a completed/near-complete PhD for a Research Scientist track, which disqualifies a May 2027 non-PhD new grad — the parallel ByteDance SWE Graduate (Infrastructure/AML) 2027 req is the correct target.</t>
+          <t>Genuine overlap on agentic LLMs, tool-use, and turning research into working code, but this is a fixed-term research residency aimed at MS/PhD candidates with a research/publication track record and deep PyTorch/RL depth — it neither matches his full-time new-grad backend/distributed-systems target nor leverages his Rust/systems/cloud-infra core.</t>
         </is>
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>Posted base range for this PhD Research Scientist role is $254,400-$480,000 plus RSUs and discretionary bonus, implying roughly $300k-$550k TC at that level. This is not the band Nate would see: ByteDance BS/MS new-grad SWE TC is approximately $180k-$240k (base ~$145-175k plus RSUs and sign-on), which still clears the ~$130k anchor.</t>
+          <t>Normal Computing is a well-funded applied-AI/semiconductor startup with NYC/SF/London/Palo Alto presence, so base pay tracks the frontier-AI-startup band; however, research residencies are typically fixed-term, stipend-style roles paying at or below full-time L3 research comp, with equity that may not meaningfully vest over a short program. No public levels data exists for this specific residency, so the band is deliberately wide and low-confidence: Palo Alto/NYC would sit near the top, London materially lower. Posting does not state residency duration, which adds further uncertainty to annualized TC.</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
@@ -8385,7 +8385,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-19</t>
         </is>
       </c>
     </row>
@@ -8394,38 +8394,38 @@
         <v>117</v>
       </c>
       <c r="B118" s="5" t="n">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>$110k–$170k</t>
+          <t>$88k–$125k</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>Normal Computing</t>
+          <t>Chamberlain Group</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>AI Research Resident</t>
+          <t>Software Engineer 1 - AI</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>Palo Alto, CA, London, UK, NYC</t>
+          <t>California</t>
         </is>
       </c>
       <c r="G118" t="inlineStr"/>
       <c r="H118" t="inlineStr"/>
       <c r="I118" t="inlineStr">
         <is>
-          <t>Genuine overlap on agentic LLMs, tool-use, and turning research into working code, but this is a fixed-term research residency aimed at MS/PhD candidates with a research/publication track record and deep PyTorch/RL depth — it neither matches his full-time new-grad backend/distributed-systems target nor leverages his Rust/systems/cloud-infra core.</t>
+          <t>Genuinely relevant AI/LLM/RAG application work that matches the candidate's agentic-AI strengths, but it's integration/prototyping rather than backend or distributed-systems depth, the posted base range caps at $118.6k (below the ~130k anchor), and it appears to be an immediate-start req rather than a May-2027 new-grad pipeline role.</t>
         </is>
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>Normal Computing is a well-funded applied-AI/semiconductor startup with NYC/SF/London/Palo Alto presence, so base pay tracks the frontier-AI-startup band; however, research residencies are typically fixed-term, stipend-style roles paying at or below full-time L3 research comp, with equity that may not meaningfully vest over a short program. No public levels data exists for this specific residency, so the band is deliberately wide and low-confidence: Palo Alto/NYC would sit near the top, London materially lower. Posting does not state residency duration, which adds further uncertainty to annualized TC.</t>
+          <t>Posting states base pay $69,495-$118,619.50 plus a short-term incentive plan; a strong CS new grad would likely land $85k-$115k base with a ~5-10% STI. Chamberlain Group is a Blackstone-owned IoT/access-hardware company, not a tech-tier compensator, and no equity component is mentioned, so realistic TC lands modestly above base and below the candidate's $130k target.</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
@@ -8451,7 +8451,7 @@
       </c>
       <c r="P118" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
@@ -8459,44 +8459,44 @@
       <c r="A119" t="n">
         <v>118</v>
       </c>
-      <c r="B119" s="5" t="n">
-        <v>48</v>
+      <c r="B119" s="4" t="n">
+        <v>50</v>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>$88k–$125k</t>
+          <t>$85k–$110k</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>Chamberlain Group</t>
+          <t>Motorola</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>Software Engineer 1 - AI</t>
+          <t>Software Engineering</t>
         </is>
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>California</t>
+          <t>Plantation, FL</t>
         </is>
       </c>
       <c r="G119" t="inlineStr"/>
       <c r="H119" t="inlineStr"/>
       <c r="I119" t="inlineStr">
         <is>
-          <t>Genuinely relevant AI/LLM/RAG application work that matches the candidate's agentic-AI strengths, but it's integration/prototyping rather than backend or distributed-systems depth, the posted base range caps at $118.6k (below the ~130k anchor), and it appears to be an immediate-start req rather than a May-2027 new-grad pipeline role.</t>
+          <t>Generic "Software Engineering" posting with no description to match against — Motorola Solutions does real backend/cloud work for public-safety systems so the skills likely transfer, but the Plantation, FL location and a comp tier that sits below the candidate's ~130k anchor pull this to a middling fit.</t>
         </is>
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>Posting states base pay $69,495-$118,619.50 plus a short-term incentive plan; a strong CS new grad would likely land $85k-$115k base with a ~5-10% STI. Chamberlain Group is a Blackstone-owned IoT/access-hardware company, not a tech-tier compensator, and no equity component is mentioned, so realistic TC lands modestly above base and below the candidate's $130k target.</t>
+          <t>Estimate, not fact — and a wide-ish band because the posting has no level, team, or description. Based on general knowledge of Motorola Solutions as a mid-tier non-FAANG hardware/公共-safety company: new-grad base typically ~$78-95k with a small bonus, and South Florida (Plantation) carries no HCOL adjustment. Likely lands below the candidate's ~120k floor.</t>
         </is>
       </c>
       <c r="K119" t="inlineStr">
         <is>
-          <t>full</t>
+          <t>metadata-only</t>
         </is>
       </c>
       <c r="L119" t="inlineStr">
@@ -8517,7 +8517,7 @@
       </c>
       <c r="P119" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -8525,49 +8525,49 @@
       <c r="A120" t="n">
         <v>119</v>
       </c>
-      <c r="B120" s="4" t="n">
-        <v>50</v>
+      <c r="B120" s="5" t="n">
+        <v>32</v>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>$85k–$110k</t>
+          <t>$160k–$230k</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>Motorola</t>
+          <t>Uniswap</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>Software Engineering</t>
+          <t>Software Engineer - Early Career</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>Plantation, FL</t>
+          <t>New York</t>
         </is>
       </c>
       <c r="G120" t="inlineStr"/>
       <c r="H120" t="inlineStr"/>
       <c r="I120" t="inlineStr">
         <is>
-          <t>Generic "Software Engineering" posting with no description to match against — Motorola Solutions does real backend/cloud work for public-safety systems so the skills likely transfer, but the Plantation, FL location and a comp tier that sits below the candidate's ~130k anchor pull this to a middling fit.</t>
+          <t>Comp, tier, and NYC location are excellent fits, but the posting hard-gates on a degree completed between December 2024 and September 2026 while the candidate graduates May 2027, making him ineligible for this cohort; the role is also full-stack/web-leaning rather than backend/distributed-systems focused.</t>
         </is>
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>Estimate, not fact — and a wide-ish band because the posting has no level, team, or description. Based on general knowledge of Motorola Solutions as a mid-tier non-FAANG hardware/公共-safety company: new-grad base typically ~$78-95k with a small bonus, and South Florida (Plantation) carries no HCOL adjustment. Likely lands below the candidate's ~120k floor.</t>
+          <t>Posted NYC base range is $138,400-$198,000; a new grad would land near the low end (~$138-155k base). Uniswap Labs is a well-funded crypto/DeFi employer paying at or above top-tier tech, and the posting explicitly lists token compensation plus benefits on top of base. The band is intentionally wide on the upper end because token grant sizing and valuation are undisclosed and volatile. Estimate, not fact.</t>
         </is>
       </c>
       <c r="K120" t="inlineStr">
         <is>
-          <t>metadata-only</t>
+          <t>full</t>
         </is>
       </c>
       <c r="L120" t="inlineStr">
         <is>
-          <t>scored</t>
+          <t>tailored</t>
         </is>
       </c>
       <c r="M120" s="3" t="inlineStr">
@@ -8575,7 +8575,11 @@
           <t>Apply ↗</t>
         </is>
       </c>
-      <c r="N120" t="inlineStr"/>
+      <c r="N120" s="3" t="inlineStr">
+        <is>
+          <t>Uniswap_Software_Engineer_Early_Career_5a340c.pdf</t>
+        </is>
+      </c>
       <c r="O120" s="3" t="inlineStr">
         <is>
           <t>levels.fyi ↗</t>
@@ -8583,7 +8587,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
@@ -8592,38 +8596,38 @@
         <v>120</v>
       </c>
       <c r="B121" s="5" t="n">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>$160k–$230k</t>
+          <t>$300k–$550k</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>Uniswap</t>
+          <t>ByteDance</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>Software Engineer - Early Career</t>
+          <t>Research Engineer Graduate - Seed Infra</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>Seattle, WA</t>
         </is>
       </c>
       <c r="G121" t="inlineStr"/>
       <c r="H121" t="inlineStr"/>
       <c r="I121" t="inlineStr">
         <is>
-          <t>Comp, tier, and NYC location are excellent fits, but the posting hard-gates on a degree completed between December 2024 and September 2026 while the candidate graduates May 2027, making him ineligible for this cohort; the role is also full-stack/web-leaning rather than backend/distributed-systems focused.</t>
+          <t>The work itself (agent runtimes, sandboxed code execution, K8s/distributed orchestration, LLM infra) maps closely to his strengths, but the role hard-requires a completed PhD and a 2026 onboarding date, both of which he cannot meet as a May 2027 BS/MS grad.</t>
         </is>
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>Posted NYC base range is $138,400-$198,000; a new grad would land near the low end (~$138-155k base). Uniswap Labs is a well-funded crypto/DeFi employer paying at or above top-tier tech, and the posting explicitly lists token compensation plus benefits on top of base. The band is intentionally wide on the upper end because token grant sizing and valuation are undisclosed and volatile. Estimate, not fact.</t>
+          <t>The posting lists base $241,680–$456,000 plus RSUs and bonus, so total package lands roughly $300k–$550k+. Note this is PhD-level research-engineer comp, not a normal new-grad band — ByteDance standard US new-grad SWE TC is more like $180k–$230k, which is the number relevant to this candidate's actual eligibility.</t>
         </is>
       </c>
       <c r="K121" t="inlineStr">
@@ -8633,7 +8637,7 @@
       </c>
       <c r="L121" t="inlineStr">
         <is>
-          <t>tailored</t>
+          <t>scored</t>
         </is>
       </c>
       <c r="M121" s="3" t="inlineStr">
@@ -8641,11 +8645,7 @@
           <t>Apply ↗</t>
         </is>
       </c>
-      <c r="N121" s="3" t="inlineStr">
-        <is>
-          <t>Uniswap_Software_Engineer_Early_Career_5a340c.pdf</t>
-        </is>
-      </c>
+      <c r="N121" t="inlineStr"/>
       <c r="O121" s="3" t="inlineStr">
         <is>
           <t>levels.fyi ↗</t>
@@ -8653,7 +8653,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
@@ -8666,7 +8666,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>$300k–$550k</t>
+          <t>$230k–$340k</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
@@ -8676,7 +8676,7 @@
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>Research Engineer Graduate - Seed Infra</t>
+          <t>Machine Learning Engineer Graduate - E-Commerce Risk Control</t>
         </is>
       </c>
       <c r="F122" t="inlineStr">
@@ -8688,12 +8688,12 @@
       <c r="H122" t="inlineStr"/>
       <c r="I122" t="inlineStr">
         <is>
-          <t>The work itself (agent runtimes, sandboxed code execution, K8s/distributed orchestration, LLM infra) maps closely to his strengths, but the role hard-requires a completed PhD and a 2026 onboarding date, both of which he cannot meet as a May 2027 BS/MS grad.</t>
+          <t>Explicit PhD-only minimum qualification disqualifies a May 2027 BS new grad, and the role's core is research-grade ML (ensemble trees, RL, graph theory, transfer learning, Hive/Hadoop) rather than his backend/distributed-systems/AI-infra strengths — only the multi-agent/ReAct/tool-use architecture overlaps with his agentic-AI experience.</t>
         </is>
       </c>
       <c r="J122" t="inlineStr">
         <is>
-          <t>The posting lists base $241,680–$456,000 plus RSUs and bonus, so total package lands roughly $300k–$550k+. Note this is PhD-level research-engineer comp, not a normal new-grad band — ByteDance standard US new-grad SWE TC is more like $180k–$230k, which is the number relevant to this candidate's actual eligibility.</t>
+          <t>Posting discloses Seattle base of $153,900–$300,960; adding ByteDance's typical RSU grant and discretionary bonus puts PhD-level new-grad ML TC roughly $230k–$340k. Note this is PhD-track compensation, not the BS new-grad band the candidate would actually be hired into (~$150–200k for a comparable non-PhD ByteDance SWE new grad).</t>
         </is>
       </c>
       <c r="K122" t="inlineStr">
@@ -8719,7 +8719,7 @@
       </c>
       <c r="P122" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-19</t>
         </is>
       </c>
     </row>
@@ -8728,38 +8728,42 @@
         <v>122</v>
       </c>
       <c r="B123" s="5" t="n">
-        <v>22</v>
+        <v>38</v>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>$230k–$340k</t>
+          <t>$140k–$180k</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>ByteDance</t>
+          <t>General Motors</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer Graduate - E-Commerce Risk Control</t>
+          <t>Machine Learning Engineer - AI Inference Solutions</t>
         </is>
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>Seattle, WA</t>
+          <t>Sunnyvale, CA</t>
         </is>
       </c>
       <c r="G123" t="inlineStr"/>
-      <c r="H123" t="inlineStr"/>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>spring 2026</t>
+        </is>
+      </c>
       <c r="I123" t="inlineStr">
         <is>
-          <t>Explicit PhD-only minimum qualification disqualifies a May 2027 BS new grad, and the role's core is research-grade ML (ensemble trees, RL, graph theory, transfer learning, Hive/Hadoop) rather than his backend/distributed-systems/AI-infra strengths — only the multi-agent/ReAct/tool-use architecture overlaps with his agentic-AI experience.</t>
+          <t>ML-inference/platform work is adjacent to his AI-infra and systems strengths, but the posting requires a degree completed by Spring/June 2026 (a year before his May 2027 grad) and leans on CUDA/ML-compiler/quantization depth he doesn't have.</t>
         </is>
       </c>
       <c r="J123" t="inlineStr">
         <is>
-          <t>Posting discloses Seattle base of $153,900–$300,960; adding ByteDance's typical RSU grant and discretionary bonus puts PhD-level new-grad ML TC roughly $230k–$340k. Note this is PhD-track compensation, not the BS new-grad band the candidate would actually be hired into (~$150–200k for a comparable non-PhD ByteDance SWE new grad).</t>
+          <t>GM's AV group in Sunnyvale pays Bay Area market (largely ex-Cruise footprint) rather than legacy-automotive rates; new-grad base ~$125-150k plus bonus and RSUs. Estimate, not fact — GM AV new-grad data points are thinner than FAANG.</t>
         </is>
       </c>
       <c r="K123" t="inlineStr">
@@ -8785,7 +8789,7 @@
       </c>
       <c r="P123" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
@@ -8794,42 +8798,34 @@
         <v>123</v>
       </c>
       <c r="B124" s="5" t="n">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>$140k–$180k</t>
+          <t>$170k–$235k</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>General Motors</t>
+          <t>NVIDIA</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer - AI Inference Solutions</t>
-        </is>
-      </c>
-      <c r="F124" t="inlineStr">
-        <is>
-          <t>Sunnyvale, CA</t>
-        </is>
-      </c>
+          <t>2027 Internships - Software Engineering</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr"/>
       <c r="G124" t="inlineStr"/>
-      <c r="H124" t="inlineStr">
-        <is>
-          <t>spring 2026</t>
-        </is>
-      </c>
+      <c r="H124" t="inlineStr"/>
       <c r="I124" t="inlineStr">
         <is>
-          <t>ML-inference/platform work is adjacent to his AI-infra and systems strengths, but the posting requires a degree completed by Spring/June 2026 (a year before his May 2027 grad) and leans on CUDA/ML-compiler/quantization depth he doesn't have.</t>
+          <t>Technical content is an excellent match (cloud storage infra, distributed systems, Kubernetes/microservices, MLOps/GPU infra), but it is a Summer 2027 12-week internship requiring active enrollment for the full duration — incompatible with a May 2027 graduation and a full-time new-grad target start.</t>
         </is>
       </c>
       <c r="J124" t="inlineStr">
         <is>
-          <t>GM's AV group in Sunnyvale pays Bay Area market (largely ex-Cruise footprint) rather than legacy-automotive rates; new-grad base ~$125-150k plus bonus and RSUs. Estimate, not fact — GM AV new-grad data points are thinner than FAANG.</t>
+          <t>Estimate for NVIDIA full-time new-grad SWE (not this internship): base ~$130-155k + RSUs ~$40-80k/yr amortized (elevated by recent stock appreciation) + annual bonus; NVIDIA sits in the top compensation tier for entry-level SWE. The internship itself would pay hourly (~$45-65/hr, ~$25-35k over 12 weeks). Estimate only, not fact.</t>
         </is>
       </c>
       <c r="K124" t="inlineStr">
@@ -8839,7 +8835,7 @@
       </c>
       <c r="L124" t="inlineStr">
         <is>
-          <t>scored</t>
+          <t>tailored</t>
         </is>
       </c>
       <c r="M124" s="3" t="inlineStr">
@@ -8847,7 +8843,11 @@
           <t>Apply ↗</t>
         </is>
       </c>
-      <c r="N124" t="inlineStr"/>
+      <c r="N124" s="3" t="inlineStr">
+        <is>
+          <t>NVIDIA_2027_Internships_Software_Engineering_4d8ba5.pdf</t>
+        </is>
+      </c>
       <c r="O124" s="3" t="inlineStr">
         <is>
           <t>levels.fyi ↗</t>
@@ -8855,7 +8855,7 @@
       </c>
       <c r="P124" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-19</t>
         </is>
       </c>
     </row>
@@ -33790,24 +33790,24 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N115" r:id="rId253"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O115" r:id="rId254"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M116" r:id="rId255"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N116" r:id="rId256"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O116" r:id="rId257"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M117" r:id="rId258"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O117" r:id="rId259"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M118" r:id="rId260"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O118" r:id="rId261"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M119" r:id="rId262"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O119" r:id="rId263"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M120" r:id="rId264"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O116" r:id="rId256"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M117" r:id="rId257"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O117" r:id="rId258"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M118" r:id="rId259"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O118" r:id="rId260"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M119" r:id="rId261"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O119" r:id="rId262"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M120" r:id="rId263"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N120" r:id="rId264"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O120" r:id="rId265"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M121" r:id="rId266"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N121" r:id="rId267"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O121" r:id="rId268"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M122" r:id="rId269"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O122" r:id="rId270"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M123" r:id="rId271"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O123" r:id="rId272"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M124" r:id="rId273"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O121" r:id="rId267"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M122" r:id="rId268"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O122" r:id="rId269"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M123" r:id="rId270"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O123" r:id="rId271"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M124" r:id="rId272"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N124" r:id="rId273"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O124" r:id="rId274"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M125" r:id="rId275"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O125" r:id="rId276"/>

</xml_diff>

<commit_message>
Ad-hoc: tailored 1 job(s) via tailor_selected.py
</commit_message>
<xml_diff>
--- a/output/tailored_resumes.xlsx
+++ b/output/tailored_resumes.xlsx
@@ -797,7 +797,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>scored</t>
+          <t>tailored</t>
         </is>
       </c>
       <c r="M5" s="3" t="inlineStr">
@@ -805,7 +805,11 @@
           <t>Apply ↗</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr"/>
+      <c r="N5" s="3" t="inlineStr">
+        <is>
+          <t>Point72_Software_Developer_Developers_a00cd4.pdf</t>
+        </is>
+      </c>
       <c r="O5" s="3" t="inlineStr">
         <is>
           <t>levels.fyi ↗</t>
@@ -33543,1019 +33547,1020 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M4" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O4" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M5" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O5" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M6" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N6" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O6" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M7" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O7" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M8" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O8" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M9" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O9" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M10" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N10" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M11" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M12" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M13" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M14" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N14" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O14" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M15" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O15" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M16" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O16" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M17" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O17" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M18" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N18" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O18" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M19" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O19" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M20" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N20" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O20" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M21" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O21" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M22" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O22" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M23" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O23" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M24" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N24" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O24" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M25" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O25" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M26" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N26" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O26" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M27" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N27" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O27" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M28" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O28" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M29" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O29" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M30" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O30" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M31" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O31" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M32" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O32" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M33" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O33" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M34" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N34" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O34" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M35" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O35" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M36" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O36" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M37" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N37" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M38" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O38" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M39" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O39" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M40" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O40" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M41" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O41" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M42" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N42" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O42" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M43" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O43" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M44" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O44" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M45" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O45" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M46" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N46" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O46" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M47" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O47" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M48" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N48" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O48" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M49" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O49" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M50" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O50" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M51" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O51" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M52" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O52" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M53" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N53" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O53" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M54" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O54" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M55" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O55" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M56" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O56" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M57" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N57" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O57" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M58" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N58" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O58" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M59" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O59" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M60" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O60" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M61" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O61" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M62" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O62" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M63" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O63" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M64" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O64" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M65" r:id="rId144"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N65" r:id="rId145"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O65" r:id="rId146"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M66" r:id="rId147"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O66" r:id="rId148"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M67" r:id="rId149"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O67" r:id="rId150"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M68" r:id="rId151"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O68" r:id="rId152"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M69" r:id="rId153"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O69" r:id="rId154"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M70" r:id="rId155"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N70" r:id="rId156"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O70" r:id="rId157"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M71" r:id="rId158"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O71" r:id="rId159"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M72" r:id="rId160"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O72" r:id="rId161"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M73" r:id="rId162"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O73" r:id="rId163"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M74" r:id="rId164"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O74" r:id="rId165"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M75" r:id="rId166"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O75" r:id="rId167"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M76" r:id="rId168"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="rId169"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M77" r:id="rId170"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O77" r:id="rId171"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M78" r:id="rId172"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N78" r:id="rId173"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O78" r:id="rId174"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M79" r:id="rId175"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O79" r:id="rId176"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M80" r:id="rId177"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N80" r:id="rId178"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O80" r:id="rId179"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M81" r:id="rId180"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O81" r:id="rId181"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M82" r:id="rId182"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N82" r:id="rId183"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O82" r:id="rId184"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M83" r:id="rId185"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O83" r:id="rId186"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M84" r:id="rId187"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O84" r:id="rId188"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M85" r:id="rId189"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O85" r:id="rId190"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M86" r:id="rId191"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O86" r:id="rId192"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M87" r:id="rId193"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N87" r:id="rId194"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O87" r:id="rId195"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M88" r:id="rId196"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O88" r:id="rId197"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M89" r:id="rId198"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O89" r:id="rId199"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M90" r:id="rId200"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O90" r:id="rId201"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M91" r:id="rId202"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O91" r:id="rId203"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M92" r:id="rId204"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O92" r:id="rId205"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M93" r:id="rId206"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O93" r:id="rId207"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M94" r:id="rId208"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O94" r:id="rId209"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M95" r:id="rId210"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O95" r:id="rId211"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M96" r:id="rId212"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O96" r:id="rId213"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M97" r:id="rId214"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O97" r:id="rId215"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M98" r:id="rId216"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O98" r:id="rId217"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M99" r:id="rId218"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O99" r:id="rId219"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M100" r:id="rId220"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N100" r:id="rId221"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O100" r:id="rId222"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M101" r:id="rId223"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O101" r:id="rId224"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M102" r:id="rId225"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O102" r:id="rId226"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M103" r:id="rId227"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O103" r:id="rId228"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M104" r:id="rId229"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O104" r:id="rId230"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M105" r:id="rId231"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O105" r:id="rId232"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M106" r:id="rId233"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O106" r:id="rId234"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M107" r:id="rId235"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O107" r:id="rId236"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M108" r:id="rId237"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O108" r:id="rId238"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M109" r:id="rId239"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O109" r:id="rId240"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M110" r:id="rId241"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O110" r:id="rId242"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M111" r:id="rId243"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N111" r:id="rId244"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O111" r:id="rId245"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M112" r:id="rId246"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O112" r:id="rId247"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M113" r:id="rId248"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O113" r:id="rId249"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M114" r:id="rId250"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O114" r:id="rId251"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M115" r:id="rId252"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N115" r:id="rId253"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O115" r:id="rId254"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M116" r:id="rId255"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O116" r:id="rId256"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M117" r:id="rId257"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O117" r:id="rId258"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M118" r:id="rId259"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O118" r:id="rId260"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M119" r:id="rId261"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O119" r:id="rId262"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M120" r:id="rId263"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N120" r:id="rId264"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O120" r:id="rId265"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M121" r:id="rId266"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O121" r:id="rId267"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M122" r:id="rId268"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O122" r:id="rId269"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M123" r:id="rId270"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O123" r:id="rId271"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M124" r:id="rId272"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N124" r:id="rId273"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O124" r:id="rId274"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M125" r:id="rId275"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O125" r:id="rId276"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M126" r:id="rId277"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O126" r:id="rId278"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M127" r:id="rId279"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O127" r:id="rId280"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M128" r:id="rId281"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O128" r:id="rId282"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M129" r:id="rId283"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O129" r:id="rId284"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M130" r:id="rId285"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O130" r:id="rId286"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M131" r:id="rId287"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O131" r:id="rId288"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M132" r:id="rId289"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O132" r:id="rId290"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M133" r:id="rId291"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O133" r:id="rId292"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M134" r:id="rId293"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O134" r:id="rId294"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M135" r:id="rId295"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O135" r:id="rId296"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M136" r:id="rId297"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O136" r:id="rId298"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M137" r:id="rId299"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O137" r:id="rId300"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M138" r:id="rId301"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O138" r:id="rId302"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M139" r:id="rId303"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O139" r:id="rId304"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M140" r:id="rId305"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O140" r:id="rId306"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M141" r:id="rId307"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O141" r:id="rId308"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M142" r:id="rId309"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O142" r:id="rId310"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M143" r:id="rId311"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O143" r:id="rId312"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M144" r:id="rId313"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N144" r:id="rId314"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O144" r:id="rId315"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M145" r:id="rId316"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O145" r:id="rId317"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M146" r:id="rId318"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O146" r:id="rId319"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M147" r:id="rId320"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O147" r:id="rId321"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M148" r:id="rId322"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O148" r:id="rId323"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M149" r:id="rId324"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O149" r:id="rId325"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M150" r:id="rId326"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O150" r:id="rId327"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M151" r:id="rId328"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N151" r:id="rId329"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O151" r:id="rId330"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M152" r:id="rId331"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O152" r:id="rId332"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M153" r:id="rId333"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O153" r:id="rId334"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M154" r:id="rId335"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N154" r:id="rId336"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O154" r:id="rId337"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M155" r:id="rId338"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O155" r:id="rId339"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M156" r:id="rId340"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N156" r:id="rId341"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O156" r:id="rId342"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M157" r:id="rId343"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O157" r:id="rId344"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M158" r:id="rId345"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O158" r:id="rId346"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M159" r:id="rId347"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O159" r:id="rId348"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M160" r:id="rId349"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O160" r:id="rId350"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M161" r:id="rId351"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O161" r:id="rId352"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M162" r:id="rId353"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O162" r:id="rId354"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M163" r:id="rId355"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O163" r:id="rId356"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M164" r:id="rId357"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O164" r:id="rId358"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M165" r:id="rId359"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O165" r:id="rId360"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M166" r:id="rId361"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O166" r:id="rId362"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M167" r:id="rId363"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O167" r:id="rId364"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M168" r:id="rId365"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O168" r:id="rId366"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M169" r:id="rId367"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O169" r:id="rId368"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M170" r:id="rId369"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O170" r:id="rId370"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M171" r:id="rId371"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O171" r:id="rId372"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M172" r:id="rId373"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O172" r:id="rId374"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M173" r:id="rId375"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O173" r:id="rId376"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M174" r:id="rId377"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O174" r:id="rId378"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M175" r:id="rId379"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O175" r:id="rId380"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M176" r:id="rId381"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O176" r:id="rId382"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M177" r:id="rId383"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O177" r:id="rId384"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M178" r:id="rId385"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O178" r:id="rId386"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M179" r:id="rId387"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O179" r:id="rId388"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M180" r:id="rId389"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O180" r:id="rId390"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M181" r:id="rId391"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O181" r:id="rId392"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M182" r:id="rId393"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O182" r:id="rId394"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M183" r:id="rId395"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O183" r:id="rId396"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M184" r:id="rId397"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O184" r:id="rId398"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M185" r:id="rId399"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O185" r:id="rId400"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M186" r:id="rId401"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O186" r:id="rId402"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M187" r:id="rId403"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O187" r:id="rId404"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M188" r:id="rId405"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O188" r:id="rId406"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M189" r:id="rId407"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O189" r:id="rId408"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M190" r:id="rId409"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O190" r:id="rId410"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M191" r:id="rId411"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O191" r:id="rId412"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M192" r:id="rId413"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O192" r:id="rId414"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M193" r:id="rId415"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O193" r:id="rId416"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M194" r:id="rId417"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O194" r:id="rId418"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M195" r:id="rId419"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O195" r:id="rId420"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M196" r:id="rId421"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O196" r:id="rId422"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M197" r:id="rId423"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O197" r:id="rId424"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M198" r:id="rId425"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O198" r:id="rId426"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M199" r:id="rId427"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O199" r:id="rId428"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M200" r:id="rId429"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O200" r:id="rId430"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M201" r:id="rId431"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O201" r:id="rId432"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M202" r:id="rId433"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O202" r:id="rId434"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M203" r:id="rId435"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O203" r:id="rId436"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M204" r:id="rId437"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O204" r:id="rId438"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M205" r:id="rId439"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O205" r:id="rId440"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M206" r:id="rId441"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O206" r:id="rId442"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M207" r:id="rId443"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O207" r:id="rId444"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M208" r:id="rId445"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O208" r:id="rId446"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M209" r:id="rId447"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O209" r:id="rId448"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M210" r:id="rId449"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O210" r:id="rId450"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M211" r:id="rId451"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O211" r:id="rId452"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M212" r:id="rId453"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O212" r:id="rId454"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M213" r:id="rId455"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O213" r:id="rId456"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M214" r:id="rId457"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O214" r:id="rId458"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M215" r:id="rId459"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O215" r:id="rId460"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M216" r:id="rId461"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O216" r:id="rId462"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M217" r:id="rId463"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O217" r:id="rId464"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M218" r:id="rId465"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O218" r:id="rId466"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M219" r:id="rId467"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O219" r:id="rId468"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M220" r:id="rId469"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O220" r:id="rId470"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M221" r:id="rId471"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O221" r:id="rId472"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M222" r:id="rId473"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O222" r:id="rId474"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M223" r:id="rId475"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O223" r:id="rId476"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M224" r:id="rId477"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O224" r:id="rId478"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M225" r:id="rId479"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O225" r:id="rId480"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M226" r:id="rId481"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O226" r:id="rId482"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M227" r:id="rId483"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O227" r:id="rId484"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M228" r:id="rId485"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O228" r:id="rId486"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M229" r:id="rId487"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O229" r:id="rId488"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M230" r:id="rId489"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O230" r:id="rId490"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M231" r:id="rId491"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O231" r:id="rId492"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M232" r:id="rId493"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O232" r:id="rId494"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M233" r:id="rId495"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N233" r:id="rId496"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O233" r:id="rId497"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M234" r:id="rId498"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O234" r:id="rId499"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M235" r:id="rId500"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O235" r:id="rId501"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M236" r:id="rId502"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O236" r:id="rId503"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M237" r:id="rId504"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O237" r:id="rId505"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M238" r:id="rId506"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O238" r:id="rId507"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M239" r:id="rId508"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O239" r:id="rId509"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M240" r:id="rId510"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O240" r:id="rId511"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M241" r:id="rId512"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O241" r:id="rId513"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M242" r:id="rId514"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O242" r:id="rId515"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M243" r:id="rId516"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O243" r:id="rId517"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M244" r:id="rId518"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O244" r:id="rId519"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M245" r:id="rId520"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O245" r:id="rId521"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M246" r:id="rId522"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O246" r:id="rId523"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M247" r:id="rId524"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O247" r:id="rId525"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M248" r:id="rId526"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O248" r:id="rId527"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M249" r:id="rId528"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O249" r:id="rId529"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M250" r:id="rId530"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O250" r:id="rId531"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M251" r:id="rId532"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O251" r:id="rId533"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M252" r:id="rId534"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O252" r:id="rId535"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M253" r:id="rId536"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O253" r:id="rId537"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M254" r:id="rId538"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O254" r:id="rId539"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M255" r:id="rId540"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O255" r:id="rId541"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M256" r:id="rId542"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O256" r:id="rId543"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M257" r:id="rId544"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O257" r:id="rId545"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M258" r:id="rId546"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O258" r:id="rId547"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M259" r:id="rId548"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O259" r:id="rId549"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M260" r:id="rId550"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O260" r:id="rId551"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M261" r:id="rId552"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O261" r:id="rId553"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M262" r:id="rId554"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O262" r:id="rId555"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M263" r:id="rId556"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O263" r:id="rId557"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M264" r:id="rId558"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O264" r:id="rId559"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M265" r:id="rId560"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O265" r:id="rId561"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M266" r:id="rId562"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O266" r:id="rId563"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M267" r:id="rId564"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O267" r:id="rId565"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M268" r:id="rId566"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O268" r:id="rId567"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M269" r:id="rId568"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O269" r:id="rId569"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M270" r:id="rId570"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O270" r:id="rId571"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M271" r:id="rId572"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O271" r:id="rId573"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M272" r:id="rId574"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O272" r:id="rId575"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M273" r:id="rId576"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O273" r:id="rId577"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M274" r:id="rId578"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O274" r:id="rId579"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M275" r:id="rId580"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O275" r:id="rId581"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M276" r:id="rId582"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O276" r:id="rId583"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M277" r:id="rId584"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O277" r:id="rId585"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M278" r:id="rId586"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O278" r:id="rId587"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M279" r:id="rId588"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O279" r:id="rId589"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M280" r:id="rId590"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O280" r:id="rId591"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M281" r:id="rId592"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O281" r:id="rId593"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M282" r:id="rId594"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O282" r:id="rId595"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M283" r:id="rId596"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O283" r:id="rId597"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M284" r:id="rId598"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O284" r:id="rId599"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M285" r:id="rId600"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O285" r:id="rId601"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M286" r:id="rId602"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O286" r:id="rId603"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M287" r:id="rId604"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O287" r:id="rId605"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M288" r:id="rId606"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O288" r:id="rId607"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M289" r:id="rId608"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O289" r:id="rId609"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M290" r:id="rId610"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O290" r:id="rId611"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M291" r:id="rId612"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O291" r:id="rId613"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M292" r:id="rId614"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O292" r:id="rId615"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M293" r:id="rId616"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O293" r:id="rId617"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M294" r:id="rId618"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O294" r:id="rId619"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M295" r:id="rId620"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O295" r:id="rId621"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M296" r:id="rId622"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O296" r:id="rId623"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M297" r:id="rId624"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O297" r:id="rId625"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M298" r:id="rId626"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O298" r:id="rId627"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M299" r:id="rId628"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O299" r:id="rId629"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M300" r:id="rId630"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O300" r:id="rId631"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M301" r:id="rId632"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O301" r:id="rId633"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M302" r:id="rId634"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O302" r:id="rId635"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M303" r:id="rId636"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O303" r:id="rId637"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M304" r:id="rId638"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O304" r:id="rId639"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M305" r:id="rId640"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O305" r:id="rId641"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M306" r:id="rId642"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O306" r:id="rId643"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M307" r:id="rId644"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O307" r:id="rId645"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M308" r:id="rId646"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O308" r:id="rId647"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M309" r:id="rId648"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O309" r:id="rId649"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M310" r:id="rId650"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O310" r:id="rId651"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M311" r:id="rId652"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O311" r:id="rId653"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M312" r:id="rId654"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O312" r:id="rId655"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M313" r:id="rId656"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O313" r:id="rId657"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M314" r:id="rId658"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O314" r:id="rId659"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M315" r:id="rId660"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O315" r:id="rId661"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M316" r:id="rId662"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O316" r:id="rId663"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M317" r:id="rId664"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O317" r:id="rId665"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M318" r:id="rId666"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O318" r:id="rId667"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M319" r:id="rId668"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O319" r:id="rId669"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M320" r:id="rId670"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O320" r:id="rId671"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M321" r:id="rId672"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O321" r:id="rId673"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M322" r:id="rId674"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O322" r:id="rId675"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M323" r:id="rId676"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O323" r:id="rId677"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M324" r:id="rId678"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O324" r:id="rId679"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M325" r:id="rId680"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O325" r:id="rId681"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M326" r:id="rId682"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O326" r:id="rId683"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M327" r:id="rId684"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O327" r:id="rId685"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M328" r:id="rId686"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O328" r:id="rId687"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M329" r:id="rId688"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O329" r:id="rId689"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M330" r:id="rId690"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O330" r:id="rId691"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M331" r:id="rId692"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O331" r:id="rId693"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M332" r:id="rId694"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O332" r:id="rId695"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M333" r:id="rId696"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O333" r:id="rId697"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M334" r:id="rId698"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O334" r:id="rId699"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M335" r:id="rId700"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O335" r:id="rId701"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M336" r:id="rId702"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O336" r:id="rId703"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M337" r:id="rId704"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O337" r:id="rId705"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M338" r:id="rId706"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O338" r:id="rId707"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M339" r:id="rId708"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O339" r:id="rId709"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M340" r:id="rId710"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O340" r:id="rId711"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M341" r:id="rId712"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O341" r:id="rId713"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M342" r:id="rId714"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O342" r:id="rId715"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M343" r:id="rId716"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O343" r:id="rId717"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M344" r:id="rId718"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O344" r:id="rId719"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M345" r:id="rId720"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O345" r:id="rId721"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M346" r:id="rId722"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O346" r:id="rId723"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M347" r:id="rId724"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O347" r:id="rId725"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M348" r:id="rId726"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O348" r:id="rId727"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M349" r:id="rId728"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O349" r:id="rId729"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M350" r:id="rId730"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O350" r:id="rId731"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M351" r:id="rId732"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O351" r:id="rId733"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M352" r:id="rId734"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O352" r:id="rId735"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M353" r:id="rId736"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O353" r:id="rId737"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M354" r:id="rId738"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O354" r:id="rId739"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M355" r:id="rId740"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O355" r:id="rId741"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M356" r:id="rId742"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O356" r:id="rId743"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M357" r:id="rId744"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O357" r:id="rId745"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M358" r:id="rId746"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O358" r:id="rId747"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M359" r:id="rId748"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O359" r:id="rId749"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M360" r:id="rId750"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O360" r:id="rId751"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M361" r:id="rId752"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O361" r:id="rId753"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M362" r:id="rId754"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O362" r:id="rId755"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M363" r:id="rId756"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O363" r:id="rId757"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M364" r:id="rId758"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O364" r:id="rId759"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M365" r:id="rId760"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O365" r:id="rId761"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M366" r:id="rId762"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O366" r:id="rId763"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M367" r:id="rId764"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O367" r:id="rId765"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M368" r:id="rId766"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O368" r:id="rId767"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M369" r:id="rId768"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O369" r:id="rId769"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M370" r:id="rId770"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O370" r:id="rId771"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M371" r:id="rId772"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O371" r:id="rId773"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M372" r:id="rId774"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O372" r:id="rId775"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M373" r:id="rId776"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O373" r:id="rId777"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M374" r:id="rId778"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O374" r:id="rId779"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M375" r:id="rId780"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O375" r:id="rId781"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M376" r:id="rId782"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O376" r:id="rId783"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M377" r:id="rId784"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O377" r:id="rId785"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M378" r:id="rId786"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O378" r:id="rId787"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M379" r:id="rId788"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O379" r:id="rId789"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M380" r:id="rId790"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O380" r:id="rId791"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M381" r:id="rId792"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O381" r:id="rId793"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M382" r:id="rId794"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O382" r:id="rId795"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M383" r:id="rId796"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O383" r:id="rId797"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M384" r:id="rId798"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O384" r:id="rId799"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M385" r:id="rId800"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O385" r:id="rId801"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M386" r:id="rId802"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O386" r:id="rId803"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M387" r:id="rId804"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O387" r:id="rId805"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M388" r:id="rId806"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O388" r:id="rId807"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M389" r:id="rId808"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O389" r:id="rId809"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M390" r:id="rId810"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O390" r:id="rId811"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M391" r:id="rId812"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O391" r:id="rId813"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M392" r:id="rId814"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O392" r:id="rId815"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M393" r:id="rId816"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O393" r:id="rId817"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M394" r:id="rId818"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O394" r:id="rId819"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M395" r:id="rId820"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O395" r:id="rId821"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M396" r:id="rId822"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O396" r:id="rId823"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M397" r:id="rId824"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O397" r:id="rId825"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M398" r:id="rId826"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O398" r:id="rId827"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M399" r:id="rId828"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O399" r:id="rId829"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M400" r:id="rId830"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O400" r:id="rId831"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M401" r:id="rId832"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O401" r:id="rId833"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M402" r:id="rId834"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O402" r:id="rId835"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M403" r:id="rId836"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O403" r:id="rId837"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M404" r:id="rId838"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O404" r:id="rId839"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M405" r:id="rId840"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O405" r:id="rId841"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M406" r:id="rId842"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O406" r:id="rId843"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M407" r:id="rId844"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O407" r:id="rId845"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M408" r:id="rId846"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O408" r:id="rId847"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M409" r:id="rId848"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O409" r:id="rId849"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M410" r:id="rId850"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O410" r:id="rId851"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M411" r:id="rId852"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O411" r:id="rId853"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M412" r:id="rId854"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O412" r:id="rId855"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M413" r:id="rId856"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O413" r:id="rId857"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M414" r:id="rId858"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O414" r:id="rId859"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M415" r:id="rId860"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O415" r:id="rId861"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M416" r:id="rId862"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O416" r:id="rId863"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M417" r:id="rId864"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O417" r:id="rId865"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M418" r:id="rId866"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O418" r:id="rId867"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M419" r:id="rId868"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O419" r:id="rId869"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M420" r:id="rId870"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O420" r:id="rId871"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M421" r:id="rId872"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O421" r:id="rId873"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M422" r:id="rId874"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O422" r:id="rId875"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M423" r:id="rId876"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O423" r:id="rId877"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M424" r:id="rId878"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O424" r:id="rId879"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M425" r:id="rId880"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O425" r:id="rId881"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M426" r:id="rId882"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O426" r:id="rId883"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M427" r:id="rId884"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O427" r:id="rId885"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M428" r:id="rId886"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O428" r:id="rId887"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M429" r:id="rId888"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O429" r:id="rId889"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M430" r:id="rId890"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O430" r:id="rId891"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M431" r:id="rId892"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O431" r:id="rId893"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M432" r:id="rId894"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O432" r:id="rId895"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M433" r:id="rId896"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O433" r:id="rId897"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M434" r:id="rId898"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O434" r:id="rId899"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M435" r:id="rId900"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O435" r:id="rId901"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M436" r:id="rId902"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O436" r:id="rId903"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M437" r:id="rId904"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O437" r:id="rId905"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M438" r:id="rId906"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O438" r:id="rId907"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M439" r:id="rId908"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O439" r:id="rId909"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M440" r:id="rId910"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O440" r:id="rId911"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M441" r:id="rId912"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O441" r:id="rId913"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M442" r:id="rId914"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O442" r:id="rId915"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M443" r:id="rId916"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O443" r:id="rId917"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M444" r:id="rId918"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O444" r:id="rId919"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M445" r:id="rId920"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O445" r:id="rId921"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M446" r:id="rId922"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O446" r:id="rId923"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M447" r:id="rId924"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O447" r:id="rId925"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M448" r:id="rId926"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O448" r:id="rId927"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M449" r:id="rId928"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O449" r:id="rId929"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M450" r:id="rId930"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O450" r:id="rId931"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M451" r:id="rId932"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O451" r:id="rId933"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M452" r:id="rId934"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O452" r:id="rId935"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M453" r:id="rId936"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O453" r:id="rId937"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M454" r:id="rId938"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O454" r:id="rId939"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M455" r:id="rId940"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O455" r:id="rId941"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M456" r:id="rId942"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O456" r:id="rId943"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M457" r:id="rId944"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O457" r:id="rId945"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M458" r:id="rId946"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O458" r:id="rId947"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M459" r:id="rId948"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O459" r:id="rId949"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M460" r:id="rId950"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O460" r:id="rId951"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M461" r:id="rId952"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O461" r:id="rId953"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M462" r:id="rId954"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O462" r:id="rId955"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M463" r:id="rId956"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O463" r:id="rId957"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M464" r:id="rId958"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O464" r:id="rId959"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M465" r:id="rId960"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O465" r:id="rId961"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M466" r:id="rId962"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O466" r:id="rId963"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M467" r:id="rId964"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O467" r:id="rId965"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M468" r:id="rId966"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O468" r:id="rId967"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M469" r:id="rId968"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O469" r:id="rId969"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M470" r:id="rId970"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O470" r:id="rId971"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M471" r:id="rId972"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O471" r:id="rId973"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M472" r:id="rId974"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O472" r:id="rId975"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M473" r:id="rId976"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O473" r:id="rId977"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M474" r:id="rId978"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O474" r:id="rId979"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M475" r:id="rId980"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O475" r:id="rId981"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M476" r:id="rId982"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O476" r:id="rId983"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M477" r:id="rId984"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O477" r:id="rId985"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M478" r:id="rId986"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O478" r:id="rId987"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M479" r:id="rId988"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O479" r:id="rId989"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M480" r:id="rId990"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O480" r:id="rId991"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M481" r:id="rId992"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O481" r:id="rId993"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M482" r:id="rId994"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O482" r:id="rId995"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M483" r:id="rId996"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O483" r:id="rId997"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M484" r:id="rId998"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O484" r:id="rId999"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M485" r:id="rId1000"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O485" r:id="rId1001"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M486" r:id="rId1002"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O486" r:id="rId1003"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M487" r:id="rId1004"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O487" r:id="rId1005"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M488" r:id="rId1006"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O488" r:id="rId1007"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M489" r:id="rId1008"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O489" r:id="rId1009"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M490" r:id="rId1010"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O490" r:id="rId1011"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M491" r:id="rId1012"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O491" r:id="rId1013"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M492" r:id="rId1014"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O492" r:id="rId1015"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M493" r:id="rId1016"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O493" r:id="rId1017"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M494" r:id="rId1018"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O494" r:id="rId1019"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M495" r:id="rId1020"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O495" r:id="rId1021"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N5" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O5" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M6" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N6" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O6" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M7" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O7" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M8" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O8" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M9" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O9" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M10" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N10" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M11" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M12" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M13" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M14" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N14" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O14" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M15" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O15" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M16" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O16" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M17" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O17" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M18" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N18" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O18" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M19" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O19" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M20" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N20" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O20" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M21" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O21" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M22" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O22" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M23" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O23" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M24" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N24" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O24" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M25" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O25" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M26" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N26" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O26" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M27" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N27" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O27" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M28" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O28" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M29" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O29" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M30" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O30" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M31" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O31" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M32" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O32" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M33" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O33" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M34" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N34" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O34" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M35" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O35" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M36" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O36" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M37" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N37" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M38" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O38" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M39" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O39" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M40" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O40" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M41" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O41" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M42" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N42" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O42" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M43" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O43" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M44" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O44" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M45" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O45" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M46" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N46" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O46" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M47" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O47" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M48" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N48" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O48" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M49" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O49" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M50" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O50" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M51" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O51" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M52" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O52" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M53" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N53" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O53" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M54" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O54" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M55" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O55" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M56" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O56" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M57" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N57" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O57" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M58" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N58" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O58" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M59" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O59" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M60" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O60" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M61" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O61" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M62" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O62" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M63" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O63" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M64" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O64" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M65" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N65" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O65" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M66" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O66" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M67" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O67" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M68" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O68" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M69" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O69" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M70" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N70" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O70" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M71" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O71" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M72" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O72" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M73" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O73" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M74" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O74" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M75" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O75" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M76" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M77" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O77" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M78" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N78" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O78" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M79" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O79" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M80" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N80" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O80" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M81" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O81" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M82" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N82" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O82" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M83" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O83" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M84" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O84" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M85" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O85" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M86" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O86" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M87" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N87" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O87" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M88" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O88" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M89" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O89" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M90" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O90" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M91" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O91" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M92" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O92" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M93" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O93" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M94" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O94" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M95" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O95" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M96" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O96" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M97" r:id="rId215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O97" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M98" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O98" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M99" r:id="rId219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O99" r:id="rId220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M100" r:id="rId221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N100" r:id="rId222"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O100" r:id="rId223"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M101" r:id="rId224"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O101" r:id="rId225"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M102" r:id="rId226"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O102" r:id="rId227"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M103" r:id="rId228"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O103" r:id="rId229"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M104" r:id="rId230"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O104" r:id="rId231"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M105" r:id="rId232"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O105" r:id="rId233"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M106" r:id="rId234"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O106" r:id="rId235"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M107" r:id="rId236"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O107" r:id="rId237"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M108" r:id="rId238"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O108" r:id="rId239"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M109" r:id="rId240"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O109" r:id="rId241"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M110" r:id="rId242"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O110" r:id="rId243"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M111" r:id="rId244"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N111" r:id="rId245"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O111" r:id="rId246"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M112" r:id="rId247"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O112" r:id="rId248"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M113" r:id="rId249"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O113" r:id="rId250"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M114" r:id="rId251"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O114" r:id="rId252"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M115" r:id="rId253"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N115" r:id="rId254"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O115" r:id="rId255"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M116" r:id="rId256"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O116" r:id="rId257"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M117" r:id="rId258"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O117" r:id="rId259"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M118" r:id="rId260"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O118" r:id="rId261"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M119" r:id="rId262"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O119" r:id="rId263"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M120" r:id="rId264"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N120" r:id="rId265"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O120" r:id="rId266"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M121" r:id="rId267"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O121" r:id="rId268"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M122" r:id="rId269"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O122" r:id="rId270"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M123" r:id="rId271"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O123" r:id="rId272"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M124" r:id="rId273"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N124" r:id="rId274"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O124" r:id="rId275"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M125" r:id="rId276"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O125" r:id="rId277"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M126" r:id="rId278"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O126" r:id="rId279"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M127" r:id="rId280"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O127" r:id="rId281"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M128" r:id="rId282"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O128" r:id="rId283"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M129" r:id="rId284"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O129" r:id="rId285"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M130" r:id="rId286"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O130" r:id="rId287"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M131" r:id="rId288"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O131" r:id="rId289"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M132" r:id="rId290"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O132" r:id="rId291"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M133" r:id="rId292"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O133" r:id="rId293"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M134" r:id="rId294"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O134" r:id="rId295"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M135" r:id="rId296"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O135" r:id="rId297"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M136" r:id="rId298"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O136" r:id="rId299"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M137" r:id="rId300"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O137" r:id="rId301"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M138" r:id="rId302"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O138" r:id="rId303"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M139" r:id="rId304"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O139" r:id="rId305"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M140" r:id="rId306"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O140" r:id="rId307"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M141" r:id="rId308"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O141" r:id="rId309"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M142" r:id="rId310"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O142" r:id="rId311"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M143" r:id="rId312"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O143" r:id="rId313"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M144" r:id="rId314"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N144" r:id="rId315"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O144" r:id="rId316"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M145" r:id="rId317"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O145" r:id="rId318"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M146" r:id="rId319"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O146" r:id="rId320"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M147" r:id="rId321"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O147" r:id="rId322"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M148" r:id="rId323"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O148" r:id="rId324"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M149" r:id="rId325"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O149" r:id="rId326"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M150" r:id="rId327"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O150" r:id="rId328"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M151" r:id="rId329"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N151" r:id="rId330"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O151" r:id="rId331"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M152" r:id="rId332"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O152" r:id="rId333"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M153" r:id="rId334"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O153" r:id="rId335"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M154" r:id="rId336"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N154" r:id="rId337"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O154" r:id="rId338"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M155" r:id="rId339"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O155" r:id="rId340"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M156" r:id="rId341"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N156" r:id="rId342"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O156" r:id="rId343"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M157" r:id="rId344"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O157" r:id="rId345"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M158" r:id="rId346"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O158" r:id="rId347"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M159" r:id="rId348"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O159" r:id="rId349"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M160" r:id="rId350"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O160" r:id="rId351"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M161" r:id="rId352"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O161" r:id="rId353"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M162" r:id="rId354"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O162" r:id="rId355"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M163" r:id="rId356"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O163" r:id="rId357"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M164" r:id="rId358"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O164" r:id="rId359"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M165" r:id="rId360"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O165" r:id="rId361"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M166" r:id="rId362"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O166" r:id="rId363"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M167" r:id="rId364"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O167" r:id="rId365"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M168" r:id="rId366"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O168" r:id="rId367"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M169" r:id="rId368"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O169" r:id="rId369"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M170" r:id="rId370"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O170" r:id="rId371"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M171" r:id="rId372"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O171" r:id="rId373"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M172" r:id="rId374"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O172" r:id="rId375"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M173" r:id="rId376"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O173" r:id="rId377"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M174" r:id="rId378"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O174" r:id="rId379"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M175" r:id="rId380"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O175" r:id="rId381"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M176" r:id="rId382"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O176" r:id="rId383"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M177" r:id="rId384"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O177" r:id="rId385"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M178" r:id="rId386"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O178" r:id="rId387"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M179" r:id="rId388"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O179" r:id="rId389"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M180" r:id="rId390"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O180" r:id="rId391"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M181" r:id="rId392"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O181" r:id="rId393"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M182" r:id="rId394"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O182" r:id="rId395"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M183" r:id="rId396"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O183" r:id="rId397"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M184" r:id="rId398"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O184" r:id="rId399"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M185" r:id="rId400"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O185" r:id="rId401"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M186" r:id="rId402"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O186" r:id="rId403"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M187" r:id="rId404"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O187" r:id="rId405"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M188" r:id="rId406"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O188" r:id="rId407"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M189" r:id="rId408"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O189" r:id="rId409"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M190" r:id="rId410"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O190" r:id="rId411"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M191" r:id="rId412"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O191" r:id="rId413"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M192" r:id="rId414"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O192" r:id="rId415"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M193" r:id="rId416"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O193" r:id="rId417"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M194" r:id="rId418"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O194" r:id="rId419"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M195" r:id="rId420"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O195" r:id="rId421"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M196" r:id="rId422"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O196" r:id="rId423"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M197" r:id="rId424"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O197" r:id="rId425"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M198" r:id="rId426"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O198" r:id="rId427"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M199" r:id="rId428"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O199" r:id="rId429"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M200" r:id="rId430"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O200" r:id="rId431"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M201" r:id="rId432"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O201" r:id="rId433"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M202" r:id="rId434"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O202" r:id="rId435"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M203" r:id="rId436"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O203" r:id="rId437"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M204" r:id="rId438"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O204" r:id="rId439"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M205" r:id="rId440"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O205" r:id="rId441"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M206" r:id="rId442"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O206" r:id="rId443"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M207" r:id="rId444"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O207" r:id="rId445"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M208" r:id="rId446"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O208" r:id="rId447"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M209" r:id="rId448"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O209" r:id="rId449"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M210" r:id="rId450"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O210" r:id="rId451"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M211" r:id="rId452"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O211" r:id="rId453"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M212" r:id="rId454"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O212" r:id="rId455"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M213" r:id="rId456"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O213" r:id="rId457"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M214" r:id="rId458"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O214" r:id="rId459"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M215" r:id="rId460"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O215" r:id="rId461"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M216" r:id="rId462"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O216" r:id="rId463"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M217" r:id="rId464"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O217" r:id="rId465"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M218" r:id="rId466"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O218" r:id="rId467"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M219" r:id="rId468"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O219" r:id="rId469"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M220" r:id="rId470"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O220" r:id="rId471"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M221" r:id="rId472"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O221" r:id="rId473"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M222" r:id="rId474"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O222" r:id="rId475"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M223" r:id="rId476"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O223" r:id="rId477"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M224" r:id="rId478"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O224" r:id="rId479"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M225" r:id="rId480"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O225" r:id="rId481"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M226" r:id="rId482"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O226" r:id="rId483"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M227" r:id="rId484"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O227" r:id="rId485"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M228" r:id="rId486"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O228" r:id="rId487"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M229" r:id="rId488"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O229" r:id="rId489"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M230" r:id="rId490"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O230" r:id="rId491"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M231" r:id="rId492"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O231" r:id="rId493"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M232" r:id="rId494"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O232" r:id="rId495"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M233" r:id="rId496"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N233" r:id="rId497"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O233" r:id="rId498"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M234" r:id="rId499"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O234" r:id="rId500"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M235" r:id="rId501"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O235" r:id="rId502"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M236" r:id="rId503"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O236" r:id="rId504"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M237" r:id="rId505"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O237" r:id="rId506"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M238" r:id="rId507"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O238" r:id="rId508"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M239" r:id="rId509"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O239" r:id="rId510"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M240" r:id="rId511"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O240" r:id="rId512"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M241" r:id="rId513"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O241" r:id="rId514"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M242" r:id="rId515"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O242" r:id="rId516"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M243" r:id="rId517"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O243" r:id="rId518"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M244" r:id="rId519"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O244" r:id="rId520"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M245" r:id="rId521"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O245" r:id="rId522"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M246" r:id="rId523"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O246" r:id="rId524"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M247" r:id="rId525"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O247" r:id="rId526"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M248" r:id="rId527"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O248" r:id="rId528"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M249" r:id="rId529"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O249" r:id="rId530"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M250" r:id="rId531"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O250" r:id="rId532"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M251" r:id="rId533"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O251" r:id="rId534"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M252" r:id="rId535"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O252" r:id="rId536"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M253" r:id="rId537"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O253" r:id="rId538"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M254" r:id="rId539"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O254" r:id="rId540"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M255" r:id="rId541"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O255" r:id="rId542"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M256" r:id="rId543"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O256" r:id="rId544"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M257" r:id="rId545"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O257" r:id="rId546"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M258" r:id="rId547"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O258" r:id="rId548"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M259" r:id="rId549"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O259" r:id="rId550"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M260" r:id="rId551"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O260" r:id="rId552"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M261" r:id="rId553"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O261" r:id="rId554"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M262" r:id="rId555"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O262" r:id="rId556"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M263" r:id="rId557"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O263" r:id="rId558"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M264" r:id="rId559"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O264" r:id="rId560"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M265" r:id="rId561"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O265" r:id="rId562"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M266" r:id="rId563"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O266" r:id="rId564"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M267" r:id="rId565"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O267" r:id="rId566"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M268" r:id="rId567"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O268" r:id="rId568"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M269" r:id="rId569"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O269" r:id="rId570"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M270" r:id="rId571"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O270" r:id="rId572"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M271" r:id="rId573"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O271" r:id="rId574"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M272" r:id="rId575"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O272" r:id="rId576"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M273" r:id="rId577"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O273" r:id="rId578"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M274" r:id="rId579"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O274" r:id="rId580"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M275" r:id="rId581"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O275" r:id="rId582"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M276" r:id="rId583"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O276" r:id="rId584"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M277" r:id="rId585"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O277" r:id="rId586"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M278" r:id="rId587"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O278" r:id="rId588"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M279" r:id="rId589"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O279" r:id="rId590"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M280" r:id="rId591"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O280" r:id="rId592"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M281" r:id="rId593"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O281" r:id="rId594"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M282" r:id="rId595"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O282" r:id="rId596"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M283" r:id="rId597"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O283" r:id="rId598"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M284" r:id="rId599"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O284" r:id="rId600"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M285" r:id="rId601"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O285" r:id="rId602"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M286" r:id="rId603"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O286" r:id="rId604"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M287" r:id="rId605"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O287" r:id="rId606"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M288" r:id="rId607"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O288" r:id="rId608"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M289" r:id="rId609"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O289" r:id="rId610"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M290" r:id="rId611"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O290" r:id="rId612"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M291" r:id="rId613"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O291" r:id="rId614"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M292" r:id="rId615"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O292" r:id="rId616"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M293" r:id="rId617"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O293" r:id="rId618"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M294" r:id="rId619"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O294" r:id="rId620"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M295" r:id="rId621"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O295" r:id="rId622"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M296" r:id="rId623"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O296" r:id="rId624"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M297" r:id="rId625"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O297" r:id="rId626"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M298" r:id="rId627"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O298" r:id="rId628"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M299" r:id="rId629"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O299" r:id="rId630"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M300" r:id="rId631"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O300" r:id="rId632"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M301" r:id="rId633"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O301" r:id="rId634"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M302" r:id="rId635"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O302" r:id="rId636"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M303" r:id="rId637"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O303" r:id="rId638"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M304" r:id="rId639"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O304" r:id="rId640"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M305" r:id="rId641"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O305" r:id="rId642"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M306" r:id="rId643"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O306" r:id="rId644"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M307" r:id="rId645"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O307" r:id="rId646"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M308" r:id="rId647"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O308" r:id="rId648"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M309" r:id="rId649"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O309" r:id="rId650"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M310" r:id="rId651"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O310" r:id="rId652"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M311" r:id="rId653"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O311" r:id="rId654"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M312" r:id="rId655"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O312" r:id="rId656"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M313" r:id="rId657"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O313" r:id="rId658"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M314" r:id="rId659"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O314" r:id="rId660"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M315" r:id="rId661"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O315" r:id="rId662"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M316" r:id="rId663"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O316" r:id="rId664"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M317" r:id="rId665"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O317" r:id="rId666"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M318" r:id="rId667"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O318" r:id="rId668"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M319" r:id="rId669"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O319" r:id="rId670"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M320" r:id="rId671"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O320" r:id="rId672"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M321" r:id="rId673"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O321" r:id="rId674"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M322" r:id="rId675"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O322" r:id="rId676"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M323" r:id="rId677"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O323" r:id="rId678"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M324" r:id="rId679"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O324" r:id="rId680"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M325" r:id="rId681"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O325" r:id="rId682"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M326" r:id="rId683"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O326" r:id="rId684"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M327" r:id="rId685"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O327" r:id="rId686"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M328" r:id="rId687"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O328" r:id="rId688"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M329" r:id="rId689"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O329" r:id="rId690"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M330" r:id="rId691"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O330" r:id="rId692"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M331" r:id="rId693"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O331" r:id="rId694"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M332" r:id="rId695"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O332" r:id="rId696"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M333" r:id="rId697"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O333" r:id="rId698"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M334" r:id="rId699"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O334" r:id="rId700"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M335" r:id="rId701"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O335" r:id="rId702"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M336" r:id="rId703"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O336" r:id="rId704"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M337" r:id="rId705"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O337" r:id="rId706"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M338" r:id="rId707"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O338" r:id="rId708"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M339" r:id="rId709"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O339" r:id="rId710"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M340" r:id="rId711"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O340" r:id="rId712"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M341" r:id="rId713"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O341" r:id="rId714"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M342" r:id="rId715"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O342" r:id="rId716"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M343" r:id="rId717"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O343" r:id="rId718"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M344" r:id="rId719"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O344" r:id="rId720"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M345" r:id="rId721"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O345" r:id="rId722"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M346" r:id="rId723"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O346" r:id="rId724"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M347" r:id="rId725"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O347" r:id="rId726"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M348" r:id="rId727"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O348" r:id="rId728"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M349" r:id="rId729"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O349" r:id="rId730"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M350" r:id="rId731"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O350" r:id="rId732"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M351" r:id="rId733"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O351" r:id="rId734"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M352" r:id="rId735"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O352" r:id="rId736"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M353" r:id="rId737"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O353" r:id="rId738"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M354" r:id="rId739"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O354" r:id="rId740"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M355" r:id="rId741"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O355" r:id="rId742"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M356" r:id="rId743"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O356" r:id="rId744"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M357" r:id="rId745"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O357" r:id="rId746"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M358" r:id="rId747"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O358" r:id="rId748"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M359" r:id="rId749"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O359" r:id="rId750"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M360" r:id="rId751"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O360" r:id="rId752"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M361" r:id="rId753"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O361" r:id="rId754"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M362" r:id="rId755"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O362" r:id="rId756"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M363" r:id="rId757"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O363" r:id="rId758"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M364" r:id="rId759"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O364" r:id="rId760"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M365" r:id="rId761"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O365" r:id="rId762"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M366" r:id="rId763"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O366" r:id="rId764"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M367" r:id="rId765"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O367" r:id="rId766"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M368" r:id="rId767"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O368" r:id="rId768"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M369" r:id="rId769"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O369" r:id="rId770"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M370" r:id="rId771"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O370" r:id="rId772"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M371" r:id="rId773"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O371" r:id="rId774"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M372" r:id="rId775"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O372" r:id="rId776"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M373" r:id="rId777"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O373" r:id="rId778"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M374" r:id="rId779"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O374" r:id="rId780"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M375" r:id="rId781"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O375" r:id="rId782"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M376" r:id="rId783"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O376" r:id="rId784"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M377" r:id="rId785"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O377" r:id="rId786"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M378" r:id="rId787"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O378" r:id="rId788"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M379" r:id="rId789"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O379" r:id="rId790"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M380" r:id="rId791"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O380" r:id="rId792"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M381" r:id="rId793"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O381" r:id="rId794"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M382" r:id="rId795"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O382" r:id="rId796"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M383" r:id="rId797"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O383" r:id="rId798"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M384" r:id="rId799"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O384" r:id="rId800"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M385" r:id="rId801"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O385" r:id="rId802"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M386" r:id="rId803"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O386" r:id="rId804"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M387" r:id="rId805"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O387" r:id="rId806"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M388" r:id="rId807"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O388" r:id="rId808"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M389" r:id="rId809"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O389" r:id="rId810"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M390" r:id="rId811"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O390" r:id="rId812"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M391" r:id="rId813"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O391" r:id="rId814"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M392" r:id="rId815"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O392" r:id="rId816"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M393" r:id="rId817"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O393" r:id="rId818"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M394" r:id="rId819"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O394" r:id="rId820"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M395" r:id="rId821"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O395" r:id="rId822"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M396" r:id="rId823"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O396" r:id="rId824"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M397" r:id="rId825"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O397" r:id="rId826"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M398" r:id="rId827"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O398" r:id="rId828"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M399" r:id="rId829"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O399" r:id="rId830"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M400" r:id="rId831"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O400" r:id="rId832"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M401" r:id="rId833"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O401" r:id="rId834"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M402" r:id="rId835"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O402" r:id="rId836"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M403" r:id="rId837"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O403" r:id="rId838"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M404" r:id="rId839"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O404" r:id="rId840"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M405" r:id="rId841"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O405" r:id="rId842"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M406" r:id="rId843"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O406" r:id="rId844"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M407" r:id="rId845"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O407" r:id="rId846"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M408" r:id="rId847"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O408" r:id="rId848"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M409" r:id="rId849"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O409" r:id="rId850"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M410" r:id="rId851"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O410" r:id="rId852"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M411" r:id="rId853"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O411" r:id="rId854"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M412" r:id="rId855"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O412" r:id="rId856"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M413" r:id="rId857"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O413" r:id="rId858"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M414" r:id="rId859"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O414" r:id="rId860"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M415" r:id="rId861"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O415" r:id="rId862"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M416" r:id="rId863"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O416" r:id="rId864"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M417" r:id="rId865"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O417" r:id="rId866"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M418" r:id="rId867"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O418" r:id="rId868"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M419" r:id="rId869"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O419" r:id="rId870"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M420" r:id="rId871"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O420" r:id="rId872"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M421" r:id="rId873"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O421" r:id="rId874"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M422" r:id="rId875"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O422" r:id="rId876"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M423" r:id="rId877"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O423" r:id="rId878"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M424" r:id="rId879"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O424" r:id="rId880"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M425" r:id="rId881"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O425" r:id="rId882"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M426" r:id="rId883"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O426" r:id="rId884"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M427" r:id="rId885"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O427" r:id="rId886"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M428" r:id="rId887"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O428" r:id="rId888"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M429" r:id="rId889"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O429" r:id="rId890"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M430" r:id="rId891"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O430" r:id="rId892"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M431" r:id="rId893"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O431" r:id="rId894"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M432" r:id="rId895"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O432" r:id="rId896"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M433" r:id="rId897"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O433" r:id="rId898"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M434" r:id="rId899"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O434" r:id="rId900"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M435" r:id="rId901"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O435" r:id="rId902"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M436" r:id="rId903"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O436" r:id="rId904"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M437" r:id="rId905"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O437" r:id="rId906"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M438" r:id="rId907"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O438" r:id="rId908"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M439" r:id="rId909"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O439" r:id="rId910"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M440" r:id="rId911"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O440" r:id="rId912"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M441" r:id="rId913"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O441" r:id="rId914"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M442" r:id="rId915"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O442" r:id="rId916"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M443" r:id="rId917"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O443" r:id="rId918"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M444" r:id="rId919"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O444" r:id="rId920"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M445" r:id="rId921"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O445" r:id="rId922"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M446" r:id="rId923"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O446" r:id="rId924"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M447" r:id="rId925"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O447" r:id="rId926"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M448" r:id="rId927"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O448" r:id="rId928"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M449" r:id="rId929"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O449" r:id="rId930"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M450" r:id="rId931"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O450" r:id="rId932"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M451" r:id="rId933"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O451" r:id="rId934"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M452" r:id="rId935"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O452" r:id="rId936"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M453" r:id="rId937"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O453" r:id="rId938"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M454" r:id="rId939"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O454" r:id="rId940"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M455" r:id="rId941"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O455" r:id="rId942"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M456" r:id="rId943"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O456" r:id="rId944"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M457" r:id="rId945"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O457" r:id="rId946"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M458" r:id="rId947"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O458" r:id="rId948"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M459" r:id="rId949"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O459" r:id="rId950"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M460" r:id="rId951"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O460" r:id="rId952"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M461" r:id="rId953"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O461" r:id="rId954"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M462" r:id="rId955"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O462" r:id="rId956"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M463" r:id="rId957"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O463" r:id="rId958"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M464" r:id="rId959"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O464" r:id="rId960"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M465" r:id="rId961"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O465" r:id="rId962"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M466" r:id="rId963"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O466" r:id="rId964"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M467" r:id="rId965"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O467" r:id="rId966"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M468" r:id="rId967"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O468" r:id="rId968"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M469" r:id="rId969"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O469" r:id="rId970"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M470" r:id="rId971"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O470" r:id="rId972"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M471" r:id="rId973"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O471" r:id="rId974"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M472" r:id="rId975"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O472" r:id="rId976"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M473" r:id="rId977"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O473" r:id="rId978"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M474" r:id="rId979"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O474" r:id="rId980"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M475" r:id="rId981"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O475" r:id="rId982"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M476" r:id="rId983"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O476" r:id="rId984"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M477" r:id="rId985"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O477" r:id="rId986"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M478" r:id="rId987"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O478" r:id="rId988"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M479" r:id="rId989"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O479" r:id="rId990"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M480" r:id="rId991"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O480" r:id="rId992"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M481" r:id="rId993"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O481" r:id="rId994"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M482" r:id="rId995"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O482" r:id="rId996"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M483" r:id="rId997"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O483" r:id="rId998"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M484" r:id="rId999"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O484" r:id="rId1000"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M485" r:id="rId1001"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O485" r:id="rId1002"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M486" r:id="rId1003"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O486" r:id="rId1004"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M487" r:id="rId1005"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O487" r:id="rId1006"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M488" r:id="rId1007"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O488" r:id="rId1008"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M489" r:id="rId1009"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O489" r:id="rId1010"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M490" r:id="rId1011"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O490" r:id="rId1012"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M491" r:id="rId1013"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O491" r:id="rId1014"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M492" r:id="rId1015"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O492" r:id="rId1016"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M493" r:id="rId1017"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O493" r:id="rId1018"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M494" r:id="rId1019"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O494" r:id="rId1020"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M495" r:id="rId1021"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O495" r:id="rId1022"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add an applied=True escape hatch so untailored applications get tracked too
scan_email_status.py only matched companies from status=="tailored" jobs,
so a real posting applied to without running tailor_selected.py first
(e.g. Truveta today) never entered the matching pool even with a genuine
confirmation email sitting in the inbox. scripts/mark_applied.py flags a
job_store entry by company (+ optional --title to disambiguate) so the
next scan picks it up.
</commit_message>
<xml_diff>
--- a/output/tailored_resumes.xlsx
+++ b/output/tailored_resumes.xlsx
@@ -4144,7 +4144,11 @@
           <t>scored</t>
         </is>
       </c>
-      <c r="M52" t="inlineStr"/>
+      <c r="M52" s="5" t="inlineStr">
+        <is>
+          <t>applied</t>
+        </is>
+      </c>
       <c r="N52" s="3" t="inlineStr">
         <is>
           <t>Apply ↗</t>

</xml_diff>

<commit_message>
Recognize OA-completion wording; mark_applied.py stacks all matches by default
classify() had no signal for "assessment completed"/"is being reviewed"/
"assessment submitted" phrasing (Netic AI, Wolverine used these instead of
invite-style wording), so completing an OA wasn't recognized at all --
added as a new oa_done status, wired into the tracker dropdown's existing
color and job_store's APP_STATUS_COLORS. Added a subject pattern for
"being reviewed by X" / "assessment submitted for X" to extract the
company from that phrasing too.

mark_applied.py now marks every matching posting instead of erroring out
asking which one to disambiguate -- matches the "stacking by company" model
the rest of this pipeline already uses (Veeva Systems had 4 near-duplicate
postings in job_store; no reason to force picking one).
</commit_message>
<xml_diff>
--- a/output/tailored_resumes.xlsx
+++ b/output/tailored_resumes.xlsx
@@ -34,7 +34,7 @@
       <u val="single"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -66,6 +66,11 @@
         <fgColor rgb="00FFEB9C"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFD966"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -79,7 +84,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -87,6 +92,7 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -6624,7 +6630,11 @@
           <t>scored</t>
         </is>
       </c>
-      <c r="M88" t="inlineStr"/>
+      <c r="M88" s="7" t="inlineStr">
+        <is>
+          <t>oa_done</t>
+        </is>
+      </c>
       <c r="N88" s="3" t="inlineStr">
         <is>
           <t>Apply ↗</t>
@@ -8055,7 +8065,11 @@
           <t>scored</t>
         </is>
       </c>
-      <c r="M109" t="inlineStr"/>
+      <c r="M109" s="7" t="inlineStr">
+        <is>
+          <t>oa_done</t>
+        </is>
+      </c>
       <c r="N109" s="3" t="inlineStr">
         <is>
           <t>Apply ↗</t>
@@ -9021,7 +9035,11 @@
           <t>scored</t>
         </is>
       </c>
-      <c r="M123" t="inlineStr"/>
+      <c r="M123" s="7" t="inlineStr">
+        <is>
+          <t>oa_done</t>
+        </is>
+      </c>
       <c r="N123" s="3" t="inlineStr">
         <is>
           <t>Apply ↗</t>
@@ -16325,7 +16343,11 @@
           <t>scored</t>
         </is>
       </c>
-      <c r="M231" t="inlineStr"/>
+      <c r="M231" s="7" t="inlineStr">
+        <is>
+          <t>oa_done</t>
+        </is>
+      </c>
       <c r="N231" s="3" t="inlineStr">
         <is>
           <t>Apply ↗</t>

</xml_diff>

<commit_message>
Cap tracking to one entry per company; add Veeva vendor mapping
Both scan_email_status.py's Pass 1 and mark_applied.py were marking every
job_store posting at a matched company (feed duplicates or genuinely
different roles alike) -- Nate wants exactly one tracked entry per
company regardless of how many postings exist. Consolidated SpaceX (3
duplicates from before this fix) and Veeva (4) down to one each.

Also adds KNOWN_VENDOR_DOMAINS: RembrandtAdvantage's assessment emails
never mention the employer by name in subject or body (confirmed by
hand -- it's Veeva), so generic extraction could never recover this on
its own. Checked before the sender-name fallback, which would otherwise
extract the vendor's own name instead of the real employer.
</commit_message>
<xml_diff>
--- a/output/tailored_resumes.xlsx
+++ b/output/tailored_resumes.xlsx
@@ -3310,11 +3310,7 @@
           <t>tailored</t>
         </is>
       </c>
-      <c r="M40" s="5" t="inlineStr">
-        <is>
-          <t>applied</t>
-        </is>
-      </c>
+      <c r="M40" t="inlineStr"/>
       <c r="N40" s="3" t="inlineStr">
         <is>
           <t>Apply ↗</t>
@@ -6279,11 +6275,7 @@
           <t>tailored</t>
         </is>
       </c>
-      <c r="M83" s="5" t="inlineStr">
-        <is>
-          <t>applied</t>
-        </is>
-      </c>
+      <c r="M83" t="inlineStr"/>
       <c r="N83" s="3" t="inlineStr">
         <is>
           <t>Apply ↗</t>
@@ -6630,11 +6622,7 @@
           <t>scored</t>
         </is>
       </c>
-      <c r="M88" s="7" t="inlineStr">
-        <is>
-          <t>oa_done</t>
-        </is>
-      </c>
+      <c r="M88" t="inlineStr"/>
       <c r="N88" s="3" t="inlineStr">
         <is>
           <t>Apply ↗</t>
@@ -8065,11 +8053,7 @@
           <t>scored</t>
         </is>
       </c>
-      <c r="M109" s="7" t="inlineStr">
-        <is>
-          <t>oa_done</t>
-        </is>
-      </c>
+      <c r="M109" t="inlineStr"/>
       <c r="N109" s="3" t="inlineStr">
         <is>
           <t>Apply ↗</t>
@@ -16343,11 +16327,7 @@
           <t>scored</t>
         </is>
       </c>
-      <c r="M231" s="7" t="inlineStr">
-        <is>
-          <t>oa_done</t>
-        </is>
-      </c>
+      <c r="M231" t="inlineStr"/>
       <c r="N231" s="3" t="inlineStr">
         <is>
           <t>Apply ↗</t>

</xml_diff>

<commit_message>
Commit pending app_status updates from manual scan runs
Left the tree dirty after testing earlier, which blocked run_pipeline.ps1's
git pull --rebase on today's scheduled run (2026-08-25 08:09).
</commit_message>
<xml_diff>
--- a/output/tailored_resumes.xlsx
+++ b/output/tailored_resumes.xlsx
@@ -4016,9 +4016,9 @@
           <t>tailored</t>
         </is>
       </c>
-      <c r="M50" s="5" t="inlineStr">
-        <is>
-          <t>applied</t>
+      <c r="M50" s="2" t="inlineStr">
+        <is>
+          <t>rejected</t>
         </is>
       </c>
       <c r="N50" s="3" t="inlineStr">

</xml_diff>